<commit_message>
Cập nhật Báo Cáo Đối Soát Đông Mát - 2026-09-25 09:32:38
</commit_message>
<xml_diff>
--- a/SPAM_PHIEU_CHUYEN/CHI TIẾT MÁT/Danh sách Siêu thị.xlsx
+++ b/SPAM_PHIEU_CHUYEN/CHI TIẾT MÁT/Danh sách Siêu thị.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="687">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="694">
   <si>
     <t>Tên Siêu thị</t>
   </si>
@@ -205,7 +205,7 @@
     <t>KFM_BDU_DAN - B2.01.05 Tháp B Opal Boulevard</t>
   </si>
   <si>
-    <t>KFM_HCM_Q07 - B1.01 Chung cư Golden Star</t>
+    <t>KFM_HCM_Q7 - A165 (Golden Star)</t>
   </si>
   <si>
     <t>KFM_HCM_Q07 - Block K Happy Valley</t>
@@ -703,10 +703,19 @@
     <t>KFM_HCM_BCH - D-2.01A Westgate An Gia</t>
   </si>
   <si>
-    <t>KFM_HCM_Q7 - A248 (Garden Plaza)</t>
-  </si>
-  <si>
-    <t>KFM_HCM_Q7 - A255 (Green View)</t>
+    <t>KFM_HCM_Q7 - DC - A248 (Garden Plaza)</t>
+  </si>
+  <si>
+    <t>KFM_HCM_Q7 - DC - A255 (Green View)</t>
+  </si>
+  <si>
+    <t>KFM_HCM_Q12 - DC - A215 (Thạnh Xuân 14)</t>
+  </si>
+  <si>
+    <t>KFM_HCM_TDU - DC - A252 (DS9 An Khánh)</t>
+  </si>
+  <si>
+    <t>KFM_HCM_BTA - DC - A247 (Lê Cơ)</t>
   </si>
   <si>
     <t>A101</t>
@@ -1390,6 +1399,15 @@
     <t>A255</t>
   </si>
   <si>
+    <t>A215</t>
+  </si>
+  <si>
+    <t>A252</t>
+  </si>
+  <si>
+    <t>A247</t>
+  </si>
+  <si>
     <t>-4970846623</t>
   </si>
   <si>
@@ -1411,9 +1429,6 @@
     <t>-1003525071105</t>
   </si>
   <si>
-    <t>-4978161635</t>
-  </si>
-  <si>
     <t>-4813095752</t>
   </si>
   <si>
@@ -1441,9 +1456,6 @@
     <t>-5065492668</t>
   </si>
   <si>
-    <t>-4938449227</t>
-  </si>
-  <si>
     <t>-1003595238765</t>
   </si>
   <si>
@@ -1573,7 +1585,7 @@
     <t>-5223853892</t>
   </si>
   <si>
-    <t>-4906644767</t>
+    <t>-1004427935189</t>
   </si>
   <si>
     <t>-5135406910</t>
@@ -2075,6 +2087,15 @@
   </si>
   <si>
     <t>-1003991560755</t>
+  </si>
+  <si>
+    <t>-1004387715043</t>
+  </si>
+  <si>
+    <t>-1004488038357</t>
+  </si>
+  <si>
+    <t>-1004367466882</t>
   </si>
 </sst>
 </file>
@@ -2406,7 +2427,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D230"/>
+  <dimension ref="A1:D231"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -2428,13 +2449,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="C2" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="D2" t="s">
-        <v>458</v>
+        <v>464</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2442,13 +2463,13 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="C3" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="D3" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2456,13 +2477,13 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C4" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="D4" t="s">
-        <v>460</v>
+        <v>466</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2470,13 +2491,13 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="C5" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D5" t="s">
-        <v>461</v>
+        <v>467</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2484,13 +2505,13 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="C6" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="D6" t="s">
-        <v>462</v>
+        <v>468</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2498,13 +2519,13 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C7" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="D7" t="s">
-        <v>463</v>
+        <v>469</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2512,13 +2533,13 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C8" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="D8" t="s">
-        <v>464</v>
+        <v>470</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2526,3107 +2547,3121 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C9" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="D9" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C10" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="D10" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="C11" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="D11" t="s">
-        <v>467</v>
+        <v>473</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="C12" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="D12" t="s">
-        <v>468</v>
+        <v>474</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C13" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="D13" t="s">
-        <v>469</v>
+        <v>475</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="C14" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="D14" t="s">
-        <v>470</v>
+        <v>476</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="C15" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="D15" t="s">
-        <v>471</v>
+        <v>477</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="C16" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="D16" t="s">
-        <v>472</v>
+        <v>478</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="C17" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="D17" t="s">
-        <v>473</v>
+        <v>479</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="C18" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="D18" t="s">
-        <v>474</v>
+        <v>480</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="C19" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="D19" t="s">
-        <v>475</v>
+        <v>481</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B20" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="C20" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="D20" t="s">
-        <v>476</v>
+        <v>482</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B21" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="C21" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="D21" t="s">
-        <v>477</v>
+        <v>483</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B22" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="C22" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="D22" t="s">
-        <v>478</v>
+        <v>484</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="C23" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="D23" t="s">
-        <v>479</v>
+        <v>485</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B24" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="C24" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D24" t="s">
-        <v>480</v>
+        <v>486</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="C25" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="D25" t="s">
-        <v>481</v>
+        <v>487</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B26" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="C26" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="D26" t="s">
-        <v>482</v>
+        <v>488</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B27" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="C27" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="D27" t="s">
-        <v>483</v>
+        <v>489</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B28" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="C28" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="D28" t="s">
-        <v>484</v>
+        <v>490</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B29" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="C29" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="D29" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B30" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="C30" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="D30" t="s">
-        <v>486</v>
+        <v>492</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B31" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="C31" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="D31" t="s">
-        <v>487</v>
+        <v>493</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B32" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="C32" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D32" t="s">
-        <v>488</v>
+        <v>494</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B33" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="C33" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="D33" t="s">
-        <v>489</v>
+        <v>495</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B34" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="C34" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="D34" t="s">
-        <v>490</v>
+        <v>496</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B35" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C35" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="D35" t="s">
-        <v>491</v>
+        <v>497</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B36" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="C36" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D36" t="s">
-        <v>492</v>
+        <v>498</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B37" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="C37" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="D37" t="s">
-        <v>493</v>
+        <v>499</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B38" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="C38" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="D38" t="s">
-        <v>494</v>
+        <v>500</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B39" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C39" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="D39" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B40" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="C40" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="D40" t="s">
-        <v>496</v>
+        <v>502</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B41" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C41" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="D41" t="s">
-        <v>497</v>
+        <v>503</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B42" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="C42" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="D42" t="s">
-        <v>498</v>
+        <v>504</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B43" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="C43" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="D43" t="s">
-        <v>499</v>
+        <v>505</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B44" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="C44" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="D44" t="s">
-        <v>500</v>
+        <v>506</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B45" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C45" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="D45" t="s">
-        <v>501</v>
+        <v>507</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B46" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="C46" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D46" t="s">
-        <v>502</v>
+        <v>508</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B47" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="C47" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="D47" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B48" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="C48" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="D48" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B49" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C49" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="D49" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B50" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="C50" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="D50" t="s">
-        <v>506</v>
+        <v>512</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B51" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="C51" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="D51" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B52" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="C52" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="D52" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B53" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="C53" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="D53" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B54" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="C54" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="D54" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B55" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="C55" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="D55" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B56" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C56" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="D56" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B57" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="C57" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="D57" t="s">
-        <v>513</v>
+        <v>519</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B58" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C58" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="D58" t="s">
-        <v>514</v>
+        <v>520</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B59" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="C59" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="D59" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B60" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="C60" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="D60" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
     </row>
     <row r="61" spans="1:4">
       <c r="A61" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B61" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C61" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="D61" t="s">
-        <v>517</v>
+        <v>523</v>
       </c>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B62" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="C62" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="D62" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
     </row>
     <row r="63" spans="1:4">
       <c r="A63" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B63" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="C63" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="D63" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
     </row>
     <row r="64" spans="1:4">
       <c r="A64" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B64" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="C64" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="D64" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
     </row>
     <row r="65" spans="1:4">
       <c r="A65" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B65" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="C65" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="D65" t="s">
-        <v>521</v>
+        <v>527</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B66" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C66" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="D66" t="s">
-        <v>522</v>
+        <v>528</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B67" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="C67" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="D67" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
     </row>
     <row r="68" spans="1:4">
       <c r="A68" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B68" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="C68" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="D68" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
     </row>
     <row r="69" spans="1:4">
       <c r="A69" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B69" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="C69" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="D69" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B70" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="C70" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="D70" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
     </row>
     <row r="71" spans="1:4">
       <c r="A71" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B71" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C71" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="D71" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
     </row>
     <row r="72" spans="1:4">
       <c r="A72" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B72" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="C72" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="D72" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B73" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="C73" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="D73" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
     </row>
     <row r="74" spans="1:4">
       <c r="A74" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B74" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="C74" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="D74" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
     </row>
     <row r="75" spans="1:4">
       <c r="A75" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B75" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="C75" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="D75" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
     </row>
     <row r="76" spans="1:4">
       <c r="A76" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B76" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="C76" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="D76" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B77" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="C77" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="D77" t="s">
-        <v>533</v>
+        <v>539</v>
       </c>
     </row>
     <row r="78" spans="1:4">
       <c r="A78" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B78" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="C78" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="D78" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
     </row>
     <row r="79" spans="1:4">
       <c r="A79" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B79" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="C79" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="D79" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
     </row>
     <row r="80" spans="1:4">
       <c r="A80" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B80" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="C80" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="D80" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
     </row>
     <row r="81" spans="1:4">
       <c r="A81" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B81" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="C81" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="D81" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
     </row>
     <row r="82" spans="1:4">
       <c r="A82" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B82" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="C82" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="D82" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
     </row>
     <row r="83" spans="1:4">
       <c r="A83" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B83" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="C83" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="D83" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
     </row>
     <row r="84" spans="1:4">
       <c r="A84" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B84" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="C84" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="D84" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
     </row>
     <row r="85" spans="1:4">
       <c r="A85" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B85" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="C85" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="D85" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
     </row>
     <row r="86" spans="1:4">
       <c r="A86" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B86" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="C86" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="D86" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
     </row>
     <row r="87" spans="1:4">
       <c r="A87" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B87" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="C87" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="D87" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
     </row>
     <row r="88" spans="1:4">
       <c r="A88" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B88" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="C88" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="D88" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
     </row>
     <row r="89" spans="1:4">
       <c r="A89" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B89" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="C89" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="D89" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
     </row>
     <row r="90" spans="1:4">
       <c r="A90" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B90" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="C90" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="D90" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
     </row>
     <row r="91" spans="1:4">
       <c r="A91" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B91" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="C91" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="D91" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
     </row>
     <row r="92" spans="1:4">
       <c r="A92" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B92" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="C92" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="D92" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
     </row>
     <row r="93" spans="1:4">
       <c r="A93" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B93" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="C93" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="D93" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
     </row>
     <row r="94" spans="1:4">
       <c r="A94" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B94" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="C94" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="D94" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
     </row>
     <row r="95" spans="1:4">
       <c r="A95" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B95" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="C95" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="D95" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
     </row>
     <row r="96" spans="1:4">
       <c r="A96" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B96" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="C96" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="D96" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
     </row>
     <row r="97" spans="1:4">
       <c r="A97" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B97" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="C97" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="D97" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
     </row>
     <row r="98" spans="1:4">
       <c r="A98" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B98" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="C98" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="D98" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
     </row>
     <row r="99" spans="1:4">
       <c r="A99" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B99" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="C99" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="D99" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
     </row>
     <row r="100" spans="1:4">
       <c r="A100" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B100" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="C100" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="D100" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
     </row>
     <row r="101" spans="1:4">
       <c r="A101" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B101" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="C101" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="D101" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
     </row>
     <row r="102" spans="1:4">
       <c r="A102" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B102" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="C102" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="D102" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
     </row>
     <row r="103" spans="1:4">
       <c r="A103" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B103" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="C103" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="D103" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
     </row>
     <row r="104" spans="1:4">
       <c r="A104" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B104" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="C104" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="D104" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
     </row>
     <row r="105" spans="1:4">
       <c r="A105" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B105" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="C105" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D105" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
     </row>
     <row r="106" spans="1:4">
       <c r="A106" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B106" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="C106" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="D106" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
     </row>
     <row r="107" spans="1:4">
       <c r="A107" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B107" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="C107" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="D107" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
     </row>
     <row r="108" spans="1:4">
       <c r="A108" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B108" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="C108" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="D108" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
     </row>
     <row r="109" spans="1:4">
       <c r="A109" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B109" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="C109" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="D109" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
     </row>
     <row r="110" spans="1:4">
       <c r="A110" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B110" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="C110" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="D110" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
     </row>
     <row r="111" spans="1:4">
       <c r="A111" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B111" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="C111" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="D111" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
     </row>
     <row r="112" spans="1:4">
       <c r="A112" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B112" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="C112" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="D112" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
     </row>
     <row r="113" spans="1:4">
       <c r="A113" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B113" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="C113" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="D113" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
     </row>
     <row r="114" spans="1:4">
       <c r="A114" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B114" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="C114" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="D114" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
     </row>
     <row r="115" spans="1:4">
       <c r="A115" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B115" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="C115" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="D115" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
     </row>
     <row r="116" spans="1:4">
       <c r="A116" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B116" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="C116" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="D116" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
     </row>
     <row r="117" spans="1:4">
       <c r="A117" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B117" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="C117" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="D117" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
     </row>
     <row r="118" spans="1:4">
       <c r="A118" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B118" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="C118" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="D118" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
     </row>
     <row r="119" spans="1:4">
       <c r="A119" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B119" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="C119" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="D119" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
     </row>
     <row r="120" spans="1:4">
       <c r="A120" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B120" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="C120" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="D120" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
     </row>
     <row r="121" spans="1:4">
       <c r="A121" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B121" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="C121" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="D121" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
     </row>
     <row r="122" spans="1:4">
       <c r="A122" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B122" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="C122" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="D122" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
     </row>
     <row r="123" spans="1:4">
       <c r="A123" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B123" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="C123" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="D123" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
     </row>
     <row r="124" spans="1:4">
       <c r="A124" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B124" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="C124" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="D124" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
     </row>
     <row r="125" spans="1:4">
       <c r="A125" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B125" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="C125" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="D125" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
     </row>
     <row r="126" spans="1:4">
       <c r="A126" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B126" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="C126" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="D126" t="s">
-        <v>582</v>
+        <v>588</v>
       </c>
     </row>
     <row r="127" spans="1:4">
       <c r="A127" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B127" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="C127" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="D127" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
     </row>
     <row r="128" spans="1:4">
       <c r="A128" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B128" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="C128" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="D128" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
     </row>
     <row r="129" spans="1:4">
       <c r="A129" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B129" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="C129" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="D129" t="s">
-        <v>585</v>
+        <v>591</v>
       </c>
     </row>
     <row r="130" spans="1:4">
       <c r="A130" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B130" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="C130" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="D130" t="s">
-        <v>586</v>
+        <v>592</v>
       </c>
     </row>
     <row r="131" spans="1:4">
       <c r="A131" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B131" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="C131" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="D131" t="s">
-        <v>587</v>
+        <v>593</v>
       </c>
     </row>
     <row r="132" spans="1:4">
       <c r="A132" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B132" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="C132" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="D132" t="s">
-        <v>588</v>
+        <v>594</v>
       </c>
     </row>
     <row r="133" spans="1:4">
       <c r="A133" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B133" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="C133" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="D133" t="s">
-        <v>589</v>
+        <v>595</v>
       </c>
     </row>
     <row r="134" spans="1:4">
       <c r="A134" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B134" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="C134" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="D134" t="s">
-        <v>590</v>
+        <v>596</v>
       </c>
     </row>
     <row r="135" spans="1:4">
       <c r="A135" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B135" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="C135" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="D135" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
     </row>
     <row r="136" spans="1:4">
       <c r="A136" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B136" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="C136" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="D136" t="s">
-        <v>592</v>
+        <v>598</v>
       </c>
     </row>
     <row r="137" spans="1:4">
       <c r="A137" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B137" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C137" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="D137" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
     </row>
     <row r="138" spans="1:4">
       <c r="A138" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B138" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="C138" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="D138" t="s">
-        <v>594</v>
+        <v>600</v>
       </c>
     </row>
     <row r="139" spans="1:4">
       <c r="A139" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B139" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="C139" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="D139" t="s">
-        <v>595</v>
+        <v>601</v>
       </c>
     </row>
     <row r="140" spans="1:4">
       <c r="A140" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B140" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="C140" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="D140" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
     </row>
     <row r="141" spans="1:4">
       <c r="A141" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B141" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="C141" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="D141" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
     </row>
     <row r="142" spans="1:4">
       <c r="A142" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B142" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="C142" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="D142" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
     </row>
     <row r="143" spans="1:4">
       <c r="A143" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B143" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="C143" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="D143" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
     </row>
     <row r="144" spans="1:4">
       <c r="A144" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B144" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="C144" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="D144" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
     </row>
     <row r="145" spans="1:4">
       <c r="A145" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B145" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="C145" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="D145" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
     </row>
     <row r="146" spans="1:4">
       <c r="A146" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B146" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="C146" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="D146" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
     </row>
     <row r="147" spans="1:4">
       <c r="A147" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B147" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="C147" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="D147" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
     </row>
     <row r="148" spans="1:4">
       <c r="A148" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B148" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="C148" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="D148" t="s">
-        <v>604</v>
+        <v>610</v>
       </c>
     </row>
     <row r="149" spans="1:4">
       <c r="A149" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B149" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="C149" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="D149" t="s">
-        <v>605</v>
+        <v>611</v>
       </c>
     </row>
     <row r="150" spans="1:4">
       <c r="A150" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B150" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="C150" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="D150" t="s">
-        <v>606</v>
+        <v>612</v>
       </c>
     </row>
     <row r="151" spans="1:4">
       <c r="A151" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B151" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="C151" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="D151" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
     </row>
     <row r="152" spans="1:4">
       <c r="A152" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B152" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="C152" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="D152" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
     </row>
     <row r="153" spans="1:4">
       <c r="A153" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B153" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="C153" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="D153" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
     </row>
     <row r="154" spans="1:4">
       <c r="A154" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B154" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="C154" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="D154" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
     </row>
     <row r="155" spans="1:4">
       <c r="A155" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B155" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="C155" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="D155" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
     </row>
     <row r="156" spans="1:4">
       <c r="A156" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B156" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="C156" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="D156" t="s">
-        <v>612</v>
+        <v>618</v>
       </c>
     </row>
     <row r="157" spans="1:4">
       <c r="A157" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B157" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="C157" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="D157" t="s">
-        <v>613</v>
+        <v>619</v>
       </c>
     </row>
     <row r="158" spans="1:4">
       <c r="A158" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B158" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="C158" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="D158" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
     </row>
     <row r="159" spans="1:4">
       <c r="A159" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B159" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="C159" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="D159" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
     </row>
     <row r="160" spans="1:4">
       <c r="A160" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B160" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="C160" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="D160" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
     </row>
     <row r="161" spans="1:4">
       <c r="A161" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B161" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="C161" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="D161" t="s">
-        <v>617</v>
+        <v>623</v>
       </c>
     </row>
     <row r="162" spans="1:4">
       <c r="A162" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B162" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="C162" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="D162" t="s">
-        <v>618</v>
+        <v>624</v>
       </c>
     </row>
     <row r="163" spans="1:4">
       <c r="A163" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B163" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="C163" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="D163" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
     </row>
     <row r="164" spans="1:4">
       <c r="A164" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B164" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="C164" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="D164" t="s">
-        <v>620</v>
+        <v>626</v>
       </c>
     </row>
     <row r="165" spans="1:4">
       <c r="A165" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B165" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="C165" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="D165" t="s">
-        <v>621</v>
+        <v>627</v>
       </c>
     </row>
     <row r="166" spans="1:4">
       <c r="A166" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B166" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="C166" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="D166" t="s">
-        <v>622</v>
+        <v>628</v>
       </c>
     </row>
     <row r="167" spans="1:4">
       <c r="A167" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B167" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="C167" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="D167" t="s">
-        <v>623</v>
+        <v>629</v>
       </c>
     </row>
     <row r="168" spans="1:4">
       <c r="A168" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B168" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="C168" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="D168" t="s">
-        <v>624</v>
+        <v>630</v>
       </c>
     </row>
     <row r="169" spans="1:4">
       <c r="A169" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B169" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="C169" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="D169" t="s">
-        <v>625</v>
+        <v>631</v>
       </c>
     </row>
     <row r="170" spans="1:4">
       <c r="A170" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B170" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="C170" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="D170" t="s">
-        <v>626</v>
+        <v>632</v>
       </c>
     </row>
     <row r="171" spans="1:4">
       <c r="A171" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B171" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="C171" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="D171" t="s">
-        <v>627</v>
+        <v>633</v>
       </c>
     </row>
     <row r="172" spans="1:4">
       <c r="A172" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B172" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="C172" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="D172" t="s">
-        <v>628</v>
+        <v>634</v>
       </c>
     </row>
     <row r="173" spans="1:4">
       <c r="A173" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B173" t="s">
-        <v>400</v>
+        <v>405</v>
       </c>
       <c r="C173" t="s">
-        <v>400</v>
+        <v>405</v>
       </c>
       <c r="D173" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
     </row>
     <row r="174" spans="1:4">
       <c r="A174" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B174" t="s">
-        <v>401</v>
+        <v>406</v>
       </c>
       <c r="C174" t="s">
-        <v>401</v>
+        <v>406</v>
       </c>
       <c r="D174" t="s">
-        <v>630</v>
+        <v>636</v>
       </c>
     </row>
     <row r="175" spans="1:4">
       <c r="A175" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B175" t="s">
-        <v>402</v>
+        <v>407</v>
       </c>
       <c r="C175" t="s">
-        <v>402</v>
+        <v>407</v>
       </c>
       <c r="D175" t="s">
-        <v>631</v>
+        <v>637</v>
       </c>
     </row>
     <row r="176" spans="1:4">
       <c r="A176" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B176" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
       <c r="C176" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
       <c r="D176" t="s">
-        <v>632</v>
+        <v>638</v>
       </c>
     </row>
     <row r="177" spans="1:4">
       <c r="A177" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B177" t="s">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="C177" t="s">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="D177" t="s">
-        <v>633</v>
+        <v>639</v>
       </c>
     </row>
     <row r="178" spans="1:4">
       <c r="A178" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B178" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="C178" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="D178" t="s">
-        <v>634</v>
+        <v>640</v>
       </c>
     </row>
     <row r="179" spans="1:4">
       <c r="A179" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B179" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
       <c r="C179" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
       <c r="D179" t="s">
-        <v>635</v>
+        <v>641</v>
       </c>
     </row>
     <row r="180" spans="1:4">
       <c r="A180" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B180" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
       <c r="C180" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
       <c r="D180" t="s">
-        <v>636</v>
+        <v>642</v>
       </c>
     </row>
     <row r="181" spans="1:4">
       <c r="A181" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B181" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
       <c r="C181" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
       <c r="D181" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
     </row>
     <row r="182" spans="1:4">
       <c r="A182" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B182" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="C182" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="D182" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
     </row>
     <row r="183" spans="1:4">
       <c r="A183" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B183" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="C183" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="D183" t="s">
-        <v>639</v>
+        <v>645</v>
       </c>
     </row>
     <row r="184" spans="1:4">
       <c r="A184" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B184" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="C184" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="D184" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
     </row>
     <row r="185" spans="1:4">
       <c r="A185" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B185" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="C185" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="D185" t="s">
-        <v>641</v>
+        <v>647</v>
       </c>
     </row>
     <row r="186" spans="1:4">
       <c r="A186" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B186" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="C186" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="D186" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
     </row>
     <row r="187" spans="1:4">
       <c r="A187" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B187" t="s">
-        <v>414</v>
+        <v>419</v>
       </c>
       <c r="C187" t="s">
-        <v>414</v>
+        <v>419</v>
       </c>
       <c r="D187" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
     </row>
     <row r="188" spans="1:4">
       <c r="A188" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B188" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
       <c r="C188" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
       <c r="D188" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
     </row>
     <row r="189" spans="1:4">
       <c r="A189" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B189" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="C189" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="D189" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
     </row>
     <row r="190" spans="1:4">
       <c r="A190" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B190" t="s">
-        <v>417</v>
+        <v>422</v>
       </c>
       <c r="C190" t="s">
-        <v>417</v>
+        <v>422</v>
       </c>
       <c r="D190" t="s">
-        <v>646</v>
+        <v>652</v>
       </c>
     </row>
     <row r="191" spans="1:4">
       <c r="A191" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B191" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="C191" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="D191" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
     </row>
     <row r="192" spans="1:4">
       <c r="A192" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B192" t="s">
-        <v>419</v>
+        <v>424</v>
       </c>
       <c r="C192" t="s">
-        <v>419</v>
+        <v>424</v>
       </c>
       <c r="D192" t="s">
-        <v>648</v>
+        <v>654</v>
       </c>
     </row>
     <row r="193" spans="1:4">
       <c r="A193" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B193" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="C193" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="D193" t="s">
-        <v>649</v>
+        <v>655</v>
       </c>
     </row>
     <row r="194" spans="1:4">
       <c r="A194" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B194" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="C194" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="D194" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
     </row>
     <row r="195" spans="1:4">
       <c r="A195" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B195" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="C195" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="D195" t="s">
-        <v>651</v>
+        <v>657</v>
       </c>
     </row>
     <row r="196" spans="1:4">
       <c r="A196" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B196" t="s">
-        <v>423</v>
+        <v>428</v>
       </c>
       <c r="C196" t="s">
-        <v>423</v>
+        <v>428</v>
       </c>
       <c r="D196" t="s">
-        <v>652</v>
+        <v>658</v>
       </c>
     </row>
     <row r="197" spans="1:4">
       <c r="A197" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B197" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="C197" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="D197" t="s">
-        <v>653</v>
+        <v>659</v>
       </c>
     </row>
     <row r="198" spans="1:4">
       <c r="A198" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B198" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="C198" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="D198" t="s">
-        <v>654</v>
+        <v>660</v>
       </c>
     </row>
     <row r="199" spans="1:4">
       <c r="A199" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B199" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
       <c r="C199" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
       <c r="D199" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
     </row>
     <row r="200" spans="1:4">
       <c r="A200" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B200" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
       <c r="C200" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
       <c r="D200" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
     </row>
     <row r="201" spans="1:4">
       <c r="A201" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B201" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
       <c r="C201" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
       <c r="D201" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
     </row>
     <row r="202" spans="1:4">
       <c r="A202" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B202" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="C202" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
       <c r="D202" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
     </row>
     <row r="203" spans="1:4">
       <c r="A203" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B203" t="s">
-        <v>430</v>
+        <v>435</v>
       </c>
       <c r="C203" t="s">
-        <v>430</v>
+        <v>435</v>
       </c>
       <c r="D203" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
     </row>
     <row r="204" spans="1:4">
       <c r="A204" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B204" t="s">
-        <v>431</v>
+        <v>436</v>
       </c>
       <c r="C204" t="s">
-        <v>431</v>
+        <v>436</v>
       </c>
       <c r="D204" t="s">
-        <v>660</v>
+        <v>666</v>
       </c>
     </row>
     <row r="205" spans="1:4">
       <c r="A205" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B205" t="s">
-        <v>432</v>
+        <v>437</v>
       </c>
       <c r="C205" t="s">
-        <v>432</v>
+        <v>437</v>
       </c>
       <c r="D205" t="s">
-        <v>661</v>
+        <v>667</v>
       </c>
     </row>
     <row r="206" spans="1:4">
       <c r="A206" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B206" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
       <c r="C206" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
       <c r="D206" t="s">
-        <v>662</v>
+        <v>668</v>
       </c>
     </row>
     <row r="207" spans="1:4">
       <c r="A207" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B207" t="s">
-        <v>434</v>
+        <v>439</v>
       </c>
       <c r="C207" t="s">
-        <v>434</v>
+        <v>439</v>
       </c>
       <c r="D207" t="s">
-        <v>663</v>
+        <v>669</v>
       </c>
     </row>
     <row r="208" spans="1:4">
       <c r="A208" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B208" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
       <c r="C208" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
       <c r="D208" t="s">
-        <v>664</v>
+        <v>670</v>
       </c>
     </row>
     <row r="209" spans="1:4">
       <c r="A209" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B209" t="s">
-        <v>436</v>
+        <v>441</v>
       </c>
       <c r="C209" t="s">
-        <v>436</v>
+        <v>441</v>
       </c>
       <c r="D209" t="s">
-        <v>665</v>
+        <v>671</v>
       </c>
     </row>
     <row r="210" spans="1:4">
       <c r="A210" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B210" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
       <c r="C210" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
       <c r="D210" t="s">
-        <v>666</v>
+        <v>672</v>
       </c>
     </row>
     <row r="211" spans="1:4">
       <c r="A211" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B211" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
       <c r="C211" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
       <c r="D211" t="s">
-        <v>667</v>
+        <v>673</v>
       </c>
     </row>
     <row r="212" spans="1:4">
       <c r="A212" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B212" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
       <c r="C212" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
       <c r="D212" t="s">
-        <v>668</v>
+        <v>674</v>
       </c>
     </row>
     <row r="213" spans="1:4">
       <c r="A213" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B213" t="s">
-        <v>440</v>
+        <v>445</v>
       </c>
       <c r="C213" t="s">
-        <v>440</v>
+        <v>445</v>
       </c>
       <c r="D213" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
     </row>
     <row r="214" spans="1:4">
       <c r="A214" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B214" t="s">
-        <v>441</v>
+        <v>446</v>
       </c>
       <c r="C214" t="s">
-        <v>441</v>
+        <v>446</v>
       </c>
       <c r="D214" t="s">
-        <v>670</v>
+        <v>676</v>
       </c>
     </row>
     <row r="215" spans="1:4">
       <c r="A215" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B215" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="C215" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="D215" t="s">
-        <v>671</v>
+        <v>677</v>
       </c>
     </row>
     <row r="216" spans="1:4">
       <c r="A216" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B216" t="s">
-        <v>443</v>
+        <v>448</v>
       </c>
       <c r="C216" t="s">
-        <v>443</v>
+        <v>448</v>
       </c>
       <c r="D216" t="s">
-        <v>672</v>
+        <v>678</v>
       </c>
     </row>
     <row r="217" spans="1:4">
       <c r="A217" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B217" t="s">
-        <v>444</v>
+        <v>449</v>
       </c>
       <c r="C217" t="s">
-        <v>444</v>
+        <v>449</v>
       </c>
       <c r="D217" t="s">
-        <v>673</v>
+        <v>679</v>
       </c>
     </row>
     <row r="218" spans="1:4">
       <c r="A218" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B218" t="s">
-        <v>445</v>
+        <v>450</v>
       </c>
       <c r="C218" t="s">
-        <v>445</v>
+        <v>450</v>
       </c>
       <c r="D218" t="s">
-        <v>674</v>
+        <v>680</v>
       </c>
     </row>
     <row r="219" spans="1:4">
       <c r="A219" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B219" t="s">
-        <v>446</v>
+        <v>451</v>
       </c>
       <c r="C219" t="s">
-        <v>446</v>
+        <v>451</v>
       </c>
       <c r="D219" t="s">
-        <v>675</v>
+        <v>681</v>
       </c>
     </row>
     <row r="220" spans="1:4">
       <c r="A220" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B220" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
       <c r="C220" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
       <c r="D220" t="s">
-        <v>676</v>
+        <v>682</v>
       </c>
     </row>
     <row r="221" spans="1:4">
       <c r="A221" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B221" t="s">
-        <v>448</v>
+        <v>453</v>
       </c>
       <c r="C221" t="s">
-        <v>448</v>
+        <v>453</v>
       </c>
       <c r="D221" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
     </row>
     <row r="222" spans="1:4">
       <c r="A222" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B222" t="s">
-        <v>449</v>
+        <v>454</v>
       </c>
       <c r="C222" t="s">
-        <v>449</v>
+        <v>454</v>
       </c>
       <c r="D222" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
     </row>
     <row r="223" spans="1:4">
       <c r="A223" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B223" t="s">
-        <v>450</v>
+        <v>455</v>
       </c>
       <c r="C223" t="s">
-        <v>450</v>
+        <v>455</v>
       </c>
       <c r="D223" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
     </row>
     <row r="224" spans="1:4">
       <c r="A224" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B224" t="s">
-        <v>451</v>
+        <v>456</v>
       </c>
       <c r="C224" t="s">
-        <v>451</v>
+        <v>456</v>
       </c>
       <c r="D224" t="s">
-        <v>680</v>
+        <v>686</v>
       </c>
     </row>
     <row r="225" spans="1:4">
       <c r="A225" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B225" t="s">
-        <v>452</v>
+        <v>457</v>
       </c>
       <c r="C225" t="s">
-        <v>452</v>
+        <v>457</v>
       </c>
       <c r="D225" t="s">
-        <v>681</v>
+        <v>687</v>
       </c>
     </row>
     <row r="226" spans="1:4">
       <c r="A226" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B226" t="s">
-        <v>453</v>
+        <v>458</v>
       </c>
       <c r="C226" t="s">
-        <v>453</v>
+        <v>458</v>
       </c>
       <c r="D226" t="s">
-        <v>682</v>
+        <v>688</v>
       </c>
     </row>
     <row r="227" spans="1:4">
       <c r="A227" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B227" t="s">
-        <v>454</v>
+        <v>459</v>
       </c>
       <c r="C227" t="s">
-        <v>454</v>
+        <v>459</v>
       </c>
       <c r="D227" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
     </row>
     <row r="228" spans="1:4">
       <c r="A228" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B228" t="s">
-        <v>455</v>
+        <v>460</v>
       </c>
       <c r="C228" t="s">
-        <v>455</v>
+        <v>460</v>
       </c>
       <c r="D228" t="s">
-        <v>684</v>
+        <v>690</v>
       </c>
     </row>
     <row r="229" spans="1:4">
       <c r="A229" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B229" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="C229" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="D229" t="s">
-        <v>685</v>
+        <v>691</v>
       </c>
     </row>
     <row r="230" spans="1:4">
       <c r="A230" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B230" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="C230" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="D230" t="s">
-        <v>686</v>
+        <v>692</v>
+      </c>
+    </row>
+    <row r="231" spans="1:4">
+      <c r="A231" t="s">
+        <v>233</v>
+      </c>
+      <c r="B231" t="s">
+        <v>463</v>
+      </c>
+      <c r="C231" t="s">
+        <v>463</v>
+      </c>
+      <c r="D231" t="s">
+        <v>693</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cập nhật Báo Cáo Đối Soát Đông Mát - 2026-10-07 10:42:33
</commit_message>
<xml_diff>
--- a/SPAM_PHIEU_CHUYEN/CHI TIẾT MÁT/Danh sách Siêu thị.xlsx
+++ b/SPAM_PHIEU_CHUYEN/CHI TIẾT MÁT/Danh sách Siêu thị.xlsx
@@ -205,7 +205,7 @@
     <t>KFM_BDU_DAN - B2.01.05 Tháp B Opal Boulevard</t>
   </si>
   <si>
-    <t>KFM_HCM_Q7 - A165 (Golden Star)</t>
+    <t>KFM_HCM_Q07 - B1.01 Chung cư Golden Star</t>
   </si>
   <si>
     <t>KFM_HCM_Q07 - Block K Happy Valley</t>
@@ -1585,7 +1585,7 @@
     <t>-5223853892</t>
   </si>
   <si>
-    <t>-1004427935189</t>
+    <t>-4906644767</t>
   </si>
   <si>
     <t>-5135406910</t>

</xml_diff>

<commit_message>
Cập nhật Báo Cáo Đối Soát Đông Mát - 2026-10-07 10:54:09
</commit_message>
<xml_diff>
--- a/SPAM_PHIEU_CHUYEN/CHI TIẾT MÁT/Danh sách Siêu thị.xlsx
+++ b/SPAM_PHIEU_CHUYEN/CHI TIẾT MÁT/Danh sách Siêu thị.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="694">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="928" uniqueCount="697">
   <si>
     <t>Tên Siêu thị</t>
   </si>
@@ -718,6 +718,9 @@
     <t>KFM_HCM_BTA - DC - A247 (Lê Cơ)</t>
   </si>
   <si>
+    <t>KFM_HCM_Q01 - Vinhomes Golden River</t>
+  </si>
+  <si>
     <t>A101</t>
   </si>
   <si>
@@ -1408,6 +1411,9 @@
     <t>A247</t>
   </si>
   <si>
+    <t>A222</t>
+  </si>
+  <si>
     <t>-4970846623</t>
   </si>
   <si>
@@ -2096,6 +2102,9 @@
   </si>
   <si>
     <t>-1004367466882</t>
+  </si>
+  <si>
+    <t>-1004368025959</t>
   </si>
 </sst>
 </file>
@@ -2427,7 +2436,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D231"/>
+  <dimension ref="A1:D232"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -2449,13 +2458,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D2" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2463,13 +2472,13 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D3" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2477,13 +2486,13 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D4" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2491,13 +2500,13 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C5" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D5" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2505,13 +2514,13 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D6" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2519,13 +2528,13 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C7" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D7" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2533,13 +2542,13 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C8" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D8" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2547,13 +2556,13 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C9" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D9" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2561,13 +2570,13 @@
         <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C10" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D10" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2575,13 +2584,13 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C11" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D11" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2589,13 +2598,13 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C12" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D12" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -2603,13 +2612,13 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C13" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D13" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -2617,13 +2626,13 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C14" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D14" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -2631,13 +2640,13 @@
         <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C15" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D15" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -2645,13 +2654,13 @@
         <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C16" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D16" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -2659,13 +2668,13 @@
         <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C17" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D17" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2673,13 +2682,13 @@
         <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C18" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D18" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -2687,13 +2696,13 @@
         <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C19" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D19" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -2701,13 +2710,13 @@
         <v>22</v>
       </c>
       <c r="B20" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C20" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D20" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -2715,13 +2724,13 @@
         <v>23</v>
       </c>
       <c r="B21" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C21" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D21" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -2729,13 +2738,13 @@
         <v>24</v>
       </c>
       <c r="B22" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C22" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D22" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -2743,13 +2752,13 @@
         <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C23" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D23" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -2757,13 +2766,13 @@
         <v>26</v>
       </c>
       <c r="B24" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C24" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D24" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -2771,13 +2780,13 @@
         <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C25" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D25" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -2785,13 +2794,13 @@
         <v>28</v>
       </c>
       <c r="B26" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C26" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D26" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -2799,13 +2808,13 @@
         <v>29</v>
       </c>
       <c r="B27" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C27" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D27" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -2813,13 +2822,13 @@
         <v>30</v>
       </c>
       <c r="B28" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C28" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D28" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -2827,13 +2836,13 @@
         <v>31</v>
       </c>
       <c r="B29" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C29" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D29" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -2841,13 +2850,13 @@
         <v>32</v>
       </c>
       <c r="B30" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C30" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D30" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -2855,13 +2864,13 @@
         <v>33</v>
       </c>
       <c r="B31" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C31" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D31" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -2869,13 +2878,13 @@
         <v>34</v>
       </c>
       <c r="B32" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C32" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D32" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -2883,13 +2892,13 @@
         <v>35</v>
       </c>
       <c r="B33" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C33" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D33" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -2897,13 +2906,13 @@
         <v>36</v>
       </c>
       <c r="B34" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C34" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D34" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -2911,13 +2920,13 @@
         <v>37</v>
       </c>
       <c r="B35" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C35" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D35" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -2925,13 +2934,13 @@
         <v>38</v>
       </c>
       <c r="B36" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C36" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D36" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -2939,13 +2948,13 @@
         <v>39</v>
       </c>
       <c r="B37" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C37" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D37" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -2953,13 +2962,13 @@
         <v>40</v>
       </c>
       <c r="B38" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C38" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D38" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -2967,13 +2976,13 @@
         <v>41</v>
       </c>
       <c r="B39" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C39" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D39" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -2981,13 +2990,13 @@
         <v>42</v>
       </c>
       <c r="B40" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C40" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D40" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -2995,13 +3004,13 @@
         <v>43</v>
       </c>
       <c r="B41" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C41" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D41" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -3009,13 +3018,13 @@
         <v>44</v>
       </c>
       <c r="B42" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C42" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D42" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -3023,13 +3032,13 @@
         <v>45</v>
       </c>
       <c r="B43" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C43" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D43" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -3037,13 +3046,13 @@
         <v>46</v>
       </c>
       <c r="B44" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C44" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D44" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -3051,13 +3060,13 @@
         <v>47</v>
       </c>
       <c r="B45" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C45" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D45" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -3065,13 +3074,13 @@
         <v>48</v>
       </c>
       <c r="B46" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C46" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D46" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -3079,13 +3088,13 @@
         <v>49</v>
       </c>
       <c r="B47" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C47" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D47" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -3093,13 +3102,13 @@
         <v>50</v>
       </c>
       <c r="B48" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C48" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D48" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -3107,13 +3116,13 @@
         <v>51</v>
       </c>
       <c r="B49" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C49" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D49" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -3121,13 +3130,13 @@
         <v>52</v>
       </c>
       <c r="B50" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C50" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D50" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -3135,13 +3144,13 @@
         <v>53</v>
       </c>
       <c r="B51" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C51" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D51" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -3149,13 +3158,13 @@
         <v>54</v>
       </c>
       <c r="B52" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C52" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D52" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -3163,13 +3172,13 @@
         <v>55</v>
       </c>
       <c r="B53" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C53" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D53" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -3177,13 +3186,13 @@
         <v>56</v>
       </c>
       <c r="B54" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C54" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D54" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -3191,13 +3200,13 @@
         <v>57</v>
       </c>
       <c r="B55" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C55" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D55" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -3205,13 +3214,13 @@
         <v>58</v>
       </c>
       <c r="B56" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C56" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D56" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -3219,13 +3228,13 @@
         <v>59</v>
       </c>
       <c r="B57" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C57" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D57" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -3233,13 +3242,13 @@
         <v>60</v>
       </c>
       <c r="B58" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C58" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D58" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -3247,13 +3256,13 @@
         <v>61</v>
       </c>
       <c r="B59" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C59" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D59" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -3261,13 +3270,13 @@
         <v>62</v>
       </c>
       <c r="B60" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C60" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D60" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -3275,13 +3284,13 @@
         <v>63</v>
       </c>
       <c r="B61" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C61" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D61" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -3289,13 +3298,13 @@
         <v>64</v>
       </c>
       <c r="B62" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C62" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D62" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -3303,13 +3312,13 @@
         <v>65</v>
       </c>
       <c r="B63" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C63" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D63" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -3317,13 +3326,13 @@
         <v>66</v>
       </c>
       <c r="B64" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C64" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D64" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -3331,13 +3340,13 @@
         <v>67</v>
       </c>
       <c r="B65" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C65" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D65" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -3345,13 +3354,13 @@
         <v>68</v>
       </c>
       <c r="B66" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C66" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D66" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -3359,13 +3368,13 @@
         <v>69</v>
       </c>
       <c r="B67" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C67" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D67" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -3373,13 +3382,13 @@
         <v>70</v>
       </c>
       <c r="B68" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C68" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D68" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -3387,13 +3396,13 @@
         <v>71</v>
       </c>
       <c r="B69" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C69" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D69" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -3401,13 +3410,13 @@
         <v>72</v>
       </c>
       <c r="B70" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C70" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D70" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -3415,13 +3424,13 @@
         <v>73</v>
       </c>
       <c r="B71" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C71" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D71" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -3429,13 +3438,13 @@
         <v>74</v>
       </c>
       <c r="B72" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C72" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D72" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -3443,13 +3452,13 @@
         <v>75</v>
       </c>
       <c r="B73" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C73" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D73" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -3457,13 +3466,13 @@
         <v>76</v>
       </c>
       <c r="B74" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C74" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D74" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -3471,13 +3480,13 @@
         <v>77</v>
       </c>
       <c r="B75" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C75" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D75" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -3485,13 +3494,13 @@
         <v>78</v>
       </c>
       <c r="B76" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C76" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D76" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -3499,13 +3508,13 @@
         <v>79</v>
       </c>
       <c r="B77" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C77" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D77" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -3513,13 +3522,13 @@
         <v>80</v>
       </c>
       <c r="B78" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C78" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D78" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -3527,13 +3536,13 @@
         <v>81</v>
       </c>
       <c r="B79" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C79" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D79" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -3541,13 +3550,13 @@
         <v>82</v>
       </c>
       <c r="B80" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C80" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D80" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -3555,13 +3564,13 @@
         <v>83</v>
       </c>
       <c r="B81" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C81" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D81" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
     </row>
     <row r="82" spans="1:4">
@@ -3569,13 +3578,13 @@
         <v>84</v>
       </c>
       <c r="B82" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C82" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D82" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -3583,13 +3592,13 @@
         <v>85</v>
       </c>
       <c r="B83" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C83" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D83" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -3597,13 +3606,13 @@
         <v>86</v>
       </c>
       <c r="B84" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C84" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D84" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -3611,13 +3620,13 @@
         <v>87</v>
       </c>
       <c r="B85" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C85" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D85" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="86" spans="1:4">
@@ -3625,13 +3634,13 @@
         <v>88</v>
       </c>
       <c r="B86" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C86" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D86" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
     </row>
     <row r="87" spans="1:4">
@@ -3639,13 +3648,13 @@
         <v>89</v>
       </c>
       <c r="B87" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C87" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D87" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
     </row>
     <row r="88" spans="1:4">
@@ -3653,13 +3662,13 @@
         <v>90</v>
       </c>
       <c r="B88" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C88" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D88" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -3667,13 +3676,13 @@
         <v>91</v>
       </c>
       <c r="B89" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C89" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D89" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
     </row>
     <row r="90" spans="1:4">
@@ -3681,13 +3690,13 @@
         <v>92</v>
       </c>
       <c r="B90" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C90" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D90" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -3695,13 +3704,13 @@
         <v>93</v>
       </c>
       <c r="B91" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C91" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D91" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
     </row>
     <row r="92" spans="1:4">
@@ -3709,13 +3718,13 @@
         <v>94</v>
       </c>
       <c r="B92" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C92" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D92" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
     </row>
     <row r="93" spans="1:4">
@@ -3723,13 +3732,13 @@
         <v>95</v>
       </c>
       <c r="B93" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C93" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D93" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
     </row>
     <row r="94" spans="1:4">
@@ -3737,13 +3746,13 @@
         <v>96</v>
       </c>
       <c r="B94" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C94" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D94" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
     </row>
     <row r="95" spans="1:4">
@@ -3751,13 +3760,13 @@
         <v>97</v>
       </c>
       <c r="B95" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C95" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D95" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
     </row>
     <row r="96" spans="1:4">
@@ -3765,13 +3774,13 @@
         <v>98</v>
       </c>
       <c r="B96" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C96" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D96" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
     </row>
     <row r="97" spans="1:4">
@@ -3779,13 +3788,13 @@
         <v>99</v>
       </c>
       <c r="B97" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C97" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D97" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
     </row>
     <row r="98" spans="1:4">
@@ -3793,13 +3802,13 @@
         <v>100</v>
       </c>
       <c r="B98" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C98" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D98" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
     </row>
     <row r="99" spans="1:4">
@@ -3807,13 +3816,13 @@
         <v>101</v>
       </c>
       <c r="B99" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C99" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D99" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
     </row>
     <row r="100" spans="1:4">
@@ -3821,13 +3830,13 @@
         <v>102</v>
       </c>
       <c r="B100" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C100" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D100" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
     </row>
     <row r="101" spans="1:4">
@@ -3835,13 +3844,13 @@
         <v>103</v>
       </c>
       <c r="B101" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C101" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D101" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
     </row>
     <row r="102" spans="1:4">
@@ -3849,13 +3858,13 @@
         <v>104</v>
       </c>
       <c r="B102" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C102" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D102" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
     </row>
     <row r="103" spans="1:4">
@@ -3863,13 +3872,13 @@
         <v>105</v>
       </c>
       <c r="B103" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C103" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D103" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
     </row>
     <row r="104" spans="1:4">
@@ -3877,13 +3886,13 @@
         <v>106</v>
       </c>
       <c r="B104" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C104" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D104" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
     </row>
     <row r="105" spans="1:4">
@@ -3891,13 +3900,13 @@
         <v>107</v>
       </c>
       <c r="B105" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C105" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D105" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
     </row>
     <row r="106" spans="1:4">
@@ -3905,13 +3914,13 @@
         <v>108</v>
       </c>
       <c r="B106" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C106" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D106" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
     </row>
     <row r="107" spans="1:4">
@@ -3919,13 +3928,13 @@
         <v>109</v>
       </c>
       <c r="B107" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C107" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D107" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="108" spans="1:4">
@@ -3933,13 +3942,13 @@
         <v>110</v>
       </c>
       <c r="B108" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C108" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D108" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="109" spans="1:4">
@@ -3947,13 +3956,13 @@
         <v>111</v>
       </c>
       <c r="B109" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C109" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D109" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
     </row>
     <row r="110" spans="1:4">
@@ -3961,13 +3970,13 @@
         <v>112</v>
       </c>
       <c r="B110" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C110" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D110" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
     </row>
     <row r="111" spans="1:4">
@@ -3975,13 +3984,13 @@
         <v>113</v>
       </c>
       <c r="B111" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C111" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D111" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
     </row>
     <row r="112" spans="1:4">
@@ -3989,13 +3998,13 @@
         <v>114</v>
       </c>
       <c r="B112" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C112" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D112" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
     </row>
     <row r="113" spans="1:4">
@@ -4003,13 +4012,13 @@
         <v>115</v>
       </c>
       <c r="B113" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C113" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D113" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
     </row>
     <row r="114" spans="1:4">
@@ -4017,13 +4026,13 @@
         <v>116</v>
       </c>
       <c r="B114" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C114" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D114" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
     </row>
     <row r="115" spans="1:4">
@@ -4031,13 +4040,13 @@
         <v>117</v>
       </c>
       <c r="B115" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C115" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D115" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
     </row>
     <row r="116" spans="1:4">
@@ -4045,13 +4054,13 @@
         <v>118</v>
       </c>
       <c r="B116" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C116" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D116" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
     </row>
     <row r="117" spans="1:4">
@@ -4059,13 +4068,13 @@
         <v>119</v>
       </c>
       <c r="B117" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C117" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D117" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
     <row r="118" spans="1:4">
@@ -4073,13 +4082,13 @@
         <v>120</v>
       </c>
       <c r="B118" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C118" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D118" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
     </row>
     <row r="119" spans="1:4">
@@ -4087,13 +4096,13 @@
         <v>121</v>
       </c>
       <c r="B119" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C119" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D119" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
     </row>
     <row r="120" spans="1:4">
@@ -4101,13 +4110,13 @@
         <v>122</v>
       </c>
       <c r="B120" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C120" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D120" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
     </row>
     <row r="121" spans="1:4">
@@ -4115,13 +4124,13 @@
         <v>123</v>
       </c>
       <c r="B121" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C121" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D121" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
     </row>
     <row r="122" spans="1:4">
@@ -4129,13 +4138,13 @@
         <v>124</v>
       </c>
       <c r="B122" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C122" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D122" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
     </row>
     <row r="123" spans="1:4">
@@ -4143,13 +4152,13 @@
         <v>125</v>
       </c>
       <c r="B123" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C123" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D123" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="124" spans="1:4">
@@ -4157,13 +4166,13 @@
         <v>126</v>
       </c>
       <c r="B124" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C124" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D124" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
     </row>
     <row r="125" spans="1:4">
@@ -4171,13 +4180,13 @@
         <v>127</v>
       </c>
       <c r="B125" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C125" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D125" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
     </row>
     <row r="126" spans="1:4">
@@ -4185,13 +4194,13 @@
         <v>128</v>
       </c>
       <c r="B126" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C126" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D126" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
     </row>
     <row r="127" spans="1:4">
@@ -4199,13 +4208,13 @@
         <v>129</v>
       </c>
       <c r="B127" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C127" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D127" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
     </row>
     <row r="128" spans="1:4">
@@ -4213,13 +4222,13 @@
         <v>130</v>
       </c>
       <c r="B128" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C128" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D128" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
     </row>
     <row r="129" spans="1:4">
@@ -4227,13 +4236,13 @@
         <v>131</v>
       </c>
       <c r="B129" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C129" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D129" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
     </row>
     <row r="130" spans="1:4">
@@ -4241,13 +4250,13 @@
         <v>132</v>
       </c>
       <c r="B130" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C130" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D130" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
     </row>
     <row r="131" spans="1:4">
@@ -4255,13 +4264,13 @@
         <v>133</v>
       </c>
       <c r="B131" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C131" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D131" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
     </row>
     <row r="132" spans="1:4">
@@ -4269,13 +4278,13 @@
         <v>134</v>
       </c>
       <c r="B132" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C132" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D132" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
     </row>
     <row r="133" spans="1:4">
@@ -4283,13 +4292,13 @@
         <v>135</v>
       </c>
       <c r="B133" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C133" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D133" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="134" spans="1:4">
@@ -4297,13 +4306,13 @@
         <v>136</v>
       </c>
       <c r="B134" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C134" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D134" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
     </row>
     <row r="135" spans="1:4">
@@ -4311,13 +4320,13 @@
         <v>137</v>
       </c>
       <c r="B135" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C135" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D135" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
     </row>
     <row r="136" spans="1:4">
@@ -4325,13 +4334,13 @@
         <v>138</v>
       </c>
       <c r="B136" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C136" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D136" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
     </row>
     <row r="137" spans="1:4">
@@ -4339,13 +4348,13 @@
         <v>139</v>
       </c>
       <c r="B137" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C137" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D137" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
     </row>
     <row r="138" spans="1:4">
@@ -4353,13 +4362,13 @@
         <v>140</v>
       </c>
       <c r="B138" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C138" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D138" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
     </row>
     <row r="139" spans="1:4">
@@ -4367,13 +4376,13 @@
         <v>141</v>
       </c>
       <c r="B139" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C139" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D139" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
     </row>
     <row r="140" spans="1:4">
@@ -4381,13 +4390,13 @@
         <v>142</v>
       </c>
       <c r="B140" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C140" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D140" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
     </row>
     <row r="141" spans="1:4">
@@ -4395,13 +4404,13 @@
         <v>143</v>
       </c>
       <c r="B141" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C141" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D141" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
     </row>
     <row r="142" spans="1:4">
@@ -4409,13 +4418,13 @@
         <v>144</v>
       </c>
       <c r="B142" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C142" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D142" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
     </row>
     <row r="143" spans="1:4">
@@ -4423,13 +4432,13 @@
         <v>145</v>
       </c>
       <c r="B143" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C143" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D143" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
     </row>
     <row r="144" spans="1:4">
@@ -4437,13 +4446,13 @@
         <v>146</v>
       </c>
       <c r="B144" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C144" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D144" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
     </row>
     <row r="145" spans="1:4">
@@ -4451,13 +4460,13 @@
         <v>147</v>
       </c>
       <c r="B145" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C145" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D145" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
     </row>
     <row r="146" spans="1:4">
@@ -4465,13 +4474,13 @@
         <v>148</v>
       </c>
       <c r="B146" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C146" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D146" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
     </row>
     <row r="147" spans="1:4">
@@ -4479,13 +4488,13 @@
         <v>149</v>
       </c>
       <c r="B147" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C147" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D147" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
     </row>
     <row r="148" spans="1:4">
@@ -4493,13 +4502,13 @@
         <v>150</v>
       </c>
       <c r="B148" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C148" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D148" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
     </row>
     <row r="149" spans="1:4">
@@ -4507,13 +4516,13 @@
         <v>151</v>
       </c>
       <c r="B149" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C149" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D149" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
     </row>
     <row r="150" spans="1:4">
@@ -4521,13 +4530,13 @@
         <v>152</v>
       </c>
       <c r="B150" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C150" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D150" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
     </row>
     <row r="151" spans="1:4">
@@ -4535,13 +4544,13 @@
         <v>153</v>
       </c>
       <c r="B151" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C151" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D151" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
     </row>
     <row r="152" spans="1:4">
@@ -4549,13 +4558,13 @@
         <v>154</v>
       </c>
       <c r="B152" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C152" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="D152" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
     </row>
     <row r="153" spans="1:4">
@@ -4563,13 +4572,13 @@
         <v>155</v>
       </c>
       <c r="B153" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C153" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D153" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
     </row>
     <row r="154" spans="1:4">
@@ -4577,13 +4586,13 @@
         <v>156</v>
       </c>
       <c r="B154" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C154" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="D154" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
     </row>
     <row r="155" spans="1:4">
@@ -4591,13 +4600,13 @@
         <v>157</v>
       </c>
       <c r="B155" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C155" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D155" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
     </row>
     <row r="156" spans="1:4">
@@ -4605,13 +4614,13 @@
         <v>158</v>
       </c>
       <c r="B156" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C156" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D156" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
     </row>
     <row r="157" spans="1:4">
@@ -4619,13 +4628,13 @@
         <v>159</v>
       </c>
       <c r="B157" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C157" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D157" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
     </row>
     <row r="158" spans="1:4">
@@ -4633,13 +4642,13 @@
         <v>160</v>
       </c>
       <c r="B158" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C158" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D158" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
     </row>
     <row r="159" spans="1:4">
@@ -4647,13 +4656,13 @@
         <v>161</v>
       </c>
       <c r="B159" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C159" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D159" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
     </row>
     <row r="160" spans="1:4">
@@ -4661,13 +4670,13 @@
         <v>162</v>
       </c>
       <c r="B160" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C160" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D160" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
     </row>
     <row r="161" spans="1:4">
@@ -4675,13 +4684,13 @@
         <v>163</v>
       </c>
       <c r="B161" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C161" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D161" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
     </row>
     <row r="162" spans="1:4">
@@ -4689,13 +4698,13 @@
         <v>164</v>
       </c>
       <c r="B162" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C162" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="D162" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
     </row>
     <row r="163" spans="1:4">
@@ -4703,13 +4712,13 @@
         <v>165</v>
       </c>
       <c r="B163" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C163" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D163" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
     </row>
     <row r="164" spans="1:4">
@@ -4717,13 +4726,13 @@
         <v>166</v>
       </c>
       <c r="B164" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C164" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D164" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
     </row>
     <row r="165" spans="1:4">
@@ -4731,13 +4740,13 @@
         <v>167</v>
       </c>
       <c r="B165" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C165" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="D165" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
     </row>
     <row r="166" spans="1:4">
@@ -4745,13 +4754,13 @@
         <v>168</v>
       </c>
       <c r="B166" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C166" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D166" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
     </row>
     <row r="167" spans="1:4">
@@ -4759,13 +4768,13 @@
         <v>169</v>
       </c>
       <c r="B167" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C167" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D167" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
     </row>
     <row r="168" spans="1:4">
@@ -4773,13 +4782,13 @@
         <v>170</v>
       </c>
       <c r="B168" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C168" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D168" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
     </row>
     <row r="169" spans="1:4">
@@ -4787,13 +4796,13 @@
         <v>171</v>
       </c>
       <c r="B169" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C169" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D169" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
     </row>
     <row r="170" spans="1:4">
@@ -4801,13 +4810,13 @@
         <v>172</v>
       </c>
       <c r="B170" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C170" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="D170" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
     </row>
     <row r="171" spans="1:4">
@@ -4815,13 +4824,13 @@
         <v>173</v>
       </c>
       <c r="B171" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C171" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D171" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
     </row>
     <row r="172" spans="1:4">
@@ -4829,13 +4838,13 @@
         <v>174</v>
       </c>
       <c r="B172" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C172" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D172" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
     </row>
     <row r="173" spans="1:4">
@@ -4843,13 +4852,13 @@
         <v>175</v>
       </c>
       <c r="B173" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C173" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D173" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
     </row>
     <row r="174" spans="1:4">
@@ -4857,13 +4866,13 @@
         <v>176</v>
       </c>
       <c r="B174" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C174" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D174" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
     </row>
     <row r="175" spans="1:4">
@@ -4871,13 +4880,13 @@
         <v>177</v>
       </c>
       <c r="B175" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C175" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D175" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
     </row>
     <row r="176" spans="1:4">
@@ -4885,13 +4894,13 @@
         <v>178</v>
       </c>
       <c r="B176" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C176" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="D176" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
     </row>
     <row r="177" spans="1:4">
@@ -4899,13 +4908,13 @@
         <v>179</v>
       </c>
       <c r="B177" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C177" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D177" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
     </row>
     <row r="178" spans="1:4">
@@ -4913,13 +4922,13 @@
         <v>180</v>
       </c>
       <c r="B178" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C178" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D178" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
     </row>
     <row r="179" spans="1:4">
@@ -4927,13 +4936,13 @@
         <v>181</v>
       </c>
       <c r="B179" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C179" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D179" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
     </row>
     <row r="180" spans="1:4">
@@ -4941,13 +4950,13 @@
         <v>182</v>
       </c>
       <c r="B180" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C180" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D180" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
     </row>
     <row r="181" spans="1:4">
@@ -4955,13 +4964,13 @@
         <v>183</v>
       </c>
       <c r="B181" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C181" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D181" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
     </row>
     <row r="182" spans="1:4">
@@ -4969,13 +4978,13 @@
         <v>184</v>
       </c>
       <c r="B182" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C182" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="D182" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
     </row>
     <row r="183" spans="1:4">
@@ -4983,13 +4992,13 @@
         <v>185</v>
       </c>
       <c r="B183" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C183" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D183" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
     </row>
     <row r="184" spans="1:4">
@@ -4997,13 +5006,13 @@
         <v>186</v>
       </c>
       <c r="B184" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C184" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D184" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
     </row>
     <row r="185" spans="1:4">
@@ -5011,13 +5020,13 @@
         <v>187</v>
       </c>
       <c r="B185" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C185" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D185" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
     </row>
     <row r="186" spans="1:4">
@@ -5025,13 +5034,13 @@
         <v>188</v>
       </c>
       <c r="B186" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C186" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D186" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
     </row>
     <row r="187" spans="1:4">
@@ -5039,13 +5048,13 @@
         <v>189</v>
       </c>
       <c r="B187" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C187" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D187" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
     </row>
     <row r="188" spans="1:4">
@@ -5053,13 +5062,13 @@
         <v>190</v>
       </c>
       <c r="B188" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C188" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D188" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
     </row>
     <row r="189" spans="1:4">
@@ -5067,13 +5076,13 @@
         <v>191</v>
       </c>
       <c r="B189" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C189" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D189" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
     </row>
     <row r="190" spans="1:4">
@@ -5081,13 +5090,13 @@
         <v>192</v>
       </c>
       <c r="B190" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C190" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D190" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
     </row>
     <row r="191" spans="1:4">
@@ -5095,13 +5104,13 @@
         <v>193</v>
       </c>
       <c r="B191" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C191" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D191" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
     </row>
     <row r="192" spans="1:4">
@@ -5109,13 +5118,13 @@
         <v>194</v>
       </c>
       <c r="B192" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C192" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D192" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
     </row>
     <row r="193" spans="1:4">
@@ -5123,13 +5132,13 @@
         <v>195</v>
       </c>
       <c r="B193" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C193" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D193" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
     </row>
     <row r="194" spans="1:4">
@@ -5137,13 +5146,13 @@
         <v>196</v>
       </c>
       <c r="B194" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C194" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="D194" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
     </row>
     <row r="195" spans="1:4">
@@ -5151,13 +5160,13 @@
         <v>197</v>
       </c>
       <c r="B195" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C195" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D195" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
     </row>
     <row r="196" spans="1:4">
@@ -5165,13 +5174,13 @@
         <v>198</v>
       </c>
       <c r="B196" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C196" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="D196" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
     </row>
     <row r="197" spans="1:4">
@@ -5179,13 +5188,13 @@
         <v>199</v>
       </c>
       <c r="B197" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C197" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="D197" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
     </row>
     <row r="198" spans="1:4">
@@ -5193,13 +5202,13 @@
         <v>200</v>
       </c>
       <c r="B198" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C198" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="D198" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
     </row>
     <row r="199" spans="1:4">
@@ -5207,13 +5216,13 @@
         <v>201</v>
       </c>
       <c r="B199" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C199" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="D199" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
     </row>
     <row r="200" spans="1:4">
@@ -5221,13 +5230,13 @@
         <v>202</v>
       </c>
       <c r="B200" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C200" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="D200" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
     </row>
     <row r="201" spans="1:4">
@@ -5235,13 +5244,13 @@
         <v>203</v>
       </c>
       <c r="B201" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C201" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="D201" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
     </row>
     <row r="202" spans="1:4">
@@ -5249,13 +5258,13 @@
         <v>204</v>
       </c>
       <c r="B202" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C202" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="D202" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
     </row>
     <row r="203" spans="1:4">
@@ -5263,13 +5272,13 @@
         <v>205</v>
       </c>
       <c r="B203" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C203" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="D203" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
     </row>
     <row r="204" spans="1:4">
@@ -5277,13 +5286,13 @@
         <v>206</v>
       </c>
       <c r="B204" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C204" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="D204" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
     </row>
     <row r="205" spans="1:4">
@@ -5291,13 +5300,13 @@
         <v>207</v>
       </c>
       <c r="B205" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C205" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D205" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
     </row>
     <row r="206" spans="1:4">
@@ -5305,13 +5314,13 @@
         <v>208</v>
       </c>
       <c r="B206" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C206" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D206" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
     </row>
     <row r="207" spans="1:4">
@@ -5319,13 +5328,13 @@
         <v>209</v>
       </c>
       <c r="B207" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C207" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="D207" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
     </row>
     <row r="208" spans="1:4">
@@ -5333,13 +5342,13 @@
         <v>210</v>
       </c>
       <c r="B208" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C208" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D208" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
     </row>
     <row r="209" spans="1:4">
@@ -5347,13 +5356,13 @@
         <v>211</v>
       </c>
       <c r="B209" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C209" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D209" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
     </row>
     <row r="210" spans="1:4">
@@ -5361,13 +5370,13 @@
         <v>212</v>
       </c>
       <c r="B210" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C210" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D210" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
     </row>
     <row r="211" spans="1:4">
@@ -5375,13 +5384,13 @@
         <v>213</v>
       </c>
       <c r="B211" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C211" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="D211" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
     </row>
     <row r="212" spans="1:4">
@@ -5389,13 +5398,13 @@
         <v>214</v>
       </c>
       <c r="B212" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C212" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D212" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
     </row>
     <row r="213" spans="1:4">
@@ -5403,13 +5412,13 @@
         <v>215</v>
       </c>
       <c r="B213" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C213" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D213" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
     </row>
     <row r="214" spans="1:4">
@@ -5417,13 +5426,13 @@
         <v>216</v>
       </c>
       <c r="B214" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C214" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D214" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
     </row>
     <row r="215" spans="1:4">
@@ -5431,13 +5440,13 @@
         <v>217</v>
       </c>
       <c r="B215" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C215" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D215" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
     </row>
     <row r="216" spans="1:4">
@@ -5445,13 +5454,13 @@
         <v>218</v>
       </c>
       <c r="B216" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C216" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D216" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
     </row>
     <row r="217" spans="1:4">
@@ -5459,13 +5468,13 @@
         <v>219</v>
       </c>
       <c r="B217" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C217" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D217" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
     </row>
     <row r="218" spans="1:4">
@@ -5473,13 +5482,13 @@
         <v>220</v>
       </c>
       <c r="B218" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C218" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D218" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
     </row>
     <row r="219" spans="1:4">
@@ -5487,13 +5496,13 @@
         <v>221</v>
       </c>
       <c r="B219" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C219" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D219" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
     </row>
     <row r="220" spans="1:4">
@@ -5501,13 +5510,13 @@
         <v>222</v>
       </c>
       <c r="B220" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C220" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D220" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
     </row>
     <row r="221" spans="1:4">
@@ -5515,13 +5524,13 @@
         <v>223</v>
       </c>
       <c r="B221" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C221" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D221" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
     </row>
     <row r="222" spans="1:4">
@@ -5529,13 +5538,13 @@
         <v>224</v>
       </c>
       <c r="B222" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="C222" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D222" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
     </row>
     <row r="223" spans="1:4">
@@ -5543,13 +5552,13 @@
         <v>225</v>
       </c>
       <c r="B223" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C223" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="D223" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
     </row>
     <row r="224" spans="1:4">
@@ -5557,13 +5566,13 @@
         <v>226</v>
       </c>
       <c r="B224" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C224" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="D224" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
     </row>
     <row r="225" spans="1:4">
@@ -5571,13 +5580,13 @@
         <v>227</v>
       </c>
       <c r="B225" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C225" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D225" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
     </row>
     <row r="226" spans="1:4">
@@ -5585,13 +5594,13 @@
         <v>228</v>
       </c>
       <c r="B226" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C226" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="D226" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
     </row>
     <row r="227" spans="1:4">
@@ -5599,13 +5608,13 @@
         <v>229</v>
       </c>
       <c r="B227" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C227" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D227" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
     </row>
     <row r="228" spans="1:4">
@@ -5613,13 +5622,13 @@
         <v>230</v>
       </c>
       <c r="B228" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C228" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D228" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
     </row>
     <row r="229" spans="1:4">
@@ -5627,13 +5636,13 @@
         <v>231</v>
       </c>
       <c r="B229" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C229" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="D229" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
     </row>
     <row r="230" spans="1:4">
@@ -5641,13 +5650,13 @@
         <v>232</v>
       </c>
       <c r="B230" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C230" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D230" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
     </row>
     <row r="231" spans="1:4">
@@ -5655,13 +5664,27 @@
         <v>233</v>
       </c>
       <c r="B231" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C231" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="D231" t="s">
-        <v>693</v>
+        <v>695</v>
+      </c>
+    </row>
+    <row r="232" spans="1:4">
+      <c r="A232" t="s">
+        <v>234</v>
+      </c>
+      <c r="B232" t="s">
+        <v>465</v>
+      </c>
+      <c r="C232" t="s">
+        <v>465</v>
+      </c>
+      <c r="D232" t="s">
+        <v>696</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Realtime Telegram groups and store clusters
</commit_message>
<xml_diff>
--- a/SPAM_PHIEU_CHUYEN/CHI TIẾT MÁT/Danh sách Siêu thị.xlsx
+++ b/SPAM_PHIEU_CHUYEN/CHI TIẾT MÁT/Danh sách Siêu thị.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="928" uniqueCount="697">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="932" uniqueCount="700">
   <si>
     <t>Tên Siêu thị</t>
   </si>
@@ -721,6 +721,9 @@
     <t>KFM_HCM_Q01 - Vinhomes Golden River</t>
   </si>
   <si>
+    <t>KFM_BDU_TAN - 275 D33 KDC Viet Sing</t>
+  </si>
+  <si>
     <t>A101</t>
   </si>
   <si>
@@ -1414,6 +1417,9 @@
     <t>A222</t>
   </si>
   <si>
+    <t>A259</t>
+  </si>
+  <si>
     <t>-4970846623</t>
   </si>
   <si>
@@ -2105,6 +2111,9 @@
   </si>
   <si>
     <t>-1004368025959</t>
+  </si>
+  <si>
+    <t>-1004469485931</t>
   </si>
 </sst>
 </file>
@@ -2436,7 +2445,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D232"/>
+  <dimension ref="A1:D233"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -2458,13 +2467,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D2" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2472,13 +2481,13 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D3" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2486,13 +2495,13 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D4" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2500,13 +2509,13 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C5" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D5" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2514,13 +2523,13 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C6" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D6" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2528,13 +2537,13 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C7" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D7" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2542,13 +2551,13 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C8" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D8" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2556,13 +2565,13 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C9" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D9" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2570,13 +2579,13 @@
         <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D10" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2584,13 +2593,13 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C11" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D11" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2598,13 +2607,13 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C12" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D12" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -2612,13 +2621,13 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C13" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D13" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -2626,13 +2635,13 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C14" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D14" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -2640,13 +2649,13 @@
         <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C15" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D15" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -2654,13 +2663,13 @@
         <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C16" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D16" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -2668,13 +2677,13 @@
         <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C17" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D17" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2682,13 +2691,13 @@
         <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C18" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D18" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -2696,13 +2705,13 @@
         <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C19" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D19" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -2710,13 +2719,13 @@
         <v>22</v>
       </c>
       <c r="B20" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C20" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D20" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -2724,13 +2733,13 @@
         <v>23</v>
       </c>
       <c r="B21" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C21" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D21" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -2738,13 +2747,13 @@
         <v>24</v>
       </c>
       <c r="B22" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C22" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D22" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -2752,13 +2761,13 @@
         <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C23" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D23" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -2766,13 +2775,13 @@
         <v>26</v>
       </c>
       <c r="B24" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C24" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D24" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -2780,13 +2789,13 @@
         <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C25" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D25" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -2794,13 +2803,13 @@
         <v>28</v>
       </c>
       <c r="B26" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C26" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D26" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -2808,13 +2817,13 @@
         <v>29</v>
       </c>
       <c r="B27" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C27" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D27" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -2822,13 +2831,13 @@
         <v>30</v>
       </c>
       <c r="B28" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C28" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D28" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -2836,13 +2845,13 @@
         <v>31</v>
       </c>
       <c r="B29" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C29" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D29" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -2850,13 +2859,13 @@
         <v>32</v>
       </c>
       <c r="B30" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C30" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D30" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -2864,13 +2873,13 @@
         <v>33</v>
       </c>
       <c r="B31" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C31" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D31" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -2878,13 +2887,13 @@
         <v>34</v>
       </c>
       <c r="B32" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C32" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D32" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -2892,13 +2901,13 @@
         <v>35</v>
       </c>
       <c r="B33" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C33" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D33" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -2906,13 +2915,13 @@
         <v>36</v>
       </c>
       <c r="B34" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C34" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D34" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -2920,13 +2929,13 @@
         <v>37</v>
       </c>
       <c r="B35" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C35" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D35" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -2934,13 +2943,13 @@
         <v>38</v>
       </c>
       <c r="B36" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C36" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D36" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -2948,13 +2957,13 @@
         <v>39</v>
       </c>
       <c r="B37" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C37" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D37" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -2962,13 +2971,13 @@
         <v>40</v>
       </c>
       <c r="B38" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C38" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D38" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -2976,13 +2985,13 @@
         <v>41</v>
       </c>
       <c r="B39" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C39" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D39" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -2990,13 +2999,13 @@
         <v>42</v>
       </c>
       <c r="B40" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C40" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D40" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -3004,13 +3013,13 @@
         <v>43</v>
       </c>
       <c r="B41" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C41" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D41" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -3018,13 +3027,13 @@
         <v>44</v>
       </c>
       <c r="B42" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C42" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D42" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -3032,13 +3041,13 @@
         <v>45</v>
       </c>
       <c r="B43" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C43" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D43" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -3046,13 +3055,13 @@
         <v>46</v>
       </c>
       <c r="B44" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C44" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D44" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -3060,13 +3069,13 @@
         <v>47</v>
       </c>
       <c r="B45" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C45" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D45" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -3074,13 +3083,13 @@
         <v>48</v>
       </c>
       <c r="B46" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C46" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D46" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -3088,13 +3097,13 @@
         <v>49</v>
       </c>
       <c r="B47" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C47" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D47" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -3102,13 +3111,13 @@
         <v>50</v>
       </c>
       <c r="B48" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C48" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D48" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -3116,13 +3125,13 @@
         <v>51</v>
       </c>
       <c r="B49" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C49" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D49" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -3130,13 +3139,13 @@
         <v>52</v>
       </c>
       <c r="B50" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C50" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D50" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -3144,13 +3153,13 @@
         <v>53</v>
       </c>
       <c r="B51" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C51" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D51" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -3158,13 +3167,13 @@
         <v>54</v>
       </c>
       <c r="B52" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C52" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D52" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -3172,13 +3181,13 @@
         <v>55</v>
       </c>
       <c r="B53" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C53" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D53" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -3186,13 +3195,13 @@
         <v>56</v>
       </c>
       <c r="B54" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C54" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D54" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -3200,13 +3209,13 @@
         <v>57</v>
       </c>
       <c r="B55" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C55" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D55" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -3214,13 +3223,13 @@
         <v>58</v>
       </c>
       <c r="B56" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C56" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D56" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -3228,13 +3237,13 @@
         <v>59</v>
       </c>
       <c r="B57" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C57" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D57" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -3242,13 +3251,13 @@
         <v>60</v>
       </c>
       <c r="B58" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C58" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D58" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -3256,13 +3265,13 @@
         <v>61</v>
       </c>
       <c r="B59" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C59" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D59" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -3270,13 +3279,13 @@
         <v>62</v>
       </c>
       <c r="B60" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C60" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D60" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -3284,13 +3293,13 @@
         <v>63</v>
       </c>
       <c r="B61" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C61" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D61" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -3298,13 +3307,13 @@
         <v>64</v>
       </c>
       <c r="B62" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C62" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D62" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -3312,13 +3321,13 @@
         <v>65</v>
       </c>
       <c r="B63" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C63" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D63" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -3326,13 +3335,13 @@
         <v>66</v>
       </c>
       <c r="B64" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C64" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D64" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -3340,13 +3349,13 @@
         <v>67</v>
       </c>
       <c r="B65" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C65" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D65" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -3354,13 +3363,13 @@
         <v>68</v>
       </c>
       <c r="B66" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C66" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D66" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -3368,13 +3377,13 @@
         <v>69</v>
       </c>
       <c r="B67" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C67" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D67" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -3382,13 +3391,13 @@
         <v>70</v>
       </c>
       <c r="B68" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C68" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D68" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -3396,13 +3405,13 @@
         <v>71</v>
       </c>
       <c r="B69" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C69" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D69" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -3410,13 +3419,13 @@
         <v>72</v>
       </c>
       <c r="B70" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C70" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D70" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -3424,13 +3433,13 @@
         <v>73</v>
       </c>
       <c r="B71" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C71" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D71" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -3438,13 +3447,13 @@
         <v>74</v>
       </c>
       <c r="B72" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C72" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D72" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -3452,13 +3461,13 @@
         <v>75</v>
       </c>
       <c r="B73" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C73" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D73" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -3466,13 +3475,13 @@
         <v>76</v>
       </c>
       <c r="B74" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C74" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D74" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -3480,13 +3489,13 @@
         <v>77</v>
       </c>
       <c r="B75" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C75" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D75" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -3494,13 +3503,13 @@
         <v>78</v>
       </c>
       <c r="B76" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C76" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D76" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -3508,13 +3517,13 @@
         <v>79</v>
       </c>
       <c r="B77" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C77" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D77" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -3522,13 +3531,13 @@
         <v>80</v>
       </c>
       <c r="B78" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C78" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D78" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -3536,13 +3545,13 @@
         <v>81</v>
       </c>
       <c r="B79" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C79" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D79" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -3550,13 +3559,13 @@
         <v>82</v>
       </c>
       <c r="B80" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C80" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D80" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -3564,13 +3573,13 @@
         <v>83</v>
       </c>
       <c r="B81" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C81" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D81" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
     </row>
     <row r="82" spans="1:4">
@@ -3578,13 +3587,13 @@
         <v>84</v>
       </c>
       <c r="B82" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C82" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D82" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -3592,13 +3601,13 @@
         <v>85</v>
       </c>
       <c r="B83" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C83" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D83" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -3606,13 +3615,13 @@
         <v>86</v>
       </c>
       <c r="B84" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C84" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D84" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -3620,13 +3629,13 @@
         <v>87</v>
       </c>
       <c r="B85" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C85" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D85" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
     </row>
     <row r="86" spans="1:4">
@@ -3634,13 +3643,13 @@
         <v>88</v>
       </c>
       <c r="B86" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C86" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D86" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="87" spans="1:4">
@@ -3648,13 +3657,13 @@
         <v>89</v>
       </c>
       <c r="B87" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C87" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D87" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
     </row>
     <row r="88" spans="1:4">
@@ -3662,13 +3671,13 @@
         <v>90</v>
       </c>
       <c r="B88" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C88" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D88" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -3676,13 +3685,13 @@
         <v>91</v>
       </c>
       <c r="B89" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C89" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D89" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
     </row>
     <row r="90" spans="1:4">
@@ -3690,13 +3699,13 @@
         <v>92</v>
       </c>
       <c r="B90" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C90" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D90" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -3704,13 +3713,13 @@
         <v>93</v>
       </c>
       <c r="B91" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C91" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D91" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
     </row>
     <row r="92" spans="1:4">
@@ -3718,13 +3727,13 @@
         <v>94</v>
       </c>
       <c r="B92" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C92" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D92" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
     </row>
     <row r="93" spans="1:4">
@@ -3732,13 +3741,13 @@
         <v>95</v>
       </c>
       <c r="B93" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C93" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D93" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
     </row>
     <row r="94" spans="1:4">
@@ -3746,13 +3755,13 @@
         <v>96</v>
       </c>
       <c r="B94" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C94" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D94" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
     </row>
     <row r="95" spans="1:4">
@@ -3760,13 +3769,13 @@
         <v>97</v>
       </c>
       <c r="B95" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C95" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D95" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
     </row>
     <row r="96" spans="1:4">
@@ -3774,13 +3783,13 @@
         <v>98</v>
       </c>
       <c r="B96" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C96" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D96" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
     </row>
     <row r="97" spans="1:4">
@@ -3788,13 +3797,13 @@
         <v>99</v>
       </c>
       <c r="B97" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C97" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D97" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
     </row>
     <row r="98" spans="1:4">
@@ -3802,13 +3811,13 @@
         <v>100</v>
       </c>
       <c r="B98" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C98" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D98" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
     </row>
     <row r="99" spans="1:4">
@@ -3816,13 +3825,13 @@
         <v>101</v>
       </c>
       <c r="B99" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C99" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D99" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
     </row>
     <row r="100" spans="1:4">
@@ -3830,13 +3839,13 @@
         <v>102</v>
       </c>
       <c r="B100" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C100" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D100" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
     </row>
     <row r="101" spans="1:4">
@@ -3844,13 +3853,13 @@
         <v>103</v>
       </c>
       <c r="B101" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C101" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D101" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
     </row>
     <row r="102" spans="1:4">
@@ -3858,13 +3867,13 @@
         <v>104</v>
       </c>
       <c r="B102" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C102" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D102" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
     </row>
     <row r="103" spans="1:4">
@@ -3872,13 +3881,13 @@
         <v>105</v>
       </c>
       <c r="B103" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C103" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D103" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
     </row>
     <row r="104" spans="1:4">
@@ -3886,13 +3895,13 @@
         <v>106</v>
       </c>
       <c r="B104" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C104" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D104" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
     </row>
     <row r="105" spans="1:4">
@@ -3900,13 +3909,13 @@
         <v>107</v>
       </c>
       <c r="B105" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C105" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D105" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="106" spans="1:4">
@@ -3914,13 +3923,13 @@
         <v>108</v>
       </c>
       <c r="B106" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C106" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D106" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="107" spans="1:4">
@@ -3928,13 +3937,13 @@
         <v>109</v>
       </c>
       <c r="B107" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C107" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D107" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
     </row>
     <row r="108" spans="1:4">
@@ -3942,13 +3951,13 @@
         <v>110</v>
       </c>
       <c r="B108" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C108" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D108" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
     </row>
     <row r="109" spans="1:4">
@@ -3956,13 +3965,13 @@
         <v>111</v>
       </c>
       <c r="B109" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C109" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D109" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
     </row>
     <row r="110" spans="1:4">
@@ -3970,13 +3979,13 @@
         <v>112</v>
       </c>
       <c r="B110" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C110" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D110" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
     </row>
     <row r="111" spans="1:4">
@@ -3984,13 +3993,13 @@
         <v>113</v>
       </c>
       <c r="B111" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C111" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D111" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
     </row>
     <row r="112" spans="1:4">
@@ -3998,13 +4007,13 @@
         <v>114</v>
       </c>
       <c r="B112" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C112" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D112" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
     </row>
     <row r="113" spans="1:4">
@@ -4012,13 +4021,13 @@
         <v>115</v>
       </c>
       <c r="B113" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C113" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D113" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
     </row>
     <row r="114" spans="1:4">
@@ -4026,13 +4035,13 @@
         <v>116</v>
       </c>
       <c r="B114" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C114" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D114" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
     </row>
     <row r="115" spans="1:4">
@@ -4040,13 +4049,13 @@
         <v>117</v>
       </c>
       <c r="B115" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C115" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D115" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
     <row r="116" spans="1:4">
@@ -4054,13 +4063,13 @@
         <v>118</v>
       </c>
       <c r="B116" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C116" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D116" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
     </row>
     <row r="117" spans="1:4">
@@ -4068,13 +4077,13 @@
         <v>119</v>
       </c>
       <c r="B117" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C117" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D117" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
     </row>
     <row r="118" spans="1:4">
@@ -4082,13 +4091,13 @@
         <v>120</v>
       </c>
       <c r="B118" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C118" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D118" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
     </row>
     <row r="119" spans="1:4">
@@ -4096,13 +4105,13 @@
         <v>121</v>
       </c>
       <c r="B119" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C119" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D119" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
     </row>
     <row r="120" spans="1:4">
@@ -4110,13 +4119,13 @@
         <v>122</v>
       </c>
       <c r="B120" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C120" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D120" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
     </row>
     <row r="121" spans="1:4">
@@ -4124,13 +4133,13 @@
         <v>123</v>
       </c>
       <c r="B121" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C121" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D121" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="122" spans="1:4">
@@ -4138,13 +4147,13 @@
         <v>124</v>
       </c>
       <c r="B122" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C122" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D122" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
     </row>
     <row r="123" spans="1:4">
@@ -4152,13 +4161,13 @@
         <v>125</v>
       </c>
       <c r="B123" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C123" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D123" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
     </row>
     <row r="124" spans="1:4">
@@ -4166,13 +4175,13 @@
         <v>126</v>
       </c>
       <c r="B124" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C124" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D124" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
     </row>
     <row r="125" spans="1:4">
@@ -4180,13 +4189,13 @@
         <v>127</v>
       </c>
       <c r="B125" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C125" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D125" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
     </row>
     <row r="126" spans="1:4">
@@ -4194,13 +4203,13 @@
         <v>128</v>
       </c>
       <c r="B126" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C126" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D126" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
     </row>
     <row r="127" spans="1:4">
@@ -4208,13 +4217,13 @@
         <v>129</v>
       </c>
       <c r="B127" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C127" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D127" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
     </row>
     <row r="128" spans="1:4">
@@ -4222,13 +4231,13 @@
         <v>130</v>
       </c>
       <c r="B128" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C128" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D128" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
     </row>
     <row r="129" spans="1:4">
@@ -4236,13 +4245,13 @@
         <v>131</v>
       </c>
       <c r="B129" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C129" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D129" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
     </row>
     <row r="130" spans="1:4">
@@ -4250,13 +4259,13 @@
         <v>132</v>
       </c>
       <c r="B130" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C130" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D130" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
     </row>
     <row r="131" spans="1:4">
@@ -4264,13 +4273,13 @@
         <v>133</v>
       </c>
       <c r="B131" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C131" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D131" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="132" spans="1:4">
@@ -4278,13 +4287,13 @@
         <v>134</v>
       </c>
       <c r="B132" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C132" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D132" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
     </row>
     <row r="133" spans="1:4">
@@ -4292,13 +4301,13 @@
         <v>135</v>
       </c>
       <c r="B133" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C133" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D133" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
     </row>
     <row r="134" spans="1:4">
@@ -4306,13 +4315,13 @@
         <v>136</v>
       </c>
       <c r="B134" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C134" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D134" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
     </row>
     <row r="135" spans="1:4">
@@ -4320,13 +4329,13 @@
         <v>137</v>
       </c>
       <c r="B135" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C135" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D135" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
     </row>
     <row r="136" spans="1:4">
@@ -4334,13 +4343,13 @@
         <v>138</v>
       </c>
       <c r="B136" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C136" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D136" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
     </row>
     <row r="137" spans="1:4">
@@ -4348,13 +4357,13 @@
         <v>139</v>
       </c>
       <c r="B137" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C137" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D137" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
     </row>
     <row r="138" spans="1:4">
@@ -4362,13 +4371,13 @@
         <v>140</v>
       </c>
       <c r="B138" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C138" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D138" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
     </row>
     <row r="139" spans="1:4">
@@ -4376,13 +4385,13 @@
         <v>141</v>
       </c>
       <c r="B139" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C139" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D139" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
     </row>
     <row r="140" spans="1:4">
@@ -4390,13 +4399,13 @@
         <v>142</v>
       </c>
       <c r="B140" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C140" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D140" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
     </row>
     <row r="141" spans="1:4">
@@ -4404,13 +4413,13 @@
         <v>143</v>
       </c>
       <c r="B141" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C141" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D141" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
     </row>
     <row r="142" spans="1:4">
@@ -4418,13 +4427,13 @@
         <v>144</v>
       </c>
       <c r="B142" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C142" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D142" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
     </row>
     <row r="143" spans="1:4">
@@ -4432,13 +4441,13 @@
         <v>145</v>
       </c>
       <c r="B143" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C143" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D143" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
     </row>
     <row r="144" spans="1:4">
@@ -4446,13 +4455,13 @@
         <v>146</v>
       </c>
       <c r="B144" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C144" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D144" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
     </row>
     <row r="145" spans="1:4">
@@ -4460,13 +4469,13 @@
         <v>147</v>
       </c>
       <c r="B145" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C145" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D145" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
     </row>
     <row r="146" spans="1:4">
@@ -4474,13 +4483,13 @@
         <v>148</v>
       </c>
       <c r="B146" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C146" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D146" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
     </row>
     <row r="147" spans="1:4">
@@ -4488,13 +4497,13 @@
         <v>149</v>
       </c>
       <c r="B147" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C147" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D147" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
     </row>
     <row r="148" spans="1:4">
@@ -4502,13 +4511,13 @@
         <v>150</v>
       </c>
       <c r="B148" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C148" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D148" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
     </row>
     <row r="149" spans="1:4">
@@ -4516,13 +4525,13 @@
         <v>151</v>
       </c>
       <c r="B149" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C149" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D149" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
     </row>
     <row r="150" spans="1:4">
@@ -4530,13 +4539,13 @@
         <v>152</v>
       </c>
       <c r="B150" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C150" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D150" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
     </row>
     <row r="151" spans="1:4">
@@ -4544,13 +4553,13 @@
         <v>153</v>
       </c>
       <c r="B151" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C151" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="D151" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
     </row>
     <row r="152" spans="1:4">
@@ -4558,13 +4567,13 @@
         <v>154</v>
       </c>
       <c r="B152" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C152" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D152" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
     </row>
     <row r="153" spans="1:4">
@@ -4572,13 +4581,13 @@
         <v>155</v>
       </c>
       <c r="B153" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C153" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="D153" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
     </row>
     <row r="154" spans="1:4">
@@ -4586,13 +4595,13 @@
         <v>156</v>
       </c>
       <c r="B154" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C154" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D154" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
     </row>
     <row r="155" spans="1:4">
@@ -4600,13 +4609,13 @@
         <v>157</v>
       </c>
       <c r="B155" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C155" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D155" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
     </row>
     <row r="156" spans="1:4">
@@ -4614,13 +4623,13 @@
         <v>158</v>
       </c>
       <c r="B156" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C156" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D156" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
     </row>
     <row r="157" spans="1:4">
@@ -4628,13 +4637,13 @@
         <v>159</v>
       </c>
       <c r="B157" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C157" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D157" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
     </row>
     <row r="158" spans="1:4">
@@ -4642,13 +4651,13 @@
         <v>160</v>
       </c>
       <c r="B158" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C158" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D158" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
     </row>
     <row r="159" spans="1:4">
@@ -4656,13 +4665,13 @@
         <v>161</v>
       </c>
       <c r="B159" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C159" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D159" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
     </row>
     <row r="160" spans="1:4">
@@ -4670,13 +4679,13 @@
         <v>162</v>
       </c>
       <c r="B160" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C160" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D160" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
     </row>
     <row r="161" spans="1:4">
@@ -4684,13 +4693,13 @@
         <v>163</v>
       </c>
       <c r="B161" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C161" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="D161" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
     </row>
     <row r="162" spans="1:4">
@@ -4698,13 +4707,13 @@
         <v>164</v>
       </c>
       <c r="B162" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C162" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D162" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
     </row>
     <row r="163" spans="1:4">
@@ -4712,13 +4721,13 @@
         <v>165</v>
       </c>
       <c r="B163" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C163" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D163" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
     </row>
     <row r="164" spans="1:4">
@@ -4726,13 +4735,13 @@
         <v>166</v>
       </c>
       <c r="B164" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C164" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="D164" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
     </row>
     <row r="165" spans="1:4">
@@ -4740,13 +4749,13 @@
         <v>167</v>
       </c>
       <c r="B165" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C165" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D165" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
     </row>
     <row r="166" spans="1:4">
@@ -4754,13 +4763,13 @@
         <v>168</v>
       </c>
       <c r="B166" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C166" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D166" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
     </row>
     <row r="167" spans="1:4">
@@ -4768,13 +4777,13 @@
         <v>169</v>
       </c>
       <c r="B167" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C167" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D167" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
     </row>
     <row r="168" spans="1:4">
@@ -4782,13 +4791,13 @@
         <v>170</v>
       </c>
       <c r="B168" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C168" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D168" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
     </row>
     <row r="169" spans="1:4">
@@ -4796,13 +4805,13 @@
         <v>171</v>
       </c>
       <c r="B169" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C169" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="D169" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
     </row>
     <row r="170" spans="1:4">
@@ -4810,13 +4819,13 @@
         <v>172</v>
       </c>
       <c r="B170" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C170" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D170" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
     </row>
     <row r="171" spans="1:4">
@@ -4824,13 +4833,13 @@
         <v>173</v>
       </c>
       <c r="B171" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C171" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D171" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
     </row>
     <row r="172" spans="1:4">
@@ -4838,13 +4847,13 @@
         <v>174</v>
       </c>
       <c r="B172" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C172" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D172" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
     </row>
     <row r="173" spans="1:4">
@@ -4852,13 +4861,13 @@
         <v>175</v>
       </c>
       <c r="B173" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C173" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D173" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
     </row>
     <row r="174" spans="1:4">
@@ -4866,13 +4875,13 @@
         <v>176</v>
       </c>
       <c r="B174" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C174" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D174" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
     </row>
     <row r="175" spans="1:4">
@@ -4880,13 +4889,13 @@
         <v>177</v>
       </c>
       <c r="B175" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C175" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="D175" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
     </row>
     <row r="176" spans="1:4">
@@ -4894,13 +4903,13 @@
         <v>178</v>
       </c>
       <c r="B176" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C176" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D176" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
     </row>
     <row r="177" spans="1:4">
@@ -4908,13 +4917,13 @@
         <v>179</v>
       </c>
       <c r="B177" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C177" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D177" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
     </row>
     <row r="178" spans="1:4">
@@ -4922,13 +4931,13 @@
         <v>180</v>
       </c>
       <c r="B178" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C178" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D178" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
     </row>
     <row r="179" spans="1:4">
@@ -4936,13 +4945,13 @@
         <v>181</v>
       </c>
       <c r="B179" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C179" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D179" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
     </row>
     <row r="180" spans="1:4">
@@ -4950,13 +4959,13 @@
         <v>182</v>
       </c>
       <c r="B180" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C180" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D180" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
     </row>
     <row r="181" spans="1:4">
@@ -4964,13 +4973,13 @@
         <v>183</v>
       </c>
       <c r="B181" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C181" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="D181" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
     </row>
     <row r="182" spans="1:4">
@@ -4978,13 +4987,13 @@
         <v>184</v>
       </c>
       <c r="B182" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C182" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D182" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
     </row>
     <row r="183" spans="1:4">
@@ -4992,13 +5001,13 @@
         <v>185</v>
       </c>
       <c r="B183" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C183" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D183" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
     </row>
     <row r="184" spans="1:4">
@@ -5006,13 +5015,13 @@
         <v>186</v>
       </c>
       <c r="B184" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C184" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D184" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
     </row>
     <row r="185" spans="1:4">
@@ -5020,13 +5029,13 @@
         <v>187</v>
       </c>
       <c r="B185" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C185" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D185" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
     </row>
     <row r="186" spans="1:4">
@@ -5034,13 +5043,13 @@
         <v>188</v>
       </c>
       <c r="B186" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C186" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D186" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
     </row>
     <row r="187" spans="1:4">
@@ -5048,13 +5057,13 @@
         <v>189</v>
       </c>
       <c r="B187" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C187" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D187" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
     </row>
     <row r="188" spans="1:4">
@@ -5062,13 +5071,13 @@
         <v>190</v>
       </c>
       <c r="B188" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C188" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D188" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
     </row>
     <row r="189" spans="1:4">
@@ -5076,13 +5085,13 @@
         <v>191</v>
       </c>
       <c r="B189" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C189" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D189" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
     </row>
     <row r="190" spans="1:4">
@@ -5090,13 +5099,13 @@
         <v>192</v>
       </c>
       <c r="B190" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C190" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D190" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
     </row>
     <row r="191" spans="1:4">
@@ -5104,13 +5113,13 @@
         <v>193</v>
       </c>
       <c r="B191" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C191" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D191" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
     </row>
     <row r="192" spans="1:4">
@@ -5118,13 +5127,13 @@
         <v>194</v>
       </c>
       <c r="B192" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C192" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D192" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
     </row>
     <row r="193" spans="1:4">
@@ -5132,13 +5141,13 @@
         <v>195</v>
       </c>
       <c r="B193" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C193" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="D193" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
     </row>
     <row r="194" spans="1:4">
@@ -5146,13 +5155,13 @@
         <v>196</v>
       </c>
       <c r="B194" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C194" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D194" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
     </row>
     <row r="195" spans="1:4">
@@ -5160,13 +5169,13 @@
         <v>197</v>
       </c>
       <c r="B195" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C195" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="D195" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
     </row>
     <row r="196" spans="1:4">
@@ -5174,13 +5183,13 @@
         <v>198</v>
       </c>
       <c r="B196" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C196" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="D196" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
     </row>
     <row r="197" spans="1:4">
@@ -5188,13 +5197,13 @@
         <v>199</v>
       </c>
       <c r="B197" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C197" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="D197" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
     </row>
     <row r="198" spans="1:4">
@@ -5202,13 +5211,13 @@
         <v>200</v>
       </c>
       <c r="B198" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C198" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="D198" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
     </row>
     <row r="199" spans="1:4">
@@ -5216,13 +5225,13 @@
         <v>201</v>
       </c>
       <c r="B199" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C199" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="D199" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
     </row>
     <row r="200" spans="1:4">
@@ -5230,13 +5239,13 @@
         <v>202</v>
       </c>
       <c r="B200" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C200" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="D200" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
     </row>
     <row r="201" spans="1:4">
@@ -5244,13 +5253,13 @@
         <v>203</v>
       </c>
       <c r="B201" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C201" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="D201" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
     </row>
     <row r="202" spans="1:4">
@@ -5258,13 +5267,13 @@
         <v>204</v>
       </c>
       <c r="B202" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C202" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="D202" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
     </row>
     <row r="203" spans="1:4">
@@ -5272,13 +5281,13 @@
         <v>205</v>
       </c>
       <c r="B203" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C203" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="D203" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
     </row>
     <row r="204" spans="1:4">
@@ -5286,13 +5295,13 @@
         <v>206</v>
       </c>
       <c r="B204" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C204" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D204" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
     </row>
     <row r="205" spans="1:4">
@@ -5300,13 +5309,13 @@
         <v>207</v>
       </c>
       <c r="B205" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C205" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D205" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
     </row>
     <row r="206" spans="1:4">
@@ -5314,13 +5323,13 @@
         <v>208</v>
       </c>
       <c r="B206" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C206" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="D206" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
     </row>
     <row r="207" spans="1:4">
@@ -5328,13 +5337,13 @@
         <v>209</v>
       </c>
       <c r="B207" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C207" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D207" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
     </row>
     <row r="208" spans="1:4">
@@ -5342,13 +5351,13 @@
         <v>210</v>
       </c>
       <c r="B208" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C208" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D208" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
     </row>
     <row r="209" spans="1:4">
@@ -5356,13 +5365,13 @@
         <v>211</v>
       </c>
       <c r="B209" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C209" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D209" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
     </row>
     <row r="210" spans="1:4">
@@ -5370,13 +5379,13 @@
         <v>212</v>
       </c>
       <c r="B210" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C210" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="D210" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
     </row>
     <row r="211" spans="1:4">
@@ -5384,13 +5393,13 @@
         <v>213</v>
       </c>
       <c r="B211" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C211" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D211" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
     </row>
     <row r="212" spans="1:4">
@@ -5398,13 +5407,13 @@
         <v>214</v>
       </c>
       <c r="B212" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C212" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D212" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
     </row>
     <row r="213" spans="1:4">
@@ -5412,13 +5421,13 @@
         <v>215</v>
       </c>
       <c r="B213" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C213" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D213" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
     </row>
     <row r="214" spans="1:4">
@@ -5426,13 +5435,13 @@
         <v>216</v>
       </c>
       <c r="B214" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C214" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D214" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
     </row>
     <row r="215" spans="1:4">
@@ -5440,13 +5449,13 @@
         <v>217</v>
       </c>
       <c r="B215" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C215" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D215" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
     </row>
     <row r="216" spans="1:4">
@@ -5454,13 +5463,13 @@
         <v>218</v>
       </c>
       <c r="B216" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C216" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D216" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
     </row>
     <row r="217" spans="1:4">
@@ -5468,13 +5477,13 @@
         <v>219</v>
       </c>
       <c r="B217" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C217" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D217" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
     </row>
     <row r="218" spans="1:4">
@@ -5482,13 +5491,13 @@
         <v>220</v>
       </c>
       <c r="B218" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C218" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D218" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
     </row>
     <row r="219" spans="1:4">
@@ -5496,13 +5505,13 @@
         <v>221</v>
       </c>
       <c r="B219" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C219" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D219" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
     </row>
     <row r="220" spans="1:4">
@@ -5510,13 +5519,13 @@
         <v>222</v>
       </c>
       <c r="B220" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C220" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D220" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
     </row>
     <row r="221" spans="1:4">
@@ -5524,13 +5533,13 @@
         <v>223</v>
       </c>
       <c r="B221" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="C221" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D221" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
     </row>
     <row r="222" spans="1:4">
@@ -5538,13 +5547,13 @@
         <v>224</v>
       </c>
       <c r="B222" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C222" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="D222" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
     </row>
     <row r="223" spans="1:4">
@@ -5552,13 +5561,13 @@
         <v>225</v>
       </c>
       <c r="B223" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C223" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="D223" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
     </row>
     <row r="224" spans="1:4">
@@ -5566,13 +5575,13 @@
         <v>226</v>
       </c>
       <c r="B224" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C224" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D224" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
     </row>
     <row r="225" spans="1:4">
@@ -5580,13 +5589,13 @@
         <v>227</v>
       </c>
       <c r="B225" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C225" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="D225" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
     </row>
     <row r="226" spans="1:4">
@@ -5594,13 +5603,13 @@
         <v>228</v>
       </c>
       <c r="B226" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C226" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D226" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
     </row>
     <row r="227" spans="1:4">
@@ -5608,13 +5617,13 @@
         <v>229</v>
       </c>
       <c r="B227" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C227" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D227" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
     </row>
     <row r="228" spans="1:4">
@@ -5622,13 +5631,13 @@
         <v>230</v>
       </c>
       <c r="B228" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C228" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="D228" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
     </row>
     <row r="229" spans="1:4">
@@ -5636,13 +5645,13 @@
         <v>231</v>
       </c>
       <c r="B229" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C229" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D229" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
     </row>
     <row r="230" spans="1:4">
@@ -5650,13 +5659,13 @@
         <v>232</v>
       </c>
       <c r="B230" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C230" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="D230" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
     </row>
     <row r="231" spans="1:4">
@@ -5664,13 +5673,13 @@
         <v>233</v>
       </c>
       <c r="B231" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C231" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D231" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
     </row>
     <row r="232" spans="1:4">
@@ -5678,13 +5687,27 @@
         <v>234</v>
       </c>
       <c r="B232" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="C232" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="D232" t="s">
-        <v>696</v>
+        <v>698</v>
+      </c>
+    </row>
+    <row r="233" spans="1:4">
+      <c r="A233" t="s">
+        <v>235</v>
+      </c>
+      <c r="B233" t="s">
+        <v>467</v>
+      </c>
+      <c r="C233" t="s">
+        <v>467</v>
+      </c>
+      <c r="D233" t="s">
+        <v>699</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cập nhật Tool Hậu Kiểm Kho Khô hỗ trợ lọc phiếu Còn hậu kiểm cho CKO và siêu thị chỉ định
</commit_message>
<xml_diff>
--- a/SPAM_PHIEU_CHUYEN/CHI TIẾT MÁT/Danh sách Siêu thị.xlsx
+++ b/SPAM_PHIEU_CHUYEN/CHI TIẾT MÁT/Danh sách Siêu thị.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="944" uniqueCount="707">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="948" uniqueCount="710">
   <si>
     <t>Tên Siêu thị</t>
   </si>
@@ -733,6 +733,9 @@
     <t>KFM_HNI_YHO - CT3 Yên Hoà Park View</t>
   </si>
   <si>
+    <t>KFM_HCM_PNH - Hoa Sứ</t>
+  </si>
+  <si>
     <t>A101</t>
   </si>
   <si>
@@ -1432,6 +1435,9 @@
     <t>B001</t>
   </si>
   <si>
+    <t>A266</t>
+  </si>
+  <si>
     <t>-4970846623</t>
   </si>
   <si>
@@ -2135,6 +2141,9 @@
   </si>
   <si>
     <t>-1004305022913</t>
+  </si>
+  <si>
+    <t>-1004376355185</t>
   </si>
 </sst>
 </file>
@@ -2466,7 +2475,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D236"/>
+  <dimension ref="A1:D237"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -2488,13 +2497,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D2" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2502,13 +2511,13 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D3" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2516,13 +2525,13 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D4" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2530,13 +2539,13 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D5" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2544,13 +2553,13 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D6" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2558,13 +2567,13 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C7" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D7" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2572,13 +2581,13 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C8" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D8" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2586,13 +2595,13 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C9" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D9" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2600,13 +2609,13 @@
         <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C10" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D10" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2614,13 +2623,13 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C11" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D11" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2628,13 +2637,13 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C12" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D12" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -2642,13 +2651,13 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C13" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D13" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -2656,13 +2665,13 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D14" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -2670,13 +2679,13 @@
         <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C15" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D15" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -2684,13 +2693,13 @@
         <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C16" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D16" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -2698,13 +2707,13 @@
         <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C17" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D17" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2712,13 +2721,13 @@
         <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C18" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D18" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -2726,13 +2735,13 @@
         <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C19" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D19" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -2740,13 +2749,13 @@
         <v>22</v>
       </c>
       <c r="B20" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C20" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D20" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -2754,13 +2763,13 @@
         <v>23</v>
       </c>
       <c r="B21" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C21" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D21" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -2768,13 +2777,13 @@
         <v>24</v>
       </c>
       <c r="B22" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C22" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D22" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -2782,13 +2791,13 @@
         <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C23" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D23" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -2796,13 +2805,13 @@
         <v>26</v>
       </c>
       <c r="B24" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C24" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D24" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -2810,13 +2819,13 @@
         <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C25" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D25" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -2824,13 +2833,13 @@
         <v>28</v>
       </c>
       <c r="B26" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C26" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D26" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -2838,13 +2847,13 @@
         <v>29</v>
       </c>
       <c r="B27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D27" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -2852,13 +2861,13 @@
         <v>30</v>
       </c>
       <c r="B28" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C28" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D28" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -2866,13 +2875,13 @@
         <v>31</v>
       </c>
       <c r="B29" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C29" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D29" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -2880,13 +2889,13 @@
         <v>32</v>
       </c>
       <c r="B30" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C30" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D30" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -2894,13 +2903,13 @@
         <v>33</v>
       </c>
       <c r="B31" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C31" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D31" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -2908,13 +2917,13 @@
         <v>34</v>
       </c>
       <c r="B32" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C32" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D32" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -2922,13 +2931,13 @@
         <v>35</v>
       </c>
       <c r="B33" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C33" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D33" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -2936,13 +2945,13 @@
         <v>36</v>
       </c>
       <c r="B34" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C34" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D34" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -2950,13 +2959,13 @@
         <v>37</v>
       </c>
       <c r="B35" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C35" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D35" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -2964,13 +2973,13 @@
         <v>38</v>
       </c>
       <c r="B36" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C36" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D36" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -2978,13 +2987,13 @@
         <v>39</v>
       </c>
       <c r="B37" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C37" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D37" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -2992,13 +3001,13 @@
         <v>40</v>
       </c>
       <c r="B38" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C38" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D38" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -3006,13 +3015,13 @@
         <v>41</v>
       </c>
       <c r="B39" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C39" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D39" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -3020,13 +3029,13 @@
         <v>42</v>
       </c>
       <c r="B40" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C40" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D40" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -3034,13 +3043,13 @@
         <v>43</v>
       </c>
       <c r="B41" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C41" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D41" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -3048,13 +3057,13 @@
         <v>44</v>
       </c>
       <c r="B42" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C42" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D42" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -3062,13 +3071,13 @@
         <v>45</v>
       </c>
       <c r="B43" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C43" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D43" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -3076,13 +3085,13 @@
         <v>46</v>
       </c>
       <c r="B44" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C44" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D44" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -3090,13 +3099,13 @@
         <v>47</v>
       </c>
       <c r="B45" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C45" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D45" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -3104,13 +3113,13 @@
         <v>48</v>
       </c>
       <c r="B46" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C46" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D46" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -3118,13 +3127,13 @@
         <v>49</v>
       </c>
       <c r="B47" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C47" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D47" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -3132,13 +3141,13 @@
         <v>50</v>
       </c>
       <c r="B48" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C48" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D48" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -3146,13 +3155,13 @@
         <v>51</v>
       </c>
       <c r="B49" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C49" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D49" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -3160,13 +3169,13 @@
         <v>52</v>
       </c>
       <c r="B50" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C50" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D50" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -3174,13 +3183,13 @@
         <v>53</v>
       </c>
       <c r="B51" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C51" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D51" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -3188,13 +3197,13 @@
         <v>54</v>
       </c>
       <c r="B52" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C52" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D52" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -3202,13 +3211,13 @@
         <v>55</v>
       </c>
       <c r="B53" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C53" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D53" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -3216,13 +3225,13 @@
         <v>56</v>
       </c>
       <c r="B54" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C54" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D54" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -3230,13 +3239,13 @@
         <v>57</v>
       </c>
       <c r="B55" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C55" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D55" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -3244,13 +3253,13 @@
         <v>58</v>
       </c>
       <c r="B56" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C56" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D56" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -3258,13 +3267,13 @@
         <v>59</v>
       </c>
       <c r="B57" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C57" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D57" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -3272,13 +3281,13 @@
         <v>60</v>
       </c>
       <c r="B58" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C58" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D58" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -3286,13 +3295,13 @@
         <v>61</v>
       </c>
       <c r="B59" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C59" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D59" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -3300,13 +3309,13 @@
         <v>62</v>
       </c>
       <c r="B60" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C60" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D60" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -3314,13 +3323,13 @@
         <v>63</v>
       </c>
       <c r="B61" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C61" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D61" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -3328,13 +3337,13 @@
         <v>64</v>
       </c>
       <c r="B62" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C62" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D62" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -3342,13 +3351,13 @@
         <v>65</v>
       </c>
       <c r="B63" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C63" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D63" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -3356,13 +3365,13 @@
         <v>66</v>
       </c>
       <c r="B64" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C64" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D64" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -3370,13 +3379,13 @@
         <v>67</v>
       </c>
       <c r="B65" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C65" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D65" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -3384,13 +3393,13 @@
         <v>68</v>
       </c>
       <c r="B66" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C66" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D66" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -3398,13 +3407,13 @@
         <v>69</v>
       </c>
       <c r="B67" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C67" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D67" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -3412,13 +3421,13 @@
         <v>70</v>
       </c>
       <c r="B68" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C68" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D68" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -3426,13 +3435,13 @@
         <v>71</v>
       </c>
       <c r="B69" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C69" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D69" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -3440,13 +3449,13 @@
         <v>72</v>
       </c>
       <c r="B70" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C70" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D70" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -3454,13 +3463,13 @@
         <v>73</v>
       </c>
       <c r="B71" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C71" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D71" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -3468,13 +3477,13 @@
         <v>74</v>
       </c>
       <c r="B72" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C72" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D72" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -3482,13 +3491,13 @@
         <v>75</v>
       </c>
       <c r="B73" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C73" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D73" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -3496,13 +3505,13 @@
         <v>76</v>
       </c>
       <c r="B74" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C74" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D74" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -3510,13 +3519,13 @@
         <v>77</v>
       </c>
       <c r="B75" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C75" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D75" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -3524,13 +3533,13 @@
         <v>78</v>
       </c>
       <c r="B76" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C76" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D76" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -3538,13 +3547,13 @@
         <v>79</v>
       </c>
       <c r="B77" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C77" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D77" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -3552,13 +3561,13 @@
         <v>80</v>
       </c>
       <c r="B78" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C78" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D78" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -3566,13 +3575,13 @@
         <v>81</v>
       </c>
       <c r="B79" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C79" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D79" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -3580,13 +3589,13 @@
         <v>82</v>
       </c>
       <c r="B80" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C80" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D80" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -3594,13 +3603,13 @@
         <v>83</v>
       </c>
       <c r="B81" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C81" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D81" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
     </row>
     <row r="82" spans="1:4">
@@ -3608,13 +3617,13 @@
         <v>84</v>
       </c>
       <c r="B82" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C82" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D82" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -3622,13 +3631,13 @@
         <v>85</v>
       </c>
       <c r="B83" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C83" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D83" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -3636,13 +3645,13 @@
         <v>86</v>
       </c>
       <c r="B84" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C84" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D84" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -3650,13 +3659,13 @@
         <v>87</v>
       </c>
       <c r="B85" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C85" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D85" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
     </row>
     <row r="86" spans="1:4">
@@ -3664,13 +3673,13 @@
         <v>88</v>
       </c>
       <c r="B86" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C86" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D86" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
     </row>
     <row r="87" spans="1:4">
@@ -3678,13 +3687,13 @@
         <v>89</v>
       </c>
       <c r="B87" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C87" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D87" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
     </row>
     <row r="88" spans="1:4">
@@ -3692,13 +3701,13 @@
         <v>90</v>
       </c>
       <c r="B88" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C88" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D88" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -3706,13 +3715,13 @@
         <v>91</v>
       </c>
       <c r="B89" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C89" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D89" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
     </row>
     <row r="90" spans="1:4">
@@ -3720,13 +3729,13 @@
         <v>92</v>
       </c>
       <c r="B90" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C90" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D90" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -3734,13 +3743,13 @@
         <v>93</v>
       </c>
       <c r="B91" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C91" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D91" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
     </row>
     <row r="92" spans="1:4">
@@ -3748,13 +3757,13 @@
         <v>94</v>
       </c>
       <c r="B92" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C92" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D92" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
     </row>
     <row r="93" spans="1:4">
@@ -3762,13 +3771,13 @@
         <v>95</v>
       </c>
       <c r="B93" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C93" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D93" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
     </row>
     <row r="94" spans="1:4">
@@ -3776,13 +3785,13 @@
         <v>96</v>
       </c>
       <c r="B94" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C94" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D94" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
     </row>
     <row r="95" spans="1:4">
@@ -3790,13 +3799,13 @@
         <v>97</v>
       </c>
       <c r="B95" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C95" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D95" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
     </row>
     <row r="96" spans="1:4">
@@ -3804,13 +3813,13 @@
         <v>98</v>
       </c>
       <c r="B96" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C96" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D96" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
     </row>
     <row r="97" spans="1:4">
@@ -3818,13 +3827,13 @@
         <v>99</v>
       </c>
       <c r="B97" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C97" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D97" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
     </row>
     <row r="98" spans="1:4">
@@ -3832,13 +3841,13 @@
         <v>100</v>
       </c>
       <c r="B98" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C98" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D98" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
     </row>
     <row r="99" spans="1:4">
@@ -3846,13 +3855,13 @@
         <v>101</v>
       </c>
       <c r="B99" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C99" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D99" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="100" spans="1:4">
@@ -3860,13 +3869,13 @@
         <v>102</v>
       </c>
       <c r="B100" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C100" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D100" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="101" spans="1:4">
@@ -3874,13 +3883,13 @@
         <v>103</v>
       </c>
       <c r="B101" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C101" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D101" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
     </row>
     <row r="102" spans="1:4">
@@ -3888,13 +3897,13 @@
         <v>104</v>
       </c>
       <c r="B102" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C102" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D102" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
     </row>
     <row r="103" spans="1:4">
@@ -3902,13 +3911,13 @@
         <v>105</v>
       </c>
       <c r="B103" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C103" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D103" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
     </row>
     <row r="104" spans="1:4">
@@ -3916,13 +3925,13 @@
         <v>106</v>
       </c>
       <c r="B104" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C104" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D104" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
     </row>
     <row r="105" spans="1:4">
@@ -3930,13 +3939,13 @@
         <v>107</v>
       </c>
       <c r="B105" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C105" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D105" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
     </row>
     <row r="106" spans="1:4">
@@ -3944,13 +3953,13 @@
         <v>108</v>
       </c>
       <c r="B106" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C106" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D106" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
     </row>
     <row r="107" spans="1:4">
@@ -3958,13 +3967,13 @@
         <v>109</v>
       </c>
       <c r="B107" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C107" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D107" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
     </row>
     <row r="108" spans="1:4">
@@ -3972,13 +3981,13 @@
         <v>110</v>
       </c>
       <c r="B108" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C108" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D108" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
     </row>
     <row r="109" spans="1:4">
@@ -3986,13 +3995,13 @@
         <v>111</v>
       </c>
       <c r="B109" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C109" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D109" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
     <row r="110" spans="1:4">
@@ -4000,13 +4009,13 @@
         <v>112</v>
       </c>
       <c r="B110" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C110" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D110" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
     </row>
     <row r="111" spans="1:4">
@@ -4014,13 +4023,13 @@
         <v>113</v>
       </c>
       <c r="B111" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C111" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D111" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
     </row>
     <row r="112" spans="1:4">
@@ -4028,13 +4037,13 @@
         <v>114</v>
       </c>
       <c r="B112" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C112" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D112" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
     </row>
     <row r="113" spans="1:4">
@@ -4042,13 +4051,13 @@
         <v>115</v>
       </c>
       <c r="B113" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C113" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D113" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
     </row>
     <row r="114" spans="1:4">
@@ -4056,13 +4065,13 @@
         <v>116</v>
       </c>
       <c r="B114" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C114" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D114" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
     </row>
     <row r="115" spans="1:4">
@@ -4070,13 +4079,13 @@
         <v>117</v>
       </c>
       <c r="B115" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C115" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D115" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="116" spans="1:4">
@@ -4084,13 +4093,13 @@
         <v>118</v>
       </c>
       <c r="B116" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C116" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D116" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
     </row>
     <row r="117" spans="1:4">
@@ -4098,13 +4107,13 @@
         <v>119</v>
       </c>
       <c r="B117" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C117" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D117" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
     </row>
     <row r="118" spans="1:4">
@@ -4112,13 +4121,13 @@
         <v>120</v>
       </c>
       <c r="B118" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C118" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D118" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
     </row>
     <row r="119" spans="1:4">
@@ -4126,13 +4135,13 @@
         <v>121</v>
       </c>
       <c r="B119" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C119" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D119" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
     </row>
     <row r="120" spans="1:4">
@@ -4140,13 +4149,13 @@
         <v>122</v>
       </c>
       <c r="B120" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C120" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D120" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
     </row>
     <row r="121" spans="1:4">
@@ -4154,13 +4163,13 @@
         <v>123</v>
       </c>
       <c r="B121" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C121" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D121" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
     </row>
     <row r="122" spans="1:4">
@@ -4168,13 +4177,13 @@
         <v>124</v>
       </c>
       <c r="B122" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C122" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D122" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
     </row>
     <row r="123" spans="1:4">
@@ -4182,13 +4191,13 @@
         <v>125</v>
       </c>
       <c r="B123" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C123" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D123" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
     </row>
     <row r="124" spans="1:4">
@@ -4196,13 +4205,13 @@
         <v>126</v>
       </c>
       <c r="B124" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C124" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D124" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
     </row>
     <row r="125" spans="1:4">
@@ -4210,13 +4219,13 @@
         <v>127</v>
       </c>
       <c r="B125" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C125" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D125" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="126" spans="1:4">
@@ -4224,13 +4233,13 @@
         <v>128</v>
       </c>
       <c r="B126" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C126" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D126" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
     </row>
     <row r="127" spans="1:4">
@@ -4238,13 +4247,13 @@
         <v>129</v>
       </c>
       <c r="B127" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C127" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D127" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
     </row>
     <row r="128" spans="1:4">
@@ -4252,13 +4261,13 @@
         <v>130</v>
       </c>
       <c r="B128" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C128" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D128" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
     </row>
     <row r="129" spans="1:4">
@@ -4266,13 +4275,13 @@
         <v>131</v>
       </c>
       <c r="B129" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C129" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D129" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
     </row>
     <row r="130" spans="1:4">
@@ -4280,13 +4289,13 @@
         <v>132</v>
       </c>
       <c r="B130" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C130" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D130" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
     </row>
     <row r="131" spans="1:4">
@@ -4294,13 +4303,13 @@
         <v>133</v>
       </c>
       <c r="B131" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C131" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D131" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
     </row>
     <row r="132" spans="1:4">
@@ -4308,13 +4317,13 @@
         <v>134</v>
       </c>
       <c r="B132" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C132" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D132" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
     </row>
     <row r="133" spans="1:4">
@@ -4322,13 +4331,13 @@
         <v>135</v>
       </c>
       <c r="B133" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C133" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D133" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
     </row>
     <row r="134" spans="1:4">
@@ -4336,13 +4345,13 @@
         <v>136</v>
       </c>
       <c r="B134" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C134" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D134" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
     </row>
     <row r="135" spans="1:4">
@@ -4350,13 +4359,13 @@
         <v>137</v>
       </c>
       <c r="B135" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C135" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D135" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
     </row>
     <row r="136" spans="1:4">
@@ -4364,13 +4373,13 @@
         <v>138</v>
       </c>
       <c r="B136" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C136" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D136" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
     </row>
     <row r="137" spans="1:4">
@@ -4378,13 +4387,13 @@
         <v>139</v>
       </c>
       <c r="B137" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C137" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D137" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
     </row>
     <row r="138" spans="1:4">
@@ -4392,13 +4401,13 @@
         <v>140</v>
       </c>
       <c r="B138" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C138" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D138" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
     </row>
     <row r="139" spans="1:4">
@@ -4406,13 +4415,13 @@
         <v>141</v>
       </c>
       <c r="B139" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C139" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D139" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
     </row>
     <row r="140" spans="1:4">
@@ -4420,13 +4429,13 @@
         <v>142</v>
       </c>
       <c r="B140" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C140" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D140" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
     </row>
     <row r="141" spans="1:4">
@@ -4434,13 +4443,13 @@
         <v>143</v>
       </c>
       <c r="B141" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C141" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D141" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
     </row>
     <row r="142" spans="1:4">
@@ -4448,13 +4457,13 @@
         <v>144</v>
       </c>
       <c r="B142" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C142" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D142" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
     </row>
     <row r="143" spans="1:4">
@@ -4462,13 +4471,13 @@
         <v>145</v>
       </c>
       <c r="B143" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C143" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D143" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
     </row>
     <row r="144" spans="1:4">
@@ -4476,13 +4485,13 @@
         <v>146</v>
       </c>
       <c r="B144" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C144" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D144" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
     </row>
     <row r="145" spans="1:4">
@@ -4490,13 +4499,13 @@
         <v>147</v>
       </c>
       <c r="B145" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C145" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D145" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
     </row>
     <row r="146" spans="1:4">
@@ -4504,13 +4513,13 @@
         <v>148</v>
       </c>
       <c r="B146" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C146" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D146" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
     </row>
     <row r="147" spans="1:4">
@@ -4518,13 +4527,13 @@
         <v>149</v>
       </c>
       <c r="B147" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C147" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="D147" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
     </row>
     <row r="148" spans="1:4">
@@ -4532,13 +4541,13 @@
         <v>150</v>
       </c>
       <c r="B148" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C148" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D148" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
     </row>
     <row r="149" spans="1:4">
@@ -4546,13 +4555,13 @@
         <v>151</v>
       </c>
       <c r="B149" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C149" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="D149" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
     </row>
     <row r="150" spans="1:4">
@@ -4560,13 +4569,13 @@
         <v>152</v>
       </c>
       <c r="B150" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C150" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D150" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
     </row>
     <row r="151" spans="1:4">
@@ -4574,13 +4583,13 @@
         <v>153</v>
       </c>
       <c r="B151" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C151" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D151" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
     </row>
     <row r="152" spans="1:4">
@@ -4588,13 +4597,13 @@
         <v>154</v>
       </c>
       <c r="B152" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C152" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D152" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
     </row>
     <row r="153" spans="1:4">
@@ -4602,13 +4611,13 @@
         <v>155</v>
       </c>
       <c r="B153" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C153" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D153" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
     </row>
     <row r="154" spans="1:4">
@@ -4616,13 +4625,13 @@
         <v>156</v>
       </c>
       <c r="B154" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C154" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D154" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
     </row>
     <row r="155" spans="1:4">
@@ -4630,13 +4639,13 @@
         <v>157</v>
       </c>
       <c r="B155" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C155" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D155" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
     </row>
     <row r="156" spans="1:4">
@@ -4644,13 +4653,13 @@
         <v>158</v>
       </c>
       <c r="B156" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C156" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D156" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
     </row>
     <row r="157" spans="1:4">
@@ -4658,13 +4667,13 @@
         <v>159</v>
       </c>
       <c r="B157" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C157" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="D157" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
     </row>
     <row r="158" spans="1:4">
@@ -4672,13 +4681,13 @@
         <v>160</v>
       </c>
       <c r="B158" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C158" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D158" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
     </row>
     <row r="159" spans="1:4">
@@ -4686,13 +4695,13 @@
         <v>161</v>
       </c>
       <c r="B159" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C159" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D159" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
     </row>
     <row r="160" spans="1:4">
@@ -4700,13 +4709,13 @@
         <v>162</v>
       </c>
       <c r="B160" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C160" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="D160" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
     </row>
     <row r="161" spans="1:4">
@@ -4714,13 +4723,13 @@
         <v>163</v>
       </c>
       <c r="B161" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C161" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D161" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
     </row>
     <row r="162" spans="1:4">
@@ -4728,13 +4737,13 @@
         <v>164</v>
       </c>
       <c r="B162" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C162" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D162" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
     </row>
     <row r="163" spans="1:4">
@@ -4742,13 +4751,13 @@
         <v>165</v>
       </c>
       <c r="B163" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C163" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D163" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
     </row>
     <row r="164" spans="1:4">
@@ -4756,13 +4765,13 @@
         <v>166</v>
       </c>
       <c r="B164" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C164" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D164" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
     </row>
     <row r="165" spans="1:4">
@@ -4770,13 +4779,13 @@
         <v>167</v>
       </c>
       <c r="B165" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C165" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="D165" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
     </row>
     <row r="166" spans="1:4">
@@ -4784,13 +4793,13 @@
         <v>168</v>
       </c>
       <c r="B166" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C166" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D166" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
     </row>
     <row r="167" spans="1:4">
@@ -4798,13 +4807,13 @@
         <v>169</v>
       </c>
       <c r="B167" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C167" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D167" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
     </row>
     <row r="168" spans="1:4">
@@ -4812,13 +4821,13 @@
         <v>170</v>
       </c>
       <c r="B168" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C168" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D168" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
     </row>
     <row r="169" spans="1:4">
@@ -4826,13 +4835,13 @@
         <v>171</v>
       </c>
       <c r="B169" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C169" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D169" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
     </row>
     <row r="170" spans="1:4">
@@ -4840,13 +4849,13 @@
         <v>172</v>
       </c>
       <c r="B170" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C170" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D170" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
     </row>
     <row r="171" spans="1:4">
@@ -4854,13 +4863,13 @@
         <v>173</v>
       </c>
       <c r="B171" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C171" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="D171" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
     </row>
     <row r="172" spans="1:4">
@@ -4868,13 +4877,13 @@
         <v>174</v>
       </c>
       <c r="B172" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C172" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D172" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
     </row>
     <row r="173" spans="1:4">
@@ -4882,13 +4891,13 @@
         <v>175</v>
       </c>
       <c r="B173" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C173" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D173" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
     </row>
     <row r="174" spans="1:4">
@@ -4896,13 +4905,13 @@
         <v>176</v>
       </c>
       <c r="B174" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C174" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D174" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
     </row>
     <row r="175" spans="1:4">
@@ -4910,13 +4919,13 @@
         <v>177</v>
       </c>
       <c r="B175" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C175" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D175" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
     </row>
     <row r="176" spans="1:4">
@@ -4924,13 +4933,13 @@
         <v>178</v>
       </c>
       <c r="B176" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C176" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D176" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
     </row>
     <row r="177" spans="1:4">
@@ -4938,13 +4947,13 @@
         <v>179</v>
       </c>
       <c r="B177" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C177" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="D177" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
     </row>
     <row r="178" spans="1:4">
@@ -4952,13 +4961,13 @@
         <v>180</v>
       </c>
       <c r="B178" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C178" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D178" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
     </row>
     <row r="179" spans="1:4">
@@ -4966,13 +4975,13 @@
         <v>181</v>
       </c>
       <c r="B179" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C179" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D179" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
     </row>
     <row r="180" spans="1:4">
@@ -4980,13 +4989,13 @@
         <v>182</v>
       </c>
       <c r="B180" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C180" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D180" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
     </row>
     <row r="181" spans="1:4">
@@ -4994,13 +5003,13 @@
         <v>183</v>
       </c>
       <c r="B181" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C181" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D181" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
     </row>
     <row r="182" spans="1:4">
@@ -5008,13 +5017,13 @@
         <v>184</v>
       </c>
       <c r="B182" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C182" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D182" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
     </row>
     <row r="183" spans="1:4">
@@ -5022,13 +5031,13 @@
         <v>185</v>
       </c>
       <c r="B183" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C183" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D183" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
     </row>
     <row r="184" spans="1:4">
@@ -5036,13 +5045,13 @@
         <v>186</v>
       </c>
       <c r="B184" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C184" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D184" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
     </row>
     <row r="185" spans="1:4">
@@ -5050,13 +5059,13 @@
         <v>187</v>
       </c>
       <c r="B185" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C185" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D185" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
     </row>
     <row r="186" spans="1:4">
@@ -5064,13 +5073,13 @@
         <v>188</v>
       </c>
       <c r="B186" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C186" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D186" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
     </row>
     <row r="187" spans="1:4">
@@ -5078,13 +5087,13 @@
         <v>189</v>
       </c>
       <c r="B187" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C187" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D187" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
     </row>
     <row r="188" spans="1:4">
@@ -5092,13 +5101,13 @@
         <v>190</v>
       </c>
       <c r="B188" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C188" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D188" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
     </row>
     <row r="189" spans="1:4">
@@ -5106,13 +5115,13 @@
         <v>191</v>
       </c>
       <c r="B189" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C189" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="D189" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
     </row>
     <row r="190" spans="1:4">
@@ -5120,13 +5129,13 @@
         <v>192</v>
       </c>
       <c r="B190" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C190" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D190" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
     </row>
     <row r="191" spans="1:4">
@@ -5134,13 +5143,13 @@
         <v>193</v>
       </c>
       <c r="B191" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C191" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="D191" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
     </row>
     <row r="192" spans="1:4">
@@ -5148,13 +5157,13 @@
         <v>194</v>
       </c>
       <c r="B192" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C192" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="D192" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
     </row>
     <row r="193" spans="1:4">
@@ -5162,13 +5171,13 @@
         <v>195</v>
       </c>
       <c r="B193" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C193" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="D193" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
     </row>
     <row r="194" spans="1:4">
@@ -5176,13 +5185,13 @@
         <v>196</v>
       </c>
       <c r="B194" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C194" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="D194" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
     </row>
     <row r="195" spans="1:4">
@@ -5190,13 +5199,13 @@
         <v>197</v>
       </c>
       <c r="B195" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C195" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="D195" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
     </row>
     <row r="196" spans="1:4">
@@ -5204,13 +5213,13 @@
         <v>198</v>
       </c>
       <c r="B196" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C196" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="D196" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
     </row>
     <row r="197" spans="1:4">
@@ -5218,13 +5227,13 @@
         <v>199</v>
       </c>
       <c r="B197" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C197" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="D197" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
     </row>
     <row r="198" spans="1:4">
@@ -5232,13 +5241,13 @@
         <v>200</v>
       </c>
       <c r="B198" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C198" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="D198" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
     </row>
     <row r="199" spans="1:4">
@@ -5246,13 +5255,13 @@
         <v>201</v>
       </c>
       <c r="B199" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C199" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="D199" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
     </row>
     <row r="200" spans="1:4">
@@ -5260,13 +5269,13 @@
         <v>202</v>
       </c>
       <c r="B200" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C200" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D200" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
     </row>
     <row r="201" spans="1:4">
@@ -5274,13 +5283,13 @@
         <v>203</v>
       </c>
       <c r="B201" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C201" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D201" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
     </row>
     <row r="202" spans="1:4">
@@ -5288,13 +5297,13 @@
         <v>204</v>
       </c>
       <c r="B202" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C202" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="D202" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
     </row>
     <row r="203" spans="1:4">
@@ -5302,13 +5311,13 @@
         <v>205</v>
       </c>
       <c r="B203" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C203" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D203" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
     </row>
     <row r="204" spans="1:4">
@@ -5316,13 +5325,13 @@
         <v>206</v>
       </c>
       <c r="B204" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C204" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D204" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
     </row>
     <row r="205" spans="1:4">
@@ -5330,13 +5339,13 @@
         <v>207</v>
       </c>
       <c r="B205" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C205" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D205" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
     </row>
     <row r="206" spans="1:4">
@@ -5344,13 +5353,13 @@
         <v>208</v>
       </c>
       <c r="B206" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C206" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="D206" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
     </row>
     <row r="207" spans="1:4">
@@ -5358,13 +5367,13 @@
         <v>209</v>
       </c>
       <c r="B207" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C207" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D207" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
     </row>
     <row r="208" spans="1:4">
@@ -5372,13 +5381,13 @@
         <v>210</v>
       </c>
       <c r="B208" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C208" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D208" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
     </row>
     <row r="209" spans="1:4">
@@ -5386,13 +5395,13 @@
         <v>211</v>
       </c>
       <c r="B209" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C209" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D209" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
     </row>
     <row r="210" spans="1:4">
@@ -5400,13 +5409,13 @@
         <v>212</v>
       </c>
       <c r="B210" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C210" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D210" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
     </row>
     <row r="211" spans="1:4">
@@ -5414,13 +5423,13 @@
         <v>213</v>
       </c>
       <c r="B211" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C211" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D211" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
     </row>
     <row r="212" spans="1:4">
@@ -5428,13 +5437,13 @@
         <v>214</v>
       </c>
       <c r="B212" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C212" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D212" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
     </row>
     <row r="213" spans="1:4">
@@ -5442,13 +5451,13 @@
         <v>215</v>
       </c>
       <c r="B213" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C213" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D213" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
     </row>
     <row r="214" spans="1:4">
@@ -5456,13 +5465,13 @@
         <v>216</v>
       </c>
       <c r="B214" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C214" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D214" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
     </row>
     <row r="215" spans="1:4">
@@ -5470,13 +5479,13 @@
         <v>217</v>
       </c>
       <c r="B215" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C215" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D215" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
     </row>
     <row r="216" spans="1:4">
@@ -5484,13 +5493,13 @@
         <v>218</v>
       </c>
       <c r="B216" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C216" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D216" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
     </row>
     <row r="217" spans="1:4">
@@ -5498,13 +5507,13 @@
         <v>219</v>
       </c>
       <c r="B217" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="C217" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D217" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
     </row>
     <row r="218" spans="1:4">
@@ -5512,13 +5521,13 @@
         <v>220</v>
       </c>
       <c r="B218" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C218" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="D218" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
     </row>
     <row r="219" spans="1:4">
@@ -5526,13 +5535,13 @@
         <v>221</v>
       </c>
       <c r="B219" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C219" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="D219" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
     </row>
     <row r="220" spans="1:4">
@@ -5540,13 +5549,13 @@
         <v>222</v>
       </c>
       <c r="B220" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C220" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D220" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
     </row>
     <row r="221" spans="1:4">
@@ -5554,13 +5563,13 @@
         <v>223</v>
       </c>
       <c r="B221" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C221" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="D221" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
     </row>
     <row r="222" spans="1:4">
@@ -5568,13 +5577,13 @@
         <v>224</v>
       </c>
       <c r="B222" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C222" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D222" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
     </row>
     <row r="223" spans="1:4">
@@ -5582,13 +5591,13 @@
         <v>225</v>
       </c>
       <c r="B223" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C223" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D223" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
     </row>
     <row r="224" spans="1:4">
@@ -5596,13 +5605,13 @@
         <v>226</v>
       </c>
       <c r="B224" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C224" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="D224" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
     </row>
     <row r="225" spans="1:4">
@@ -5610,13 +5619,13 @@
         <v>227</v>
       </c>
       <c r="B225" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C225" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D225" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
     </row>
     <row r="226" spans="1:4">
@@ -5624,13 +5633,13 @@
         <v>228</v>
       </c>
       <c r="B226" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C226" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="D226" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
     </row>
     <row r="227" spans="1:4">
@@ -5638,13 +5647,13 @@
         <v>229</v>
       </c>
       <c r="B227" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C227" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D227" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
     </row>
     <row r="228" spans="1:4">
@@ -5652,13 +5661,13 @@
         <v>230</v>
       </c>
       <c r="B228" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="C228" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="D228" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
     </row>
     <row r="229" spans="1:4">
@@ -5666,13 +5675,13 @@
         <v>231</v>
       </c>
       <c r="B229" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C229" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="D229" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
     </row>
     <row r="230" spans="1:4">
@@ -5680,13 +5689,13 @@
         <v>232</v>
       </c>
       <c r="B230" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C230" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D230" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
     </row>
     <row r="231" spans="1:4">
@@ -5694,13 +5703,13 @@
         <v>233</v>
       </c>
       <c r="B231" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="C231" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D231" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
     </row>
     <row r="232" spans="1:4">
@@ -5708,13 +5717,13 @@
         <v>234</v>
       </c>
       <c r="B232" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C232" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="D232" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
     </row>
     <row r="233" spans="1:4">
@@ -5722,13 +5731,13 @@
         <v>235</v>
       </c>
       <c r="B233" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="C233" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D233" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
     </row>
     <row r="234" spans="1:4">
@@ -5742,7 +5751,7 @@
         <v>236</v>
       </c>
       <c r="D234" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
     </row>
     <row r="235" spans="1:4">
@@ -5756,7 +5765,7 @@
         <v>237</v>
       </c>
       <c r="D235" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
     <row r="236" spans="1:4">
@@ -5764,13 +5773,27 @@
         <v>238</v>
       </c>
       <c r="B236" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C236" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="D236" t="s">
-        <v>706</v>
+        <v>708</v>
+      </c>
+    </row>
+    <row r="237" spans="1:4">
+      <c r="A237" t="s">
+        <v>239</v>
+      </c>
+      <c r="B237" t="s">
+        <v>473</v>
+      </c>
+      <c r="C237" t="s">
+        <v>473</v>
+      </c>
+      <c r="D237" t="s">
+        <v>709</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cap nhat lich su gui va cau hinh sau khi spam Hau Kiem Kho Kho
</commit_message>
<xml_diff>
--- a/SPAM_PHIEU_CHUYEN/CHI TIẾT MÁT/Danh sách Siêu thị.xlsx
+++ b/SPAM_PHIEU_CHUYEN/CHI TIẾT MÁT/Danh sách Siêu thị.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="713">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="716">
   <si>
     <t>Tên Siêu thị</t>
   </si>
@@ -739,6 +739,9 @@
     <t>KFM_HCM_Q12 - S.06 Chung Cư Phú Cường Home</t>
   </si>
   <si>
+    <t>KFM_BDU_DAN - R01.14 Block A2 Charm Ruby</t>
+  </si>
+  <si>
     <t>A101</t>
   </si>
   <si>
@@ -1444,6 +1447,9 @@
     <t>A254</t>
   </si>
   <si>
+    <t>A262</t>
+  </si>
+  <si>
     <t>-4970846623</t>
   </si>
   <si>
@@ -2153,6 +2159,9 @@
   </si>
   <si>
     <t>-1003932058795</t>
+  </si>
+  <si>
+    <t>-1004438420846</t>
   </si>
 </sst>
 </file>
@@ -2484,7 +2493,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D238"/>
+  <dimension ref="A1:D239"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -2506,13 +2515,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D2" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2520,13 +2529,13 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D3" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2534,13 +2543,13 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C4" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D4" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2548,13 +2557,13 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D5" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2562,13 +2571,13 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D6" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2576,13 +2585,13 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C7" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D7" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2590,13 +2599,13 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C8" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D8" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2604,13 +2613,13 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D9" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2618,13 +2627,13 @@
         <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C10" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D10" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2632,13 +2641,13 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C11" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D11" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2646,13 +2655,13 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C12" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D12" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -2660,13 +2669,13 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C13" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D13" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -2674,13 +2683,13 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C14" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D14" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -2688,13 +2697,13 @@
         <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C15" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D15" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -2702,13 +2711,13 @@
         <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C16" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D16" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -2716,13 +2725,13 @@
         <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C17" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D17" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2730,13 +2739,13 @@
         <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C18" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D18" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -2744,13 +2753,13 @@
         <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C19" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D19" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -2758,13 +2767,13 @@
         <v>22</v>
       </c>
       <c r="B20" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C20" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D20" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -2772,13 +2781,13 @@
         <v>23</v>
       </c>
       <c r="B21" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C21" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D21" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -2786,13 +2795,13 @@
         <v>24</v>
       </c>
       <c r="B22" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C22" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D22" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -2800,13 +2809,13 @@
         <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C23" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D23" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -2814,13 +2823,13 @@
         <v>26</v>
       </c>
       <c r="B24" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C24" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D24" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -2828,13 +2837,13 @@
         <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C25" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D25" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -2842,13 +2851,13 @@
         <v>28</v>
       </c>
       <c r="B26" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C26" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D26" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -2856,13 +2865,13 @@
         <v>29</v>
       </c>
       <c r="B27" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C27" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D27" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -2870,13 +2879,13 @@
         <v>30</v>
       </c>
       <c r="B28" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C28" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D28" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -2884,13 +2893,13 @@
         <v>31</v>
       </c>
       <c r="B29" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C29" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D29" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -2898,13 +2907,13 @@
         <v>32</v>
       </c>
       <c r="B30" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C30" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D30" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -2912,13 +2921,13 @@
         <v>33</v>
       </c>
       <c r="B31" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C31" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D31" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -2926,13 +2935,13 @@
         <v>34</v>
       </c>
       <c r="B32" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C32" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D32" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -2940,13 +2949,13 @@
         <v>35</v>
       </c>
       <c r="B33" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C33" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D33" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -2954,13 +2963,13 @@
         <v>36</v>
       </c>
       <c r="B34" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C34" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D34" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -2968,13 +2977,13 @@
         <v>37</v>
       </c>
       <c r="B35" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C35" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D35" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -2982,13 +2991,13 @@
         <v>38</v>
       </c>
       <c r="B36" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C36" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D36" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -2996,13 +3005,13 @@
         <v>39</v>
       </c>
       <c r="B37" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C37" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D37" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -3010,13 +3019,13 @@
         <v>40</v>
       </c>
       <c r="B38" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C38" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D38" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -3024,13 +3033,13 @@
         <v>41</v>
       </c>
       <c r="B39" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C39" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D39" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -3038,13 +3047,13 @@
         <v>42</v>
       </c>
       <c r="B40" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C40" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D40" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -3052,13 +3061,13 @@
         <v>43</v>
       </c>
       <c r="B41" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C41" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D41" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -3066,13 +3075,13 @@
         <v>44</v>
       </c>
       <c r="B42" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C42" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D42" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -3080,13 +3089,13 @@
         <v>45</v>
       </c>
       <c r="B43" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C43" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D43" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -3094,13 +3103,13 @@
         <v>46</v>
       </c>
       <c r="B44" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C44" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D44" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -3108,13 +3117,13 @@
         <v>47</v>
       </c>
       <c r="B45" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C45" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D45" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -3122,13 +3131,13 @@
         <v>48</v>
       </c>
       <c r="B46" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C46" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D46" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -3136,13 +3145,13 @@
         <v>49</v>
       </c>
       <c r="B47" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C47" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D47" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -3150,13 +3159,13 @@
         <v>50</v>
       </c>
       <c r="B48" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C48" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D48" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -3164,13 +3173,13 @@
         <v>51</v>
       </c>
       <c r="B49" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C49" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D49" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -3178,13 +3187,13 @@
         <v>52</v>
       </c>
       <c r="B50" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C50" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D50" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -3192,13 +3201,13 @@
         <v>53</v>
       </c>
       <c r="B51" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C51" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D51" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -3206,13 +3215,13 @@
         <v>54</v>
       </c>
       <c r="B52" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C52" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D52" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -3220,13 +3229,13 @@
         <v>55</v>
       </c>
       <c r="B53" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C53" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D53" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -3234,13 +3243,13 @@
         <v>56</v>
       </c>
       <c r="B54" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C54" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D54" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -3248,13 +3257,13 @@
         <v>57</v>
       </c>
       <c r="B55" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C55" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D55" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -3262,13 +3271,13 @@
         <v>58</v>
       </c>
       <c r="B56" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C56" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D56" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -3276,13 +3285,13 @@
         <v>59</v>
       </c>
       <c r="B57" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C57" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D57" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -3290,13 +3299,13 @@
         <v>60</v>
       </c>
       <c r="B58" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C58" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D58" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -3304,13 +3313,13 @@
         <v>61</v>
       </c>
       <c r="B59" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C59" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D59" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -3318,13 +3327,13 @@
         <v>62</v>
       </c>
       <c r="B60" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C60" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D60" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -3332,13 +3341,13 @@
         <v>63</v>
       </c>
       <c r="B61" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C61" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D61" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -3346,13 +3355,13 @@
         <v>64</v>
       </c>
       <c r="B62" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C62" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D62" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -3360,13 +3369,13 @@
         <v>65</v>
       </c>
       <c r="B63" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C63" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D63" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -3374,13 +3383,13 @@
         <v>66</v>
       </c>
       <c r="B64" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C64" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D64" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -3388,13 +3397,13 @@
         <v>67</v>
       </c>
       <c r="B65" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C65" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D65" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -3402,13 +3411,13 @@
         <v>68</v>
       </c>
       <c r="B66" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C66" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D66" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -3416,13 +3425,13 @@
         <v>69</v>
       </c>
       <c r="B67" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C67" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D67" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -3430,13 +3439,13 @@
         <v>70</v>
       </c>
       <c r="B68" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C68" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D68" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -3444,13 +3453,13 @@
         <v>71</v>
       </c>
       <c r="B69" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C69" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D69" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -3458,13 +3467,13 @@
         <v>72</v>
       </c>
       <c r="B70" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C70" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D70" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -3472,13 +3481,13 @@
         <v>73</v>
       </c>
       <c r="B71" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C71" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D71" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -3486,13 +3495,13 @@
         <v>74</v>
       </c>
       <c r="B72" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C72" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D72" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -3500,13 +3509,13 @@
         <v>75</v>
       </c>
       <c r="B73" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C73" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D73" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -3514,13 +3523,13 @@
         <v>76</v>
       </c>
       <c r="B74" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C74" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D74" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -3528,13 +3537,13 @@
         <v>77</v>
       </c>
       <c r="B75" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C75" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D75" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -3542,13 +3551,13 @@
         <v>78</v>
       </c>
       <c r="B76" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C76" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D76" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -3556,13 +3565,13 @@
         <v>79</v>
       </c>
       <c r="B77" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C77" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D77" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -3570,13 +3579,13 @@
         <v>80</v>
       </c>
       <c r="B78" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C78" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D78" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -3584,13 +3593,13 @@
         <v>81</v>
       </c>
       <c r="B79" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C79" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D79" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -3598,13 +3607,13 @@
         <v>82</v>
       </c>
       <c r="B80" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C80" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D80" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -3612,13 +3621,13 @@
         <v>83</v>
       </c>
       <c r="B81" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C81" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D81" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
     </row>
     <row r="82" spans="1:4">
@@ -3626,13 +3635,13 @@
         <v>84</v>
       </c>
       <c r="B82" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C82" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D82" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -3640,13 +3649,13 @@
         <v>85</v>
       </c>
       <c r="B83" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C83" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D83" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -3654,13 +3663,13 @@
         <v>86</v>
       </c>
       <c r="B84" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C84" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D84" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -3668,13 +3677,13 @@
         <v>87</v>
       </c>
       <c r="B85" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C85" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D85" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
     </row>
     <row r="86" spans="1:4">
@@ -3682,13 +3691,13 @@
         <v>88</v>
       </c>
       <c r="B86" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C86" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D86" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
     </row>
     <row r="87" spans="1:4">
@@ -3696,13 +3705,13 @@
         <v>89</v>
       </c>
       <c r="B87" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C87" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D87" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
     </row>
     <row r="88" spans="1:4">
@@ -3710,13 +3719,13 @@
         <v>90</v>
       </c>
       <c r="B88" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C88" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D88" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -3724,13 +3733,13 @@
         <v>91</v>
       </c>
       <c r="B89" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C89" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D89" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
     </row>
     <row r="90" spans="1:4">
@@ -3738,13 +3747,13 @@
         <v>92</v>
       </c>
       <c r="B90" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C90" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D90" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -3752,13 +3761,13 @@
         <v>93</v>
       </c>
       <c r="B91" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C91" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D91" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
     </row>
     <row r="92" spans="1:4">
@@ -3766,13 +3775,13 @@
         <v>94</v>
       </c>
       <c r="B92" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C92" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D92" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
     </row>
     <row r="93" spans="1:4">
@@ -3780,13 +3789,13 @@
         <v>95</v>
       </c>
       <c r="B93" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C93" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D93" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
     </row>
     <row r="94" spans="1:4">
@@ -3794,13 +3803,13 @@
         <v>96</v>
       </c>
       <c r="B94" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C94" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D94" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
     </row>
     <row r="95" spans="1:4">
@@ -3808,13 +3817,13 @@
         <v>97</v>
       </c>
       <c r="B95" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C95" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D95" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="96" spans="1:4">
@@ -3822,13 +3831,13 @@
         <v>98</v>
       </c>
       <c r="B96" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C96" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D96" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="97" spans="1:4">
@@ -3836,13 +3845,13 @@
         <v>99</v>
       </c>
       <c r="B97" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C97" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D97" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
     </row>
     <row r="98" spans="1:4">
@@ -3850,13 +3859,13 @@
         <v>100</v>
       </c>
       <c r="B98" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C98" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D98" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
     </row>
     <row r="99" spans="1:4">
@@ -3864,13 +3873,13 @@
         <v>101</v>
       </c>
       <c r="B99" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C99" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D99" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
     </row>
     <row r="100" spans="1:4">
@@ -3878,13 +3887,13 @@
         <v>102</v>
       </c>
       <c r="B100" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C100" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D100" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
     </row>
     <row r="101" spans="1:4">
@@ -3892,13 +3901,13 @@
         <v>103</v>
       </c>
       <c r="B101" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C101" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D101" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
     </row>
     <row r="102" spans="1:4">
@@ -3906,13 +3915,13 @@
         <v>104</v>
       </c>
       <c r="B102" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C102" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D102" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
     </row>
     <row r="103" spans="1:4">
@@ -3920,13 +3929,13 @@
         <v>105</v>
       </c>
       <c r="B103" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C103" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D103" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
     </row>
     <row r="104" spans="1:4">
@@ -3934,13 +3943,13 @@
         <v>106</v>
       </c>
       <c r="B104" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C104" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D104" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
     </row>
     <row r="105" spans="1:4">
@@ -3948,13 +3957,13 @@
         <v>107</v>
       </c>
       <c r="B105" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C105" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D105" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
     <row r="106" spans="1:4">
@@ -3962,13 +3971,13 @@
         <v>108</v>
       </c>
       <c r="B106" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C106" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D106" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
     </row>
     <row r="107" spans="1:4">
@@ -3976,13 +3985,13 @@
         <v>109</v>
       </c>
       <c r="B107" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C107" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D107" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
     </row>
     <row r="108" spans="1:4">
@@ -3990,13 +3999,13 @@
         <v>110</v>
       </c>
       <c r="B108" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C108" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D108" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
     </row>
     <row r="109" spans="1:4">
@@ -4004,13 +4013,13 @@
         <v>111</v>
       </c>
       <c r="B109" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C109" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D109" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
     </row>
     <row r="110" spans="1:4">
@@ -4018,13 +4027,13 @@
         <v>112</v>
       </c>
       <c r="B110" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C110" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D110" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
     </row>
     <row r="111" spans="1:4">
@@ -4032,13 +4041,13 @@
         <v>113</v>
       </c>
       <c r="B111" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C111" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D111" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="112" spans="1:4">
@@ -4046,13 +4055,13 @@
         <v>114</v>
       </c>
       <c r="B112" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C112" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D112" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
     </row>
     <row r="113" spans="1:4">
@@ -4060,13 +4069,13 @@
         <v>115</v>
       </c>
       <c r="B113" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C113" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D113" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
     </row>
     <row r="114" spans="1:4">
@@ -4074,13 +4083,13 @@
         <v>116</v>
       </c>
       <c r="B114" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C114" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D114" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
     </row>
     <row r="115" spans="1:4">
@@ -4088,13 +4097,13 @@
         <v>117</v>
       </c>
       <c r="B115" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C115" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D115" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
     </row>
     <row r="116" spans="1:4">
@@ -4102,13 +4111,13 @@
         <v>118</v>
       </c>
       <c r="B116" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C116" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D116" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
     </row>
     <row r="117" spans="1:4">
@@ -4116,13 +4125,13 @@
         <v>119</v>
       </c>
       <c r="B117" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C117" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D117" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
     </row>
     <row r="118" spans="1:4">
@@ -4130,13 +4139,13 @@
         <v>120</v>
       </c>
       <c r="B118" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C118" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D118" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
     </row>
     <row r="119" spans="1:4">
@@ -4144,13 +4153,13 @@
         <v>121</v>
       </c>
       <c r="B119" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C119" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D119" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
     </row>
     <row r="120" spans="1:4">
@@ -4158,13 +4167,13 @@
         <v>122</v>
       </c>
       <c r="B120" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C120" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D120" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
     </row>
     <row r="121" spans="1:4">
@@ -4172,13 +4181,13 @@
         <v>123</v>
       </c>
       <c r="B121" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C121" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D121" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="122" spans="1:4">
@@ -4186,13 +4195,13 @@
         <v>124</v>
       </c>
       <c r="B122" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C122" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D122" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
     </row>
     <row r="123" spans="1:4">
@@ -4200,13 +4209,13 @@
         <v>125</v>
       </c>
       <c r="B123" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C123" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D123" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
     </row>
     <row r="124" spans="1:4">
@@ -4214,13 +4223,13 @@
         <v>126</v>
       </c>
       <c r="B124" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C124" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D124" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
     </row>
     <row r="125" spans="1:4">
@@ -4228,13 +4237,13 @@
         <v>127</v>
       </c>
       <c r="B125" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C125" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D125" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
     </row>
     <row r="126" spans="1:4">
@@ -4242,13 +4251,13 @@
         <v>128</v>
       </c>
       <c r="B126" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C126" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D126" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
     </row>
     <row r="127" spans="1:4">
@@ -4256,13 +4265,13 @@
         <v>129</v>
       </c>
       <c r="B127" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C127" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D127" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
     </row>
     <row r="128" spans="1:4">
@@ -4270,13 +4279,13 @@
         <v>130</v>
       </c>
       <c r="B128" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C128" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D128" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
     </row>
     <row r="129" spans="1:4">
@@ -4284,13 +4293,13 @@
         <v>131</v>
       </c>
       <c r="B129" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C129" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D129" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
     </row>
     <row r="130" spans="1:4">
@@ -4298,13 +4307,13 @@
         <v>132</v>
       </c>
       <c r="B130" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C130" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D130" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
     </row>
     <row r="131" spans="1:4">
@@ -4312,13 +4321,13 @@
         <v>133</v>
       </c>
       <c r="B131" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C131" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D131" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
     </row>
     <row r="132" spans="1:4">
@@ -4326,13 +4335,13 @@
         <v>134</v>
       </c>
       <c r="B132" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C132" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D132" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
     </row>
     <row r="133" spans="1:4">
@@ -4340,13 +4349,13 @@
         <v>135</v>
       </c>
       <c r="B133" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C133" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D133" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
     </row>
     <row r="134" spans="1:4">
@@ -4354,13 +4363,13 @@
         <v>136</v>
       </c>
       <c r="B134" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C134" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D134" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
     </row>
     <row r="135" spans="1:4">
@@ -4368,13 +4377,13 @@
         <v>137</v>
       </c>
       <c r="B135" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C135" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D135" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
     </row>
     <row r="136" spans="1:4">
@@ -4382,13 +4391,13 @@
         <v>138</v>
       </c>
       <c r="B136" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C136" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D136" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
     </row>
     <row r="137" spans="1:4">
@@ -4396,13 +4405,13 @@
         <v>139</v>
       </c>
       <c r="B137" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C137" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D137" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
     </row>
     <row r="138" spans="1:4">
@@ -4410,13 +4419,13 @@
         <v>140</v>
       </c>
       <c r="B138" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C138" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D138" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
     </row>
     <row r="139" spans="1:4">
@@ -4424,13 +4433,13 @@
         <v>141</v>
       </c>
       <c r="B139" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C139" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D139" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
     </row>
     <row r="140" spans="1:4">
@@ -4438,13 +4447,13 @@
         <v>142</v>
       </c>
       <c r="B140" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C140" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D140" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
     </row>
     <row r="141" spans="1:4">
@@ -4452,13 +4461,13 @@
         <v>143</v>
       </c>
       <c r="B141" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C141" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D141" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
     </row>
     <row r="142" spans="1:4">
@@ -4466,13 +4475,13 @@
         <v>144</v>
       </c>
       <c r="B142" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C142" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D142" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
     </row>
     <row r="143" spans="1:4">
@@ -4480,13 +4489,13 @@
         <v>145</v>
       </c>
       <c r="B143" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C143" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D143" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
     </row>
     <row r="144" spans="1:4">
@@ -4494,13 +4503,13 @@
         <v>146</v>
       </c>
       <c r="B144" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C144" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D144" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
     </row>
     <row r="145" spans="1:4">
@@ -4508,13 +4517,13 @@
         <v>147</v>
       </c>
       <c r="B145" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C145" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="D145" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
     </row>
     <row r="146" spans="1:4">
@@ -4522,13 +4531,13 @@
         <v>148</v>
       </c>
       <c r="B146" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C146" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D146" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
     </row>
     <row r="147" spans="1:4">
@@ -4536,13 +4545,13 @@
         <v>149</v>
       </c>
       <c r="B147" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C147" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="D147" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
     </row>
     <row r="148" spans="1:4">
@@ -4550,13 +4559,13 @@
         <v>150</v>
       </c>
       <c r="B148" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C148" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D148" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
     </row>
     <row r="149" spans="1:4">
@@ -4564,13 +4573,13 @@
         <v>151</v>
       </c>
       <c r="B149" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C149" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D149" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
     </row>
     <row r="150" spans="1:4">
@@ -4578,13 +4587,13 @@
         <v>152</v>
       </c>
       <c r="B150" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C150" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D150" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
     </row>
     <row r="151" spans="1:4">
@@ -4592,13 +4601,13 @@
         <v>153</v>
       </c>
       <c r="B151" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C151" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D151" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
     </row>
     <row r="152" spans="1:4">
@@ -4606,13 +4615,13 @@
         <v>154</v>
       </c>
       <c r="B152" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C152" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D152" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
     </row>
     <row r="153" spans="1:4">
@@ -4620,13 +4629,13 @@
         <v>155</v>
       </c>
       <c r="B153" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C153" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D153" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
     </row>
     <row r="154" spans="1:4">
@@ -4634,13 +4643,13 @@
         <v>156</v>
       </c>
       <c r="B154" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C154" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D154" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
     </row>
     <row r="155" spans="1:4">
@@ -4648,13 +4657,13 @@
         <v>157</v>
       </c>
       <c r="B155" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C155" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="D155" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
     </row>
     <row r="156" spans="1:4">
@@ -4662,13 +4671,13 @@
         <v>158</v>
       </c>
       <c r="B156" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C156" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D156" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
     </row>
     <row r="157" spans="1:4">
@@ -4676,13 +4685,13 @@
         <v>159</v>
       </c>
       <c r="B157" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C157" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D157" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
     </row>
     <row r="158" spans="1:4">
@@ -4690,13 +4699,13 @@
         <v>160</v>
       </c>
       <c r="B158" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C158" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="D158" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
     </row>
     <row r="159" spans="1:4">
@@ -4704,13 +4713,13 @@
         <v>161</v>
       </c>
       <c r="B159" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C159" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D159" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
     </row>
     <row r="160" spans="1:4">
@@ -4718,13 +4727,13 @@
         <v>162</v>
       </c>
       <c r="B160" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C160" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D160" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
     </row>
     <row r="161" spans="1:4">
@@ -4732,13 +4741,13 @@
         <v>163</v>
       </c>
       <c r="B161" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C161" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D161" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
     </row>
     <row r="162" spans="1:4">
@@ -4746,13 +4755,13 @@
         <v>164</v>
       </c>
       <c r="B162" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C162" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D162" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
     </row>
     <row r="163" spans="1:4">
@@ -4760,13 +4769,13 @@
         <v>165</v>
       </c>
       <c r="B163" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C163" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="D163" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
     </row>
     <row r="164" spans="1:4">
@@ -4774,13 +4783,13 @@
         <v>166</v>
       </c>
       <c r="B164" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C164" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D164" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
     </row>
     <row r="165" spans="1:4">
@@ -4788,13 +4797,13 @@
         <v>167</v>
       </c>
       <c r="B165" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C165" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D165" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
     </row>
     <row r="166" spans="1:4">
@@ -4802,13 +4811,13 @@
         <v>168</v>
       </c>
       <c r="B166" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C166" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D166" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
     </row>
     <row r="167" spans="1:4">
@@ -4816,13 +4825,13 @@
         <v>169</v>
       </c>
       <c r="B167" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C167" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D167" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
     </row>
     <row r="168" spans="1:4">
@@ -4830,13 +4839,13 @@
         <v>170</v>
       </c>
       <c r="B168" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C168" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D168" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
     </row>
     <row r="169" spans="1:4">
@@ -4844,13 +4853,13 @@
         <v>171</v>
       </c>
       <c r="B169" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C169" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="D169" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
     </row>
     <row r="170" spans="1:4">
@@ -4858,13 +4867,13 @@
         <v>172</v>
       </c>
       <c r="B170" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C170" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D170" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
     </row>
     <row r="171" spans="1:4">
@@ -4872,13 +4881,13 @@
         <v>173</v>
       </c>
       <c r="B171" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C171" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D171" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
     </row>
     <row r="172" spans="1:4">
@@ -4886,13 +4895,13 @@
         <v>174</v>
       </c>
       <c r="B172" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C172" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D172" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
     </row>
     <row r="173" spans="1:4">
@@ -4900,13 +4909,13 @@
         <v>175</v>
       </c>
       <c r="B173" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C173" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D173" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
     </row>
     <row r="174" spans="1:4">
@@ -4914,13 +4923,13 @@
         <v>176</v>
       </c>
       <c r="B174" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C174" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D174" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
     </row>
     <row r="175" spans="1:4">
@@ -4928,13 +4937,13 @@
         <v>177</v>
       </c>
       <c r="B175" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C175" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="D175" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
     </row>
     <row r="176" spans="1:4">
@@ -4942,13 +4951,13 @@
         <v>178</v>
       </c>
       <c r="B176" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C176" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D176" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
     </row>
     <row r="177" spans="1:4">
@@ -4956,13 +4965,13 @@
         <v>179</v>
       </c>
       <c r="B177" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C177" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D177" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
     </row>
     <row r="178" spans="1:4">
@@ -4970,13 +4979,13 @@
         <v>180</v>
       </c>
       <c r="B178" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C178" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D178" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
     </row>
     <row r="179" spans="1:4">
@@ -4984,13 +4993,13 @@
         <v>181</v>
       </c>
       <c r="B179" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C179" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D179" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
     </row>
     <row r="180" spans="1:4">
@@ -4998,13 +5007,13 @@
         <v>182</v>
       </c>
       <c r="B180" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C180" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D180" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
     </row>
     <row r="181" spans="1:4">
@@ -5012,13 +5021,13 @@
         <v>183</v>
       </c>
       <c r="B181" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C181" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D181" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
     </row>
     <row r="182" spans="1:4">
@@ -5026,13 +5035,13 @@
         <v>184</v>
       </c>
       <c r="B182" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C182" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D182" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
     </row>
     <row r="183" spans="1:4">
@@ -5040,13 +5049,13 @@
         <v>185</v>
       </c>
       <c r="B183" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C183" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D183" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
     </row>
     <row r="184" spans="1:4">
@@ -5054,13 +5063,13 @@
         <v>186</v>
       </c>
       <c r="B184" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C184" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D184" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
     </row>
     <row r="185" spans="1:4">
@@ -5068,13 +5077,13 @@
         <v>187</v>
       </c>
       <c r="B185" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C185" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D185" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
     </row>
     <row r="186" spans="1:4">
@@ -5082,13 +5091,13 @@
         <v>188</v>
       </c>
       <c r="B186" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C186" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D186" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
     </row>
     <row r="187" spans="1:4">
@@ -5096,13 +5105,13 @@
         <v>189</v>
       </c>
       <c r="B187" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C187" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="D187" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
     </row>
     <row r="188" spans="1:4">
@@ -5110,13 +5119,13 @@
         <v>190</v>
       </c>
       <c r="B188" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C188" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D188" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
     </row>
     <row r="189" spans="1:4">
@@ -5124,13 +5133,13 @@
         <v>191</v>
       </c>
       <c r="B189" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C189" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="D189" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
     </row>
     <row r="190" spans="1:4">
@@ -5138,13 +5147,13 @@
         <v>192</v>
       </c>
       <c r="B190" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C190" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="D190" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
     </row>
     <row r="191" spans="1:4">
@@ -5152,13 +5161,13 @@
         <v>193</v>
       </c>
       <c r="B191" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C191" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="D191" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
     </row>
     <row r="192" spans="1:4">
@@ -5166,13 +5175,13 @@
         <v>194</v>
       </c>
       <c r="B192" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C192" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="D192" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
     </row>
     <row r="193" spans="1:4">
@@ -5180,13 +5189,13 @@
         <v>195</v>
       </c>
       <c r="B193" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C193" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="D193" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
     </row>
     <row r="194" spans="1:4">
@@ -5194,13 +5203,13 @@
         <v>196</v>
       </c>
       <c r="B194" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C194" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="D194" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
     </row>
     <row r="195" spans="1:4">
@@ -5208,13 +5217,13 @@
         <v>197</v>
       </c>
       <c r="B195" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C195" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="D195" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
     </row>
     <row r="196" spans="1:4">
@@ -5222,13 +5231,13 @@
         <v>198</v>
       </c>
       <c r="B196" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C196" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="D196" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
     </row>
     <row r="197" spans="1:4">
@@ -5236,13 +5245,13 @@
         <v>199</v>
       </c>
       <c r="B197" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C197" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="D197" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
     </row>
     <row r="198" spans="1:4">
@@ -5250,13 +5259,13 @@
         <v>200</v>
       </c>
       <c r="B198" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C198" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D198" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
     </row>
     <row r="199" spans="1:4">
@@ -5264,13 +5273,13 @@
         <v>201</v>
       </c>
       <c r="B199" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C199" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D199" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
     </row>
     <row r="200" spans="1:4">
@@ -5278,13 +5287,13 @@
         <v>202</v>
       </c>
       <c r="B200" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C200" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="D200" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
     </row>
     <row r="201" spans="1:4">
@@ -5292,13 +5301,13 @@
         <v>203</v>
       </c>
       <c r="B201" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C201" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D201" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
     </row>
     <row r="202" spans="1:4">
@@ -5306,13 +5315,13 @@
         <v>204</v>
       </c>
       <c r="B202" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C202" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D202" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
     </row>
     <row r="203" spans="1:4">
@@ -5320,13 +5329,13 @@
         <v>205</v>
       </c>
       <c r="B203" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C203" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D203" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
     </row>
     <row r="204" spans="1:4">
@@ -5334,13 +5343,13 @@
         <v>206</v>
       </c>
       <c r="B204" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C204" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="D204" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
     </row>
     <row r="205" spans="1:4">
@@ -5348,13 +5357,13 @@
         <v>207</v>
       </c>
       <c r="B205" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C205" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D205" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
     </row>
     <row r="206" spans="1:4">
@@ -5362,13 +5371,13 @@
         <v>208</v>
       </c>
       <c r="B206" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C206" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D206" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
     </row>
     <row r="207" spans="1:4">
@@ -5376,13 +5385,13 @@
         <v>209</v>
       </c>
       <c r="B207" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C207" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D207" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
     </row>
     <row r="208" spans="1:4">
@@ -5390,13 +5399,13 @@
         <v>210</v>
       </c>
       <c r="B208" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C208" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D208" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
     </row>
     <row r="209" spans="1:4">
@@ -5404,13 +5413,13 @@
         <v>211</v>
       </c>
       <c r="B209" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C209" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D209" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
     </row>
     <row r="210" spans="1:4">
@@ -5418,13 +5427,13 @@
         <v>212</v>
       </c>
       <c r="B210" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C210" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D210" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
     </row>
     <row r="211" spans="1:4">
@@ -5432,13 +5441,13 @@
         <v>213</v>
       </c>
       <c r="B211" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C211" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D211" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
     </row>
     <row r="212" spans="1:4">
@@ -5446,13 +5455,13 @@
         <v>214</v>
       </c>
       <c r="B212" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C212" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D212" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
     </row>
     <row r="213" spans="1:4">
@@ -5460,13 +5469,13 @@
         <v>215</v>
       </c>
       <c r="B213" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C213" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D213" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
     </row>
     <row r="214" spans="1:4">
@@ -5474,13 +5483,13 @@
         <v>216</v>
       </c>
       <c r="B214" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C214" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D214" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
     </row>
     <row r="215" spans="1:4">
@@ -5488,13 +5497,13 @@
         <v>217</v>
       </c>
       <c r="B215" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="C215" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D215" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
     </row>
     <row r="216" spans="1:4">
@@ -5502,13 +5511,13 @@
         <v>218</v>
       </c>
       <c r="B216" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C216" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="D216" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
     </row>
     <row r="217" spans="1:4">
@@ -5516,13 +5525,13 @@
         <v>219</v>
       </c>
       <c r="B217" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C217" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="D217" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
     </row>
     <row r="218" spans="1:4">
@@ -5530,13 +5539,13 @@
         <v>220</v>
       </c>
       <c r="B218" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C218" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D218" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
     </row>
     <row r="219" spans="1:4">
@@ -5544,13 +5553,13 @@
         <v>221</v>
       </c>
       <c r="B219" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C219" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="D219" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
     </row>
     <row r="220" spans="1:4">
@@ -5558,13 +5567,13 @@
         <v>222</v>
       </c>
       <c r="B220" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C220" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D220" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
     </row>
     <row r="221" spans="1:4">
@@ -5572,13 +5581,13 @@
         <v>223</v>
       </c>
       <c r="B221" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C221" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D221" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
     </row>
     <row r="222" spans="1:4">
@@ -5586,13 +5595,13 @@
         <v>224</v>
       </c>
       <c r="B222" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C222" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="D222" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
     </row>
     <row r="223" spans="1:4">
@@ -5600,13 +5609,13 @@
         <v>225</v>
       </c>
       <c r="B223" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C223" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D223" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
     </row>
     <row r="224" spans="1:4">
@@ -5614,13 +5623,13 @@
         <v>226</v>
       </c>
       <c r="B224" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C224" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="D224" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
     </row>
     <row r="225" spans="1:4">
@@ -5628,13 +5637,13 @@
         <v>227</v>
       </c>
       <c r="B225" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C225" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D225" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
     </row>
     <row r="226" spans="1:4">
@@ -5642,13 +5651,13 @@
         <v>228</v>
       </c>
       <c r="B226" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="C226" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="D226" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
     </row>
     <row r="227" spans="1:4">
@@ -5656,13 +5665,13 @@
         <v>229</v>
       </c>
       <c r="B227" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C227" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="D227" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
     </row>
     <row r="228" spans="1:4">
@@ -5670,13 +5679,13 @@
         <v>230</v>
       </c>
       <c r="B228" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C228" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D228" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
     </row>
     <row r="229" spans="1:4">
@@ -5684,13 +5693,13 @@
         <v>231</v>
       </c>
       <c r="B229" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="C229" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D229" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
     </row>
     <row r="230" spans="1:4">
@@ -5698,13 +5707,13 @@
         <v>232</v>
       </c>
       <c r="B230" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C230" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="D230" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
     </row>
     <row r="231" spans="1:4">
@@ -5712,13 +5721,13 @@
         <v>233</v>
       </c>
       <c r="B231" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="C231" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D231" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
     <row r="232" spans="1:4">
@@ -5726,13 +5735,13 @@
         <v>234</v>
       </c>
       <c r="B232" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C232" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="D232" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
     </row>
     <row r="233" spans="1:4">
@@ -5740,13 +5749,13 @@
         <v>235</v>
       </c>
       <c r="B233" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C233" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="D233" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
     </row>
     <row r="234" spans="1:4">
@@ -5760,7 +5769,7 @@
         <v>236</v>
       </c>
       <c r="D234" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="235" spans="1:4">
@@ -5774,7 +5783,7 @@
         <v>237</v>
       </c>
       <c r="D235" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
     </row>
     <row r="236" spans="1:4">
@@ -5782,13 +5791,13 @@
         <v>238</v>
       </c>
       <c r="B236" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C236" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D236" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
     </row>
     <row r="237" spans="1:4">
@@ -5796,13 +5805,13 @@
         <v>239</v>
       </c>
       <c r="B237" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C237" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="D237" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
     </row>
     <row r="238" spans="1:4">
@@ -5810,13 +5819,27 @@
         <v>240</v>
       </c>
       <c r="B238" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C238" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D238" t="s">
-        <v>712</v>
+        <v>714</v>
+      </c>
+    </row>
+    <row r="239" spans="1:4">
+      <c r="A239" t="s">
+        <v>241</v>
+      </c>
+      <c r="B239" t="s">
+        <v>477</v>
+      </c>
+      <c r="C239" t="s">
+        <v>477</v>
+      </c>
+      <c r="D239" t="s">
+        <v>715</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cập nhật dữ liệu cấu hình và lịch sử spam hậu kiểm kho khô
</commit_message>
<xml_diff>
--- a/SPAM_PHIEU_CHUYEN/CHI TIẾT MÁT/Danh sách Siêu thị.xlsx
+++ b/SPAM_PHIEU_CHUYEN/CHI TIẾT MÁT/Danh sách Siêu thị.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="716">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="719">
   <si>
     <t>Tên Siêu thị</t>
   </si>
@@ -742,6 +742,9 @@
     <t>KFM_BDU_DAN - R01.14 Block A2 Charm Ruby</t>
   </si>
   <si>
+    <t>KFM_HCM_Q08 - A6-7 Block A Diamond Lotus Riverside</t>
+  </si>
+  <si>
     <t>A101</t>
   </si>
   <si>
@@ -1450,6 +1453,9 @@
     <t>A262</t>
   </si>
   <si>
+    <t>A243</t>
+  </si>
+  <si>
     <t>-4970846623</t>
   </si>
   <si>
@@ -2162,6 +2168,9 @@
   </si>
   <si>
     <t>-1004438420846</t>
+  </si>
+  <si>
+    <t>-1003932619661</t>
   </si>
 </sst>
 </file>
@@ -2493,7 +2502,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D239"/>
+  <dimension ref="A1:D240"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -2515,13 +2524,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D2" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2529,13 +2538,13 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D3" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2543,13 +2552,13 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D4" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2557,13 +2566,13 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C5" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D5" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2571,13 +2580,13 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C6" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D6" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2585,13 +2594,13 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C7" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D7" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2599,13 +2608,13 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C8" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D8" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2613,13 +2622,13 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C9" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D9" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2627,13 +2636,13 @@
         <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C10" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D10" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2641,13 +2650,13 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C11" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D11" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2655,13 +2664,13 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C12" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D12" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -2669,13 +2678,13 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C13" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D13" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -2683,13 +2692,13 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C14" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D14" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -2697,13 +2706,13 @@
         <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C15" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D15" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -2711,13 +2720,13 @@
         <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C16" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D16" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -2725,13 +2734,13 @@
         <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C17" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D17" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2739,13 +2748,13 @@
         <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C18" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D18" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -2753,13 +2762,13 @@
         <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C19" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D19" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -2767,13 +2776,13 @@
         <v>22</v>
       </c>
       <c r="B20" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C20" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D20" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -2781,13 +2790,13 @@
         <v>23</v>
       </c>
       <c r="B21" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C21" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D21" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -2795,13 +2804,13 @@
         <v>24</v>
       </c>
       <c r="B22" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C22" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D22" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -2809,13 +2818,13 @@
         <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C23" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D23" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -2823,13 +2832,13 @@
         <v>26</v>
       </c>
       <c r="B24" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C24" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D24" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -2837,13 +2846,13 @@
         <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C25" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D25" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -2851,13 +2860,13 @@
         <v>28</v>
       </c>
       <c r="B26" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C26" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D26" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -2865,13 +2874,13 @@
         <v>29</v>
       </c>
       <c r="B27" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C27" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D27" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -2879,13 +2888,13 @@
         <v>30</v>
       </c>
       <c r="B28" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C28" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D28" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -2893,13 +2902,13 @@
         <v>31</v>
       </c>
       <c r="B29" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C29" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D29" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -2907,13 +2916,13 @@
         <v>32</v>
       </c>
       <c r="B30" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C30" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D30" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -2921,13 +2930,13 @@
         <v>33</v>
       </c>
       <c r="B31" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C31" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D31" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -2935,13 +2944,13 @@
         <v>34</v>
       </c>
       <c r="B32" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C32" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D32" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -2949,13 +2958,13 @@
         <v>35</v>
       </c>
       <c r="B33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C33" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D33" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -2963,13 +2972,13 @@
         <v>36</v>
       </c>
       <c r="B34" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C34" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D34" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -2977,13 +2986,13 @@
         <v>37</v>
       </c>
       <c r="B35" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C35" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D35" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -2991,13 +3000,13 @@
         <v>38</v>
       </c>
       <c r="B36" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C36" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D36" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -3005,13 +3014,13 @@
         <v>39</v>
       </c>
       <c r="B37" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C37" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D37" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -3019,13 +3028,13 @@
         <v>40</v>
       </c>
       <c r="B38" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C38" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D38" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -3033,13 +3042,13 @@
         <v>41</v>
       </c>
       <c r="B39" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C39" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D39" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -3047,13 +3056,13 @@
         <v>42</v>
       </c>
       <c r="B40" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C40" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D40" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -3061,13 +3070,13 @@
         <v>43</v>
       </c>
       <c r="B41" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C41" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D41" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -3075,13 +3084,13 @@
         <v>44</v>
       </c>
       <c r="B42" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C42" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D42" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -3089,13 +3098,13 @@
         <v>45</v>
       </c>
       <c r="B43" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C43" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D43" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -3103,13 +3112,13 @@
         <v>46</v>
       </c>
       <c r="B44" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C44" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D44" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -3117,13 +3126,13 @@
         <v>47</v>
       </c>
       <c r="B45" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C45" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D45" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -3131,13 +3140,13 @@
         <v>48</v>
       </c>
       <c r="B46" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C46" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D46" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -3145,13 +3154,13 @@
         <v>49</v>
       </c>
       <c r="B47" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C47" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D47" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -3159,13 +3168,13 @@
         <v>50</v>
       </c>
       <c r="B48" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C48" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D48" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -3173,13 +3182,13 @@
         <v>51</v>
       </c>
       <c r="B49" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C49" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D49" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -3187,13 +3196,13 @@
         <v>52</v>
       </c>
       <c r="B50" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C50" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D50" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -3201,13 +3210,13 @@
         <v>53</v>
       </c>
       <c r="B51" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C51" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D51" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -3215,13 +3224,13 @@
         <v>54</v>
       </c>
       <c r="B52" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C52" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D52" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -3229,13 +3238,13 @@
         <v>55</v>
       </c>
       <c r="B53" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C53" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D53" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -3243,13 +3252,13 @@
         <v>56</v>
       </c>
       <c r="B54" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C54" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D54" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -3257,13 +3266,13 @@
         <v>57</v>
       </c>
       <c r="B55" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C55" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D55" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -3271,13 +3280,13 @@
         <v>58</v>
       </c>
       <c r="B56" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C56" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D56" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -3285,13 +3294,13 @@
         <v>59</v>
       </c>
       <c r="B57" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C57" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D57" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -3299,13 +3308,13 @@
         <v>60</v>
       </c>
       <c r="B58" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C58" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D58" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -3313,13 +3322,13 @@
         <v>61</v>
       </c>
       <c r="B59" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C59" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D59" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -3327,13 +3336,13 @@
         <v>62</v>
       </c>
       <c r="B60" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C60" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D60" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -3341,13 +3350,13 @@
         <v>63</v>
       </c>
       <c r="B61" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C61" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D61" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -3355,13 +3364,13 @@
         <v>64</v>
       </c>
       <c r="B62" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C62" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D62" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -3369,13 +3378,13 @@
         <v>65</v>
       </c>
       <c r="B63" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C63" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D63" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -3383,13 +3392,13 @@
         <v>66</v>
       </c>
       <c r="B64" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C64" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D64" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -3397,13 +3406,13 @@
         <v>67</v>
       </c>
       <c r="B65" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C65" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D65" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -3411,13 +3420,13 @@
         <v>68</v>
       </c>
       <c r="B66" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C66" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D66" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -3425,13 +3434,13 @@
         <v>69</v>
       </c>
       <c r="B67" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C67" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D67" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -3439,13 +3448,13 @@
         <v>70</v>
       </c>
       <c r="B68" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C68" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D68" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -3453,13 +3462,13 @@
         <v>71</v>
       </c>
       <c r="B69" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C69" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D69" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -3467,13 +3476,13 @@
         <v>72</v>
       </c>
       <c r="B70" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C70" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D70" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -3481,13 +3490,13 @@
         <v>73</v>
       </c>
       <c r="B71" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C71" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D71" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -3495,13 +3504,13 @@
         <v>74</v>
       </c>
       <c r="B72" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C72" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D72" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -3509,13 +3518,13 @@
         <v>75</v>
       </c>
       <c r="B73" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C73" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D73" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -3523,13 +3532,13 @@
         <v>76</v>
       </c>
       <c r="B74" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C74" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D74" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -3537,13 +3546,13 @@
         <v>77</v>
       </c>
       <c r="B75" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C75" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D75" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -3551,13 +3560,13 @@
         <v>78</v>
       </c>
       <c r="B76" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C76" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D76" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -3565,13 +3574,13 @@
         <v>79</v>
       </c>
       <c r="B77" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C77" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D77" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -3579,13 +3588,13 @@
         <v>80</v>
       </c>
       <c r="B78" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C78" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D78" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -3593,13 +3602,13 @@
         <v>81</v>
       </c>
       <c r="B79" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C79" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D79" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -3607,13 +3616,13 @@
         <v>82</v>
       </c>
       <c r="B80" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C80" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D80" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -3621,13 +3630,13 @@
         <v>83</v>
       </c>
       <c r="B81" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C81" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D81" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
     </row>
     <row r="82" spans="1:4">
@@ -3635,13 +3644,13 @@
         <v>84</v>
       </c>
       <c r="B82" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C82" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D82" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -3649,13 +3658,13 @@
         <v>85</v>
       </c>
       <c r="B83" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C83" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D83" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -3663,13 +3672,13 @@
         <v>86</v>
       </c>
       <c r="B84" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C84" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D84" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -3677,13 +3686,13 @@
         <v>87</v>
       </c>
       <c r="B85" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C85" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D85" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
     </row>
     <row r="86" spans="1:4">
@@ -3691,13 +3700,13 @@
         <v>88</v>
       </c>
       <c r="B86" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C86" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D86" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
     </row>
     <row r="87" spans="1:4">
@@ -3705,13 +3714,13 @@
         <v>89</v>
       </c>
       <c r="B87" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C87" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D87" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
     </row>
     <row r="88" spans="1:4">
@@ -3719,13 +3728,13 @@
         <v>90</v>
       </c>
       <c r="B88" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C88" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D88" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -3733,13 +3742,13 @@
         <v>91</v>
       </c>
       <c r="B89" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C89" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D89" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
     </row>
     <row r="90" spans="1:4">
@@ -3747,13 +3756,13 @@
         <v>92</v>
       </c>
       <c r="B90" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C90" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D90" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -3761,13 +3770,13 @@
         <v>93</v>
       </c>
       <c r="B91" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C91" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D91" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
     </row>
     <row r="92" spans="1:4">
@@ -3775,13 +3784,13 @@
         <v>94</v>
       </c>
       <c r="B92" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C92" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D92" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
     </row>
     <row r="93" spans="1:4">
@@ -3789,13 +3798,13 @@
         <v>95</v>
       </c>
       <c r="B93" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C93" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D93" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="94" spans="1:4">
@@ -3803,13 +3812,13 @@
         <v>96</v>
       </c>
       <c r="B94" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C94" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D94" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="95" spans="1:4">
@@ -3817,13 +3826,13 @@
         <v>97</v>
       </c>
       <c r="B95" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C95" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D95" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
     </row>
     <row r="96" spans="1:4">
@@ -3831,13 +3840,13 @@
         <v>98</v>
       </c>
       <c r="B96" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C96" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D96" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
     </row>
     <row r="97" spans="1:4">
@@ -3845,13 +3854,13 @@
         <v>99</v>
       </c>
       <c r="B97" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C97" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D97" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
     </row>
     <row r="98" spans="1:4">
@@ -3859,13 +3868,13 @@
         <v>100</v>
       </c>
       <c r="B98" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C98" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D98" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
     </row>
     <row r="99" spans="1:4">
@@ -3873,13 +3882,13 @@
         <v>101</v>
       </c>
       <c r="B99" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C99" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D99" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
     </row>
     <row r="100" spans="1:4">
@@ -3887,13 +3896,13 @@
         <v>102</v>
       </c>
       <c r="B100" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C100" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D100" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
     </row>
     <row r="101" spans="1:4">
@@ -3901,13 +3910,13 @@
         <v>103</v>
       </c>
       <c r="B101" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C101" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D101" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
     </row>
     <row r="102" spans="1:4">
@@ -3915,13 +3924,13 @@
         <v>104</v>
       </c>
       <c r="B102" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C102" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D102" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
     </row>
     <row r="103" spans="1:4">
@@ -3929,13 +3938,13 @@
         <v>105</v>
       </c>
       <c r="B103" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C103" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D103" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
     <row r="104" spans="1:4">
@@ -3943,13 +3952,13 @@
         <v>106</v>
       </c>
       <c r="B104" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C104" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D104" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
     </row>
     <row r="105" spans="1:4">
@@ -3957,13 +3966,13 @@
         <v>107</v>
       </c>
       <c r="B105" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C105" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D105" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
     </row>
     <row r="106" spans="1:4">
@@ -3971,13 +3980,13 @@
         <v>108</v>
       </c>
       <c r="B106" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C106" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D106" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
     </row>
     <row r="107" spans="1:4">
@@ -3985,13 +3994,13 @@
         <v>109</v>
       </c>
       <c r="B107" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C107" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D107" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
     </row>
     <row r="108" spans="1:4">
@@ -3999,13 +4008,13 @@
         <v>110</v>
       </c>
       <c r="B108" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C108" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D108" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
     </row>
     <row r="109" spans="1:4">
@@ -4013,13 +4022,13 @@
         <v>111</v>
       </c>
       <c r="B109" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C109" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D109" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="110" spans="1:4">
@@ -4027,13 +4036,13 @@
         <v>112</v>
       </c>
       <c r="B110" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C110" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D110" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
     </row>
     <row r="111" spans="1:4">
@@ -4041,13 +4050,13 @@
         <v>113</v>
       </c>
       <c r="B111" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C111" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D111" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
     </row>
     <row r="112" spans="1:4">
@@ -4055,13 +4064,13 @@
         <v>114</v>
       </c>
       <c r="B112" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C112" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D112" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
     </row>
     <row r="113" spans="1:4">
@@ -4069,13 +4078,13 @@
         <v>115</v>
       </c>
       <c r="B113" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C113" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D113" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
     </row>
     <row r="114" spans="1:4">
@@ -4083,13 +4092,13 @@
         <v>116</v>
       </c>
       <c r="B114" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C114" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D114" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
     </row>
     <row r="115" spans="1:4">
@@ -4097,13 +4106,13 @@
         <v>117</v>
       </c>
       <c r="B115" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C115" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D115" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
     </row>
     <row r="116" spans="1:4">
@@ -4111,13 +4120,13 @@
         <v>118</v>
       </c>
       <c r="B116" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C116" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D116" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
     </row>
     <row r="117" spans="1:4">
@@ -4125,13 +4134,13 @@
         <v>119</v>
       </c>
       <c r="B117" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C117" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D117" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
     </row>
     <row r="118" spans="1:4">
@@ -4139,13 +4148,13 @@
         <v>120</v>
       </c>
       <c r="B118" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C118" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D118" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
     </row>
     <row r="119" spans="1:4">
@@ -4153,13 +4162,13 @@
         <v>121</v>
       </c>
       <c r="B119" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C119" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D119" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="120" spans="1:4">
@@ -4167,13 +4176,13 @@
         <v>122</v>
       </c>
       <c r="B120" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C120" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D120" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
     </row>
     <row r="121" spans="1:4">
@@ -4181,13 +4190,13 @@
         <v>123</v>
       </c>
       <c r="B121" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C121" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D121" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
     </row>
     <row r="122" spans="1:4">
@@ -4195,13 +4204,13 @@
         <v>124</v>
       </c>
       <c r="B122" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C122" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D122" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
     </row>
     <row r="123" spans="1:4">
@@ -4209,13 +4218,13 @@
         <v>125</v>
       </c>
       <c r="B123" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C123" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D123" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
     </row>
     <row r="124" spans="1:4">
@@ -4223,13 +4232,13 @@
         <v>126</v>
       </c>
       <c r="B124" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C124" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D124" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
     </row>
     <row r="125" spans="1:4">
@@ -4237,13 +4246,13 @@
         <v>127</v>
       </c>
       <c r="B125" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C125" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D125" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
     </row>
     <row r="126" spans="1:4">
@@ -4251,13 +4260,13 @@
         <v>128</v>
       </c>
       <c r="B126" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C126" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D126" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
     </row>
     <row r="127" spans="1:4">
@@ -4265,13 +4274,13 @@
         <v>129</v>
       </c>
       <c r="B127" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C127" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D127" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
     </row>
     <row r="128" spans="1:4">
@@ -4279,13 +4288,13 @@
         <v>130</v>
       </c>
       <c r="B128" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C128" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D128" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
     </row>
     <row r="129" spans="1:4">
@@ -4293,13 +4302,13 @@
         <v>131</v>
       </c>
       <c r="B129" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C129" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D129" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
     </row>
     <row r="130" spans="1:4">
@@ -4307,13 +4316,13 @@
         <v>132</v>
       </c>
       <c r="B130" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C130" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D130" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
     </row>
     <row r="131" spans="1:4">
@@ -4321,13 +4330,13 @@
         <v>133</v>
       </c>
       <c r="B131" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C131" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D131" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
     </row>
     <row r="132" spans="1:4">
@@ -4335,13 +4344,13 @@
         <v>134</v>
       </c>
       <c r="B132" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C132" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D132" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
     </row>
     <row r="133" spans="1:4">
@@ -4349,13 +4358,13 @@
         <v>135</v>
       </c>
       <c r="B133" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C133" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D133" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
     </row>
     <row r="134" spans="1:4">
@@ -4363,13 +4372,13 @@
         <v>136</v>
       </c>
       <c r="B134" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C134" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D134" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
     </row>
     <row r="135" spans="1:4">
@@ -4377,13 +4386,13 @@
         <v>137</v>
       </c>
       <c r="B135" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C135" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D135" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
     </row>
     <row r="136" spans="1:4">
@@ -4391,13 +4400,13 @@
         <v>138</v>
       </c>
       <c r="B136" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C136" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D136" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
     </row>
     <row r="137" spans="1:4">
@@ -4405,13 +4414,13 @@
         <v>139</v>
       </c>
       <c r="B137" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C137" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D137" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
     </row>
     <row r="138" spans="1:4">
@@ -4419,13 +4428,13 @@
         <v>140</v>
       </c>
       <c r="B138" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C138" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D138" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
     </row>
     <row r="139" spans="1:4">
@@ -4433,13 +4442,13 @@
         <v>141</v>
       </c>
       <c r="B139" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C139" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D139" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
     </row>
     <row r="140" spans="1:4">
@@ -4447,13 +4456,13 @@
         <v>142</v>
       </c>
       <c r="B140" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C140" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D140" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
     </row>
     <row r="141" spans="1:4">
@@ -4461,13 +4470,13 @@
         <v>143</v>
       </c>
       <c r="B141" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C141" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D141" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
     </row>
     <row r="142" spans="1:4">
@@ -4475,13 +4484,13 @@
         <v>144</v>
       </c>
       <c r="B142" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C142" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D142" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
     </row>
     <row r="143" spans="1:4">
@@ -4489,13 +4498,13 @@
         <v>145</v>
       </c>
       <c r="B143" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C143" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D143" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
     </row>
     <row r="144" spans="1:4">
@@ -4503,13 +4512,13 @@
         <v>146</v>
       </c>
       <c r="B144" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C144" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="D144" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
     </row>
     <row r="145" spans="1:4">
@@ -4517,13 +4526,13 @@
         <v>147</v>
       </c>
       <c r="B145" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C145" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D145" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
     </row>
     <row r="146" spans="1:4">
@@ -4531,13 +4540,13 @@
         <v>148</v>
       </c>
       <c r="B146" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C146" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="D146" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
     </row>
     <row r="147" spans="1:4">
@@ -4545,13 +4554,13 @@
         <v>149</v>
       </c>
       <c r="B147" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C147" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D147" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
     </row>
     <row r="148" spans="1:4">
@@ -4559,13 +4568,13 @@
         <v>150</v>
       </c>
       <c r="B148" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C148" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D148" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
     </row>
     <row r="149" spans="1:4">
@@ -4573,13 +4582,13 @@
         <v>151</v>
       </c>
       <c r="B149" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C149" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D149" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
     </row>
     <row r="150" spans="1:4">
@@ -4587,13 +4596,13 @@
         <v>152</v>
       </c>
       <c r="B150" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C150" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D150" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
     </row>
     <row r="151" spans="1:4">
@@ -4601,13 +4610,13 @@
         <v>153</v>
       </c>
       <c r="B151" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C151" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D151" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
     </row>
     <row r="152" spans="1:4">
@@ -4615,13 +4624,13 @@
         <v>154</v>
       </c>
       <c r="B152" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C152" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D152" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
     </row>
     <row r="153" spans="1:4">
@@ -4629,13 +4638,13 @@
         <v>155</v>
       </c>
       <c r="B153" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C153" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D153" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
     </row>
     <row r="154" spans="1:4">
@@ -4643,13 +4652,13 @@
         <v>156</v>
       </c>
       <c r="B154" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C154" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="D154" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
     </row>
     <row r="155" spans="1:4">
@@ -4657,13 +4666,13 @@
         <v>157</v>
       </c>
       <c r="B155" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C155" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D155" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
     </row>
     <row r="156" spans="1:4">
@@ -4671,13 +4680,13 @@
         <v>158</v>
       </c>
       <c r="B156" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C156" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D156" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
     </row>
     <row r="157" spans="1:4">
@@ -4685,13 +4694,13 @@
         <v>159</v>
       </c>
       <c r="B157" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C157" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="D157" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
     </row>
     <row r="158" spans="1:4">
@@ -4699,13 +4708,13 @@
         <v>160</v>
       </c>
       <c r="B158" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C158" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D158" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
     </row>
     <row r="159" spans="1:4">
@@ -4713,13 +4722,13 @@
         <v>161</v>
       </c>
       <c r="B159" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C159" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D159" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
     </row>
     <row r="160" spans="1:4">
@@ -4727,13 +4736,13 @@
         <v>162</v>
       </c>
       <c r="B160" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C160" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D160" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
     </row>
     <row r="161" spans="1:4">
@@ -4741,13 +4750,13 @@
         <v>163</v>
       </c>
       <c r="B161" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C161" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D161" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
     </row>
     <row r="162" spans="1:4">
@@ -4755,13 +4764,13 @@
         <v>164</v>
       </c>
       <c r="B162" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C162" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="D162" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
     </row>
     <row r="163" spans="1:4">
@@ -4769,13 +4778,13 @@
         <v>165</v>
       </c>
       <c r="B163" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C163" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D163" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
     </row>
     <row r="164" spans="1:4">
@@ -4783,13 +4792,13 @@
         <v>166</v>
       </c>
       <c r="B164" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C164" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D164" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
     </row>
     <row r="165" spans="1:4">
@@ -4797,13 +4806,13 @@
         <v>167</v>
       </c>
       <c r="B165" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C165" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D165" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
     </row>
     <row r="166" spans="1:4">
@@ -4811,13 +4820,13 @@
         <v>168</v>
       </c>
       <c r="B166" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C166" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D166" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
     </row>
     <row r="167" spans="1:4">
@@ -4825,13 +4834,13 @@
         <v>169</v>
       </c>
       <c r="B167" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C167" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D167" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
     </row>
     <row r="168" spans="1:4">
@@ -4839,13 +4848,13 @@
         <v>170</v>
       </c>
       <c r="B168" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C168" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="D168" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
     </row>
     <row r="169" spans="1:4">
@@ -4853,13 +4862,13 @@
         <v>171</v>
       </c>
       <c r="B169" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C169" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D169" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
     </row>
     <row r="170" spans="1:4">
@@ -4867,13 +4876,13 @@
         <v>172</v>
       </c>
       <c r="B170" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C170" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D170" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
     </row>
     <row r="171" spans="1:4">
@@ -4881,13 +4890,13 @@
         <v>173</v>
       </c>
       <c r="B171" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C171" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D171" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
     </row>
     <row r="172" spans="1:4">
@@ -4895,13 +4904,13 @@
         <v>174</v>
       </c>
       <c r="B172" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C172" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D172" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
     </row>
     <row r="173" spans="1:4">
@@ -4909,13 +4918,13 @@
         <v>175</v>
       </c>
       <c r="B173" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C173" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D173" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
     </row>
     <row r="174" spans="1:4">
@@ -4923,13 +4932,13 @@
         <v>176</v>
       </c>
       <c r="B174" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C174" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="D174" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
     </row>
     <row r="175" spans="1:4">
@@ -4937,13 +4946,13 @@
         <v>177</v>
       </c>
       <c r="B175" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C175" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D175" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
     </row>
     <row r="176" spans="1:4">
@@ -4951,13 +4960,13 @@
         <v>178</v>
       </c>
       <c r="B176" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C176" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D176" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
     </row>
     <row r="177" spans="1:4">
@@ -4965,13 +4974,13 @@
         <v>179</v>
       </c>
       <c r="B177" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C177" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D177" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
     </row>
     <row r="178" spans="1:4">
@@ -4979,13 +4988,13 @@
         <v>180</v>
       </c>
       <c r="B178" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C178" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D178" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
     </row>
     <row r="179" spans="1:4">
@@ -4993,13 +5002,13 @@
         <v>181</v>
       </c>
       <c r="B179" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C179" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D179" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
     </row>
     <row r="180" spans="1:4">
@@ -5007,13 +5016,13 @@
         <v>182</v>
       </c>
       <c r="B180" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C180" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D180" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
     </row>
     <row r="181" spans="1:4">
@@ -5021,13 +5030,13 @@
         <v>183</v>
       </c>
       <c r="B181" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C181" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D181" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
     </row>
     <row r="182" spans="1:4">
@@ -5035,13 +5044,13 @@
         <v>184</v>
       </c>
       <c r="B182" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C182" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D182" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
     </row>
     <row r="183" spans="1:4">
@@ -5049,13 +5058,13 @@
         <v>185</v>
       </c>
       <c r="B183" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C183" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D183" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
     </row>
     <row r="184" spans="1:4">
@@ -5063,13 +5072,13 @@
         <v>186</v>
       </c>
       <c r="B184" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C184" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D184" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
     </row>
     <row r="185" spans="1:4">
@@ -5077,13 +5086,13 @@
         <v>187</v>
       </c>
       <c r="B185" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C185" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D185" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
     </row>
     <row r="186" spans="1:4">
@@ -5091,13 +5100,13 @@
         <v>188</v>
       </c>
       <c r="B186" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C186" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="D186" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
     </row>
     <row r="187" spans="1:4">
@@ -5105,13 +5114,13 @@
         <v>189</v>
       </c>
       <c r="B187" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C187" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D187" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
     </row>
     <row r="188" spans="1:4">
@@ -5119,13 +5128,13 @@
         <v>190</v>
       </c>
       <c r="B188" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C188" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="D188" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
     </row>
     <row r="189" spans="1:4">
@@ -5133,13 +5142,13 @@
         <v>191</v>
       </c>
       <c r="B189" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C189" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="D189" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
     </row>
     <row r="190" spans="1:4">
@@ -5147,13 +5156,13 @@
         <v>192</v>
       </c>
       <c r="B190" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C190" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="D190" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
     </row>
     <row r="191" spans="1:4">
@@ -5161,13 +5170,13 @@
         <v>193</v>
       </c>
       <c r="B191" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C191" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="D191" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
     </row>
     <row r="192" spans="1:4">
@@ -5175,13 +5184,13 @@
         <v>194</v>
       </c>
       <c r="B192" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C192" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="D192" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
     </row>
     <row r="193" spans="1:4">
@@ -5189,13 +5198,13 @@
         <v>195</v>
       </c>
       <c r="B193" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C193" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="D193" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
     </row>
     <row r="194" spans="1:4">
@@ -5203,13 +5212,13 @@
         <v>196</v>
       </c>
       <c r="B194" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C194" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="D194" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
     </row>
     <row r="195" spans="1:4">
@@ -5217,13 +5226,13 @@
         <v>197</v>
       </c>
       <c r="B195" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C195" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="D195" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
     </row>
     <row r="196" spans="1:4">
@@ -5231,13 +5240,13 @@
         <v>198</v>
       </c>
       <c r="B196" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C196" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="D196" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
     </row>
     <row r="197" spans="1:4">
@@ -5245,13 +5254,13 @@
         <v>199</v>
       </c>
       <c r="B197" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C197" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D197" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
     </row>
     <row r="198" spans="1:4">
@@ -5259,13 +5268,13 @@
         <v>200</v>
       </c>
       <c r="B198" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C198" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D198" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
     </row>
     <row r="199" spans="1:4">
@@ -5273,13 +5282,13 @@
         <v>201</v>
       </c>
       <c r="B199" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C199" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="D199" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
     </row>
     <row r="200" spans="1:4">
@@ -5287,13 +5296,13 @@
         <v>202</v>
       </c>
       <c r="B200" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C200" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D200" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
     </row>
     <row r="201" spans="1:4">
@@ -5301,13 +5310,13 @@
         <v>203</v>
       </c>
       <c r="B201" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C201" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D201" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
     </row>
     <row r="202" spans="1:4">
@@ -5315,13 +5324,13 @@
         <v>204</v>
       </c>
       <c r="B202" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C202" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D202" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
     </row>
     <row r="203" spans="1:4">
@@ -5329,13 +5338,13 @@
         <v>205</v>
       </c>
       <c r="B203" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C203" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="D203" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
     </row>
     <row r="204" spans="1:4">
@@ -5343,13 +5352,13 @@
         <v>206</v>
       </c>
       <c r="B204" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C204" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D204" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
     </row>
     <row r="205" spans="1:4">
@@ -5357,13 +5366,13 @@
         <v>207</v>
       </c>
       <c r="B205" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C205" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D205" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
     </row>
     <row r="206" spans="1:4">
@@ -5371,13 +5380,13 @@
         <v>208</v>
       </c>
       <c r="B206" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C206" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D206" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
     </row>
     <row r="207" spans="1:4">
@@ -5385,13 +5394,13 @@
         <v>209</v>
       </c>
       <c r="B207" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C207" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D207" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
     </row>
     <row r="208" spans="1:4">
@@ -5399,13 +5408,13 @@
         <v>210</v>
       </c>
       <c r="B208" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C208" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D208" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
     </row>
     <row r="209" spans="1:4">
@@ -5413,13 +5422,13 @@
         <v>211</v>
       </c>
       <c r="B209" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C209" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D209" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
     </row>
     <row r="210" spans="1:4">
@@ -5427,13 +5436,13 @@
         <v>212</v>
       </c>
       <c r="B210" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C210" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D210" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
     </row>
     <row r="211" spans="1:4">
@@ -5441,13 +5450,13 @@
         <v>213</v>
       </c>
       <c r="B211" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C211" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D211" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
     </row>
     <row r="212" spans="1:4">
@@ -5455,13 +5464,13 @@
         <v>214</v>
       </c>
       <c r="B212" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C212" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D212" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
     </row>
     <row r="213" spans="1:4">
@@ -5469,13 +5478,13 @@
         <v>215</v>
       </c>
       <c r="B213" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C213" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D213" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
     </row>
     <row r="214" spans="1:4">
@@ -5483,13 +5492,13 @@
         <v>216</v>
       </c>
       <c r="B214" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="C214" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D214" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
     </row>
     <row r="215" spans="1:4">
@@ -5497,13 +5506,13 @@
         <v>217</v>
       </c>
       <c r="B215" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C215" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="D215" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
     </row>
     <row r="216" spans="1:4">
@@ -5511,13 +5520,13 @@
         <v>218</v>
       </c>
       <c r="B216" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C216" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="D216" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
     </row>
     <row r="217" spans="1:4">
@@ -5525,13 +5534,13 @@
         <v>219</v>
       </c>
       <c r="B217" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C217" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D217" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
     </row>
     <row r="218" spans="1:4">
@@ -5539,13 +5548,13 @@
         <v>220</v>
       </c>
       <c r="B218" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C218" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="D218" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
     </row>
     <row r="219" spans="1:4">
@@ -5553,13 +5562,13 @@
         <v>221</v>
       </c>
       <c r="B219" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C219" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D219" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
     </row>
     <row r="220" spans="1:4">
@@ -5567,13 +5576,13 @@
         <v>222</v>
       </c>
       <c r="B220" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C220" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D220" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
     </row>
     <row r="221" spans="1:4">
@@ -5581,13 +5590,13 @@
         <v>223</v>
       </c>
       <c r="B221" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C221" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="D221" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
     </row>
     <row r="222" spans="1:4">
@@ -5595,13 +5604,13 @@
         <v>224</v>
       </c>
       <c r="B222" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C222" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D222" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
     </row>
     <row r="223" spans="1:4">
@@ -5609,13 +5618,13 @@
         <v>225</v>
       </c>
       <c r="B223" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C223" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="D223" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
     </row>
     <row r="224" spans="1:4">
@@ -5623,13 +5632,13 @@
         <v>226</v>
       </c>
       <c r="B224" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C224" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D224" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
     </row>
     <row r="225" spans="1:4">
@@ -5637,13 +5646,13 @@
         <v>227</v>
       </c>
       <c r="B225" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="C225" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="D225" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
     </row>
     <row r="226" spans="1:4">
@@ -5651,13 +5660,13 @@
         <v>228</v>
       </c>
       <c r="B226" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C226" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="D226" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
     </row>
     <row r="227" spans="1:4">
@@ -5665,13 +5674,13 @@
         <v>229</v>
       </c>
       <c r="B227" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C227" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D227" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
     </row>
     <row r="228" spans="1:4">
@@ -5679,13 +5688,13 @@
         <v>230</v>
       </c>
       <c r="B228" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="C228" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D228" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
     </row>
     <row r="229" spans="1:4">
@@ -5693,13 +5702,13 @@
         <v>231</v>
       </c>
       <c r="B229" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C229" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="D229" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
     <row r="230" spans="1:4">
@@ -5707,13 +5716,13 @@
         <v>232</v>
       </c>
       <c r="B230" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="C230" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D230" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
     </row>
     <row r="231" spans="1:4">
@@ -5721,13 +5730,13 @@
         <v>233</v>
       </c>
       <c r="B231" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C231" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="D231" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
     </row>
     <row r="232" spans="1:4">
@@ -5735,13 +5744,13 @@
         <v>234</v>
       </c>
       <c r="B232" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C232" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="D232" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="233" spans="1:4">
@@ -5749,13 +5758,13 @@
         <v>235</v>
       </c>
       <c r="B233" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C233" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D233" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
     </row>
     <row r="234" spans="1:4">
@@ -5769,7 +5778,7 @@
         <v>236</v>
       </c>
       <c r="D234" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
     </row>
     <row r="235" spans="1:4">
@@ -5783,7 +5792,7 @@
         <v>237</v>
       </c>
       <c r="D235" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
     </row>
     <row r="236" spans="1:4">
@@ -5791,13 +5800,13 @@
         <v>238</v>
       </c>
       <c r="B236" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C236" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="D236" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
     </row>
     <row r="237" spans="1:4">
@@ -5805,13 +5814,13 @@
         <v>239</v>
       </c>
       <c r="B237" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C237" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D237" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
     </row>
     <row r="238" spans="1:4">
@@ -5819,13 +5828,13 @@
         <v>240</v>
       </c>
       <c r="B238" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C238" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="D238" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
     </row>
     <row r="239" spans="1:4">
@@ -5833,13 +5842,27 @@
         <v>241</v>
       </c>
       <c r="B239" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C239" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="D239" t="s">
-        <v>715</v>
+        <v>717</v>
+      </c>
+    </row>
+    <row r="240" spans="1:4">
+      <c r="A240" t="s">
+        <v>242</v>
+      </c>
+      <c r="B240" t="s">
+        <v>479</v>
+      </c>
+      <c r="C240" t="s">
+        <v>479</v>
+      </c>
+      <c r="D240" t="s">
+        <v>718</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cập nhật mapping và lịch sử spam chi tiết kho khô
</commit_message>
<xml_diff>
--- a/SPAM_PHIEU_CHUYEN/CHI TIẾT MÁT/Danh sách Siêu thị.xlsx
+++ b/SPAM_PHIEU_CHUYEN/CHI TIẾT MÁT/Danh sách Siêu thị.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="719">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="964" uniqueCount="722">
   <si>
     <t>Tên Siêu thị</t>
   </si>
@@ -745,6 +745,9 @@
     <t>KFM_HCM_Q08 - A6-7 Block A Diamond Lotus Riverside</t>
   </si>
   <si>
+    <t>KFM_HCM_BCH - CA.01 Đường 19 KDC Phong Phú 4</t>
+  </si>
+  <si>
     <t>A101</t>
   </si>
   <si>
@@ -1456,6 +1459,9 @@
     <t>A243</t>
   </si>
   <si>
+    <t>A216</t>
+  </si>
+  <si>
     <t>-4970846623</t>
   </si>
   <si>
@@ -2171,6 +2177,9 @@
   </si>
   <si>
     <t>-1003932619661</t>
+  </si>
+  <si>
+    <t>-1004361944433</t>
   </si>
 </sst>
 </file>
@@ -2502,7 +2511,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D240"/>
+  <dimension ref="A1:D241"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -2524,13 +2533,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D2" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2538,13 +2547,13 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D3" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2552,13 +2561,13 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C4" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D4" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2566,13 +2575,13 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C5" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D5" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2580,13 +2589,13 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D6" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2594,13 +2603,13 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C7" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D7" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2608,13 +2617,13 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C8" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D8" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2622,13 +2631,13 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C9" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D9" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2636,13 +2645,13 @@
         <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D10" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2650,13 +2659,13 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C11" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D11" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2664,13 +2673,13 @@
         <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C12" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D12" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -2678,13 +2687,13 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C13" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D13" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -2692,13 +2701,13 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C14" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D14" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -2706,13 +2715,13 @@
         <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C15" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D15" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -2720,13 +2729,13 @@
         <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C16" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D16" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -2734,13 +2743,13 @@
         <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C17" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D17" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2748,13 +2757,13 @@
         <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C18" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D18" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -2762,13 +2771,13 @@
         <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C19" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D19" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -2776,13 +2785,13 @@
         <v>22</v>
       </c>
       <c r="B20" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C20" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D20" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -2790,13 +2799,13 @@
         <v>23</v>
       </c>
       <c r="B21" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C21" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D21" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -2804,13 +2813,13 @@
         <v>24</v>
       </c>
       <c r="B22" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C22" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D22" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -2818,13 +2827,13 @@
         <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C23" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D23" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -2832,13 +2841,13 @@
         <v>26</v>
       </c>
       <c r="B24" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C24" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D24" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -2846,13 +2855,13 @@
         <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C25" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D25" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -2860,13 +2869,13 @@
         <v>28</v>
       </c>
       <c r="B26" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C26" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D26" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -2874,13 +2883,13 @@
         <v>29</v>
       </c>
       <c r="B27" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C27" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D27" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -2888,13 +2897,13 @@
         <v>30</v>
       </c>
       <c r="B28" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C28" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D28" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -2902,13 +2911,13 @@
         <v>31</v>
       </c>
       <c r="B29" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C29" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D29" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -2916,13 +2925,13 @@
         <v>32</v>
       </c>
       <c r="B30" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C30" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D30" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -2930,13 +2939,13 @@
         <v>33</v>
       </c>
       <c r="B31" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C31" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D31" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -2944,13 +2953,13 @@
         <v>34</v>
       </c>
       <c r="B32" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C32" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D32" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -2958,13 +2967,13 @@
         <v>35</v>
       </c>
       <c r="B33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D33" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -2972,13 +2981,13 @@
         <v>36</v>
       </c>
       <c r="B34" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C34" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D34" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -2986,13 +2995,13 @@
         <v>37</v>
       </c>
       <c r="B35" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C35" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D35" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -3000,13 +3009,13 @@
         <v>38</v>
       </c>
       <c r="B36" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C36" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D36" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -3014,13 +3023,13 @@
         <v>39</v>
       </c>
       <c r="B37" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C37" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D37" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -3028,13 +3037,13 @@
         <v>40</v>
       </c>
       <c r="B38" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C38" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D38" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -3042,13 +3051,13 @@
         <v>41</v>
       </c>
       <c r="B39" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C39" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D39" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -3056,13 +3065,13 @@
         <v>42</v>
       </c>
       <c r="B40" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C40" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D40" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -3070,13 +3079,13 @@
         <v>43</v>
       </c>
       <c r="B41" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C41" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D41" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -3084,13 +3093,13 @@
         <v>44</v>
       </c>
       <c r="B42" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C42" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D42" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -3098,13 +3107,13 @@
         <v>45</v>
       </c>
       <c r="B43" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C43" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D43" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -3112,13 +3121,13 @@
         <v>46</v>
       </c>
       <c r="B44" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C44" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D44" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -3126,13 +3135,13 @@
         <v>47</v>
       </c>
       <c r="B45" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C45" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D45" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -3140,13 +3149,13 @@
         <v>48</v>
       </c>
       <c r="B46" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C46" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D46" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -3154,13 +3163,13 @@
         <v>49</v>
       </c>
       <c r="B47" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C47" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D47" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -3168,13 +3177,13 @@
         <v>50</v>
       </c>
       <c r="B48" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C48" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D48" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -3182,13 +3191,13 @@
         <v>51</v>
       </c>
       <c r="B49" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C49" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D49" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -3196,13 +3205,13 @@
         <v>52</v>
       </c>
       <c r="B50" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C50" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D50" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -3210,13 +3219,13 @@
         <v>53</v>
       </c>
       <c r="B51" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C51" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D51" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -3224,13 +3233,13 @@
         <v>54</v>
       </c>
       <c r="B52" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C52" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D52" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -3238,13 +3247,13 @@
         <v>55</v>
       </c>
       <c r="B53" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C53" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D53" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -3252,13 +3261,13 @@
         <v>56</v>
       </c>
       <c r="B54" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C54" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D54" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -3266,13 +3275,13 @@
         <v>57</v>
       </c>
       <c r="B55" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C55" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D55" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -3280,13 +3289,13 @@
         <v>58</v>
       </c>
       <c r="B56" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C56" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D56" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -3294,13 +3303,13 @@
         <v>59</v>
       </c>
       <c r="B57" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C57" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D57" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -3308,13 +3317,13 @@
         <v>60</v>
       </c>
       <c r="B58" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C58" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D58" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -3322,13 +3331,13 @@
         <v>61</v>
       </c>
       <c r="B59" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C59" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D59" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -3336,13 +3345,13 @@
         <v>62</v>
       </c>
       <c r="B60" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C60" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D60" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -3350,13 +3359,13 @@
         <v>63</v>
       </c>
       <c r="B61" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C61" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D61" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -3364,13 +3373,13 @@
         <v>64</v>
       </c>
       <c r="B62" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C62" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D62" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -3378,13 +3387,13 @@
         <v>65</v>
       </c>
       <c r="B63" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C63" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D63" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -3392,13 +3401,13 @@
         <v>66</v>
       </c>
       <c r="B64" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C64" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D64" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -3406,13 +3415,13 @@
         <v>67</v>
       </c>
       <c r="B65" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C65" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D65" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -3420,13 +3429,13 @@
         <v>68</v>
       </c>
       <c r="B66" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C66" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D66" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -3434,13 +3443,13 @@
         <v>69</v>
       </c>
       <c r="B67" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C67" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D67" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -3448,13 +3457,13 @@
         <v>70</v>
       </c>
       <c r="B68" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C68" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D68" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -3462,13 +3471,13 @@
         <v>71</v>
       </c>
       <c r="B69" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C69" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D69" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -3476,13 +3485,13 @@
         <v>72</v>
       </c>
       <c r="B70" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C70" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D70" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -3490,13 +3499,13 @@
         <v>73</v>
       </c>
       <c r="B71" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C71" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D71" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -3504,13 +3513,13 @@
         <v>74</v>
       </c>
       <c r="B72" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C72" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D72" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -3518,13 +3527,13 @@
         <v>75</v>
       </c>
       <c r="B73" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C73" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D73" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -3532,13 +3541,13 @@
         <v>76</v>
       </c>
       <c r="B74" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C74" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D74" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -3546,13 +3555,13 @@
         <v>77</v>
       </c>
       <c r="B75" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C75" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D75" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -3560,13 +3569,13 @@
         <v>78</v>
       </c>
       <c r="B76" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C76" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="D76" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -3574,13 +3583,13 @@
         <v>79</v>
       </c>
       <c r="B77" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C77" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D77" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -3588,13 +3597,13 @@
         <v>80</v>
       </c>
       <c r="B78" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C78" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D78" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -3602,13 +3611,13 @@
         <v>81</v>
       </c>
       <c r="B79" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C79" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D79" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -3616,13 +3625,13 @@
         <v>82</v>
       </c>
       <c r="B80" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C80" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D80" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -3630,13 +3639,13 @@
         <v>83</v>
       </c>
       <c r="B81" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C81" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D81" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
     </row>
     <row r="82" spans="1:4">
@@ -3644,13 +3653,13 @@
         <v>84</v>
       </c>
       <c r="B82" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C82" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D82" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -3658,13 +3667,13 @@
         <v>85</v>
       </c>
       <c r="B83" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C83" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D83" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -3672,13 +3681,13 @@
         <v>86</v>
       </c>
       <c r="B84" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C84" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D84" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -3686,13 +3695,13 @@
         <v>87</v>
       </c>
       <c r="B85" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C85" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D85" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
     </row>
     <row r="86" spans="1:4">
@@ -3700,13 +3709,13 @@
         <v>88</v>
       </c>
       <c r="B86" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C86" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D86" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
     </row>
     <row r="87" spans="1:4">
@@ -3714,13 +3723,13 @@
         <v>89</v>
       </c>
       <c r="B87" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C87" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D87" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
     </row>
     <row r="88" spans="1:4">
@@ -3728,13 +3737,13 @@
         <v>90</v>
       </c>
       <c r="B88" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C88" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D88" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -3742,13 +3751,13 @@
         <v>91</v>
       </c>
       <c r="B89" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C89" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D89" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
     </row>
     <row r="90" spans="1:4">
@@ -3756,13 +3765,13 @@
         <v>92</v>
       </c>
       <c r="B90" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C90" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D90" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -3770,13 +3779,13 @@
         <v>93</v>
       </c>
       <c r="B91" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C91" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D91" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
     </row>
     <row r="92" spans="1:4">
@@ -3784,13 +3793,13 @@
         <v>94</v>
       </c>
       <c r="B92" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C92" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D92" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="93" spans="1:4">
@@ -3798,13 +3807,13 @@
         <v>95</v>
       </c>
       <c r="B93" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C93" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D93" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
     </row>
     <row r="94" spans="1:4">
@@ -3812,13 +3821,13 @@
         <v>96</v>
       </c>
       <c r="B94" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C94" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D94" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
     </row>
     <row r="95" spans="1:4">
@@ -3826,13 +3835,13 @@
         <v>97</v>
       </c>
       <c r="B95" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C95" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D95" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
     </row>
     <row r="96" spans="1:4">
@@ -3840,13 +3849,13 @@
         <v>98</v>
       </c>
       <c r="B96" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C96" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D96" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
     </row>
     <row r="97" spans="1:4">
@@ -3854,13 +3863,13 @@
         <v>99</v>
       </c>
       <c r="B97" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C97" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D97" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
     </row>
     <row r="98" spans="1:4">
@@ -3868,13 +3877,13 @@
         <v>100</v>
       </c>
       <c r="B98" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C98" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D98" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
     </row>
     <row r="99" spans="1:4">
@@ -3882,13 +3891,13 @@
         <v>101</v>
       </c>
       <c r="B99" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C99" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D99" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
     </row>
     <row r="100" spans="1:4">
@@ -3896,13 +3905,13 @@
         <v>102</v>
       </c>
       <c r="B100" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C100" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D100" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
     </row>
     <row r="101" spans="1:4">
@@ -3910,13 +3919,13 @@
         <v>103</v>
       </c>
       <c r="B101" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C101" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D101" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
     <row r="102" spans="1:4">
@@ -3924,13 +3933,13 @@
         <v>104</v>
       </c>
       <c r="B102" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C102" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D102" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
     </row>
     <row r="103" spans="1:4">
@@ -3938,13 +3947,13 @@
         <v>105</v>
       </c>
       <c r="B103" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C103" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D103" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
     </row>
     <row r="104" spans="1:4">
@@ -3952,13 +3961,13 @@
         <v>106</v>
       </c>
       <c r="B104" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C104" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D104" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
     </row>
     <row r="105" spans="1:4">
@@ -3966,13 +3975,13 @@
         <v>107</v>
       </c>
       <c r="B105" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C105" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D105" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
     </row>
     <row r="106" spans="1:4">
@@ -3980,13 +3989,13 @@
         <v>108</v>
       </c>
       <c r="B106" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C106" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D106" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
     </row>
     <row r="107" spans="1:4">
@@ -3994,13 +4003,13 @@
         <v>109</v>
       </c>
       <c r="B107" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C107" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D107" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="108" spans="1:4">
@@ -4008,13 +4017,13 @@
         <v>110</v>
       </c>
       <c r="B108" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C108" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="D108" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
     </row>
     <row r="109" spans="1:4">
@@ -4022,13 +4031,13 @@
         <v>111</v>
       </c>
       <c r="B109" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C109" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D109" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
     </row>
     <row r="110" spans="1:4">
@@ -4036,13 +4045,13 @@
         <v>112</v>
       </c>
       <c r="B110" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C110" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D110" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
     </row>
     <row r="111" spans="1:4">
@@ -4050,13 +4059,13 @@
         <v>113</v>
       </c>
       <c r="B111" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C111" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D111" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
     </row>
     <row r="112" spans="1:4">
@@ -4064,13 +4073,13 @@
         <v>114</v>
       </c>
       <c r="B112" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C112" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D112" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
     </row>
     <row r="113" spans="1:4">
@@ -4078,13 +4087,13 @@
         <v>115</v>
       </c>
       <c r="B113" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C113" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D113" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
     </row>
     <row r="114" spans="1:4">
@@ -4092,13 +4101,13 @@
         <v>116</v>
       </c>
       <c r="B114" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C114" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D114" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
     </row>
     <row r="115" spans="1:4">
@@ -4106,13 +4115,13 @@
         <v>117</v>
       </c>
       <c r="B115" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C115" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D115" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
     </row>
     <row r="116" spans="1:4">
@@ -4120,13 +4129,13 @@
         <v>118</v>
       </c>
       <c r="B116" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C116" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D116" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
     </row>
     <row r="117" spans="1:4">
@@ -4134,13 +4143,13 @@
         <v>119</v>
       </c>
       <c r="B117" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C117" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D117" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="118" spans="1:4">
@@ -4148,13 +4157,13 @@
         <v>120</v>
       </c>
       <c r="B118" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C118" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D118" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
     </row>
     <row r="119" spans="1:4">
@@ -4162,13 +4171,13 @@
         <v>121</v>
       </c>
       <c r="B119" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C119" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D119" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
     </row>
     <row r="120" spans="1:4">
@@ -4176,13 +4185,13 @@
         <v>122</v>
       </c>
       <c r="B120" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C120" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D120" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
     </row>
     <row r="121" spans="1:4">
@@ -4190,13 +4199,13 @@
         <v>123</v>
       </c>
       <c r="B121" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C121" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="D121" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
     </row>
     <row r="122" spans="1:4">
@@ -4204,13 +4213,13 @@
         <v>124</v>
       </c>
       <c r="B122" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C122" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D122" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
     </row>
     <row r="123" spans="1:4">
@@ -4218,13 +4227,13 @@
         <v>125</v>
       </c>
       <c r="B123" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C123" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D123" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
     </row>
     <row r="124" spans="1:4">
@@ -4232,13 +4241,13 @@
         <v>126</v>
       </c>
       <c r="B124" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C124" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D124" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
     </row>
     <row r="125" spans="1:4">
@@ -4246,13 +4255,13 @@
         <v>127</v>
       </c>
       <c r="B125" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C125" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D125" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
     </row>
     <row r="126" spans="1:4">
@@ -4260,13 +4269,13 @@
         <v>128</v>
       </c>
       <c r="B126" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C126" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D126" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
     </row>
     <row r="127" spans="1:4">
@@ -4274,13 +4283,13 @@
         <v>129</v>
       </c>
       <c r="B127" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C127" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D127" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
     </row>
     <row r="128" spans="1:4">
@@ -4288,13 +4297,13 @@
         <v>130</v>
       </c>
       <c r="B128" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C128" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D128" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
     </row>
     <row r="129" spans="1:4">
@@ -4302,13 +4311,13 @@
         <v>131</v>
       </c>
       <c r="B129" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C129" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D129" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
     </row>
     <row r="130" spans="1:4">
@@ -4316,13 +4325,13 @@
         <v>132</v>
       </c>
       <c r="B130" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C130" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D130" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
     </row>
     <row r="131" spans="1:4">
@@ -4330,13 +4339,13 @@
         <v>133</v>
       </c>
       <c r="B131" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C131" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D131" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
     </row>
     <row r="132" spans="1:4">
@@ -4344,13 +4353,13 @@
         <v>134</v>
       </c>
       <c r="B132" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C132" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D132" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
     </row>
     <row r="133" spans="1:4">
@@ -4358,13 +4367,13 @@
         <v>135</v>
       </c>
       <c r="B133" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C133" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D133" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
     </row>
     <row r="134" spans="1:4">
@@ -4372,13 +4381,13 @@
         <v>136</v>
       </c>
       <c r="B134" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C134" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D134" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
     </row>
     <row r="135" spans="1:4">
@@ -4386,13 +4395,13 @@
         <v>137</v>
       </c>
       <c r="B135" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C135" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D135" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
     </row>
     <row r="136" spans="1:4">
@@ -4400,13 +4409,13 @@
         <v>138</v>
       </c>
       <c r="B136" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C136" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D136" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
     </row>
     <row r="137" spans="1:4">
@@ -4414,13 +4423,13 @@
         <v>139</v>
       </c>
       <c r="B137" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C137" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D137" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
     </row>
     <row r="138" spans="1:4">
@@ -4428,13 +4437,13 @@
         <v>140</v>
       </c>
       <c r="B138" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C138" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D138" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
     </row>
     <row r="139" spans="1:4">
@@ -4442,13 +4451,13 @@
         <v>141</v>
       </c>
       <c r="B139" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C139" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D139" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
     </row>
     <row r="140" spans="1:4">
@@ -4456,13 +4465,13 @@
         <v>142</v>
       </c>
       <c r="B140" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C140" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D140" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
     </row>
     <row r="141" spans="1:4">
@@ -4470,13 +4479,13 @@
         <v>143</v>
       </c>
       <c r="B141" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C141" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D141" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
     </row>
     <row r="142" spans="1:4">
@@ -4484,13 +4493,13 @@
         <v>144</v>
       </c>
       <c r="B142" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C142" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D142" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
     </row>
     <row r="143" spans="1:4">
@@ -4498,13 +4507,13 @@
         <v>145</v>
       </c>
       <c r="B143" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C143" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="D143" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
     </row>
     <row r="144" spans="1:4">
@@ -4512,13 +4521,13 @@
         <v>146</v>
       </c>
       <c r="B144" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C144" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D144" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
     </row>
     <row r="145" spans="1:4">
@@ -4526,13 +4535,13 @@
         <v>147</v>
       </c>
       <c r="B145" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C145" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="D145" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
     </row>
     <row r="146" spans="1:4">
@@ -4540,13 +4549,13 @@
         <v>148</v>
       </c>
       <c r="B146" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C146" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D146" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
     </row>
     <row r="147" spans="1:4">
@@ -4554,13 +4563,13 @@
         <v>149</v>
       </c>
       <c r="B147" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C147" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D147" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
     </row>
     <row r="148" spans="1:4">
@@ -4568,13 +4577,13 @@
         <v>150</v>
       </c>
       <c r="B148" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C148" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D148" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
     </row>
     <row r="149" spans="1:4">
@@ -4582,13 +4591,13 @@
         <v>151</v>
       </c>
       <c r="B149" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C149" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D149" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
     </row>
     <row r="150" spans="1:4">
@@ -4596,13 +4605,13 @@
         <v>152</v>
       </c>
       <c r="B150" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C150" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D150" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
     </row>
     <row r="151" spans="1:4">
@@ -4610,13 +4619,13 @@
         <v>153</v>
       </c>
       <c r="B151" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C151" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D151" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
     </row>
     <row r="152" spans="1:4">
@@ -4624,13 +4633,13 @@
         <v>154</v>
       </c>
       <c r="B152" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C152" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D152" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
     </row>
     <row r="153" spans="1:4">
@@ -4638,13 +4647,13 @@
         <v>155</v>
       </c>
       <c r="B153" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C153" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="D153" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
     </row>
     <row r="154" spans="1:4">
@@ -4652,13 +4661,13 @@
         <v>156</v>
       </c>
       <c r="B154" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C154" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D154" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
     </row>
     <row r="155" spans="1:4">
@@ -4666,13 +4675,13 @@
         <v>157</v>
       </c>
       <c r="B155" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C155" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D155" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
     </row>
     <row r="156" spans="1:4">
@@ -4680,13 +4689,13 @@
         <v>158</v>
       </c>
       <c r="B156" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C156" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="D156" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
     </row>
     <row r="157" spans="1:4">
@@ -4694,13 +4703,13 @@
         <v>159</v>
       </c>
       <c r="B157" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C157" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D157" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
     </row>
     <row r="158" spans="1:4">
@@ -4708,13 +4717,13 @@
         <v>160</v>
       </c>
       <c r="B158" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C158" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D158" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
     </row>
     <row r="159" spans="1:4">
@@ -4722,13 +4731,13 @@
         <v>161</v>
       </c>
       <c r="B159" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C159" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D159" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
     </row>
     <row r="160" spans="1:4">
@@ -4736,13 +4745,13 @@
         <v>162</v>
       </c>
       <c r="B160" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C160" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D160" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
     </row>
     <row r="161" spans="1:4">
@@ -4750,13 +4759,13 @@
         <v>163</v>
       </c>
       <c r="B161" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C161" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="D161" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
     </row>
     <row r="162" spans="1:4">
@@ -4764,13 +4773,13 @@
         <v>164</v>
       </c>
       <c r="B162" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C162" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D162" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
     </row>
     <row r="163" spans="1:4">
@@ -4778,13 +4787,13 @@
         <v>165</v>
       </c>
       <c r="B163" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C163" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D163" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
     </row>
     <row r="164" spans="1:4">
@@ -4792,13 +4801,13 @@
         <v>166</v>
       </c>
       <c r="B164" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C164" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D164" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
     </row>
     <row r="165" spans="1:4">
@@ -4806,13 +4815,13 @@
         <v>167</v>
       </c>
       <c r="B165" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C165" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D165" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
     </row>
     <row r="166" spans="1:4">
@@ -4820,13 +4829,13 @@
         <v>168</v>
       </c>
       <c r="B166" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C166" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D166" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
     </row>
     <row r="167" spans="1:4">
@@ -4834,13 +4843,13 @@
         <v>169</v>
       </c>
       <c r="B167" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C167" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="D167" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
     </row>
     <row r="168" spans="1:4">
@@ -4848,13 +4857,13 @@
         <v>170</v>
       </c>
       <c r="B168" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C168" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D168" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
     </row>
     <row r="169" spans="1:4">
@@ -4862,13 +4871,13 @@
         <v>171</v>
       </c>
       <c r="B169" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C169" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D169" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
     </row>
     <row r="170" spans="1:4">
@@ -4876,13 +4885,13 @@
         <v>172</v>
       </c>
       <c r="B170" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C170" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D170" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
     </row>
     <row r="171" spans="1:4">
@@ -4890,13 +4899,13 @@
         <v>173</v>
       </c>
       <c r="B171" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C171" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D171" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
     </row>
     <row r="172" spans="1:4">
@@ -4904,13 +4913,13 @@
         <v>174</v>
       </c>
       <c r="B172" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C172" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D172" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
     </row>
     <row r="173" spans="1:4">
@@ -4918,13 +4927,13 @@
         <v>175</v>
       </c>
       <c r="B173" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C173" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="D173" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
     </row>
     <row r="174" spans="1:4">
@@ -4932,13 +4941,13 @@
         <v>176</v>
       </c>
       <c r="B174" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C174" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D174" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
     </row>
     <row r="175" spans="1:4">
@@ -4946,13 +4955,13 @@
         <v>177</v>
       </c>
       <c r="B175" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="C175" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D175" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
     </row>
     <row r="176" spans="1:4">
@@ -4960,13 +4969,13 @@
         <v>178</v>
       </c>
       <c r="B176" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C176" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D176" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
     </row>
     <row r="177" spans="1:4">
@@ -4974,13 +4983,13 @@
         <v>179</v>
       </c>
       <c r="B177" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C177" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="D177" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
     </row>
     <row r="178" spans="1:4">
@@ -4988,13 +4997,13 @@
         <v>180</v>
       </c>
       <c r="B178" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C178" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D178" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
     </row>
     <row r="179" spans="1:4">
@@ -5002,13 +5011,13 @@
         <v>181</v>
       </c>
       <c r="B179" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="C179" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D179" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
     </row>
     <row r="180" spans="1:4">
@@ -5016,13 +5025,13 @@
         <v>182</v>
       </c>
       <c r="B180" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C180" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D180" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
     </row>
     <row r="181" spans="1:4">
@@ -5030,13 +5039,13 @@
         <v>183</v>
       </c>
       <c r="B181" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C181" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="D181" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
     </row>
     <row r="182" spans="1:4">
@@ -5044,13 +5053,13 @@
         <v>184</v>
       </c>
       <c r="B182" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C182" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D182" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
     </row>
     <row r="183" spans="1:4">
@@ -5058,13 +5067,13 @@
         <v>185</v>
       </c>
       <c r="B183" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C183" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D183" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
     </row>
     <row r="184" spans="1:4">
@@ -5072,13 +5081,13 @@
         <v>186</v>
       </c>
       <c r="B184" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C184" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D184" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
     </row>
     <row r="185" spans="1:4">
@@ -5086,13 +5095,13 @@
         <v>187</v>
       </c>
       <c r="B185" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C185" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="D185" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
     </row>
     <row r="186" spans="1:4">
@@ -5100,13 +5109,13 @@
         <v>188</v>
       </c>
       <c r="B186" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C186" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D186" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
     </row>
     <row r="187" spans="1:4">
@@ -5114,13 +5123,13 @@
         <v>189</v>
       </c>
       <c r="B187" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="C187" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="D187" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
     </row>
     <row r="188" spans="1:4">
@@ -5128,13 +5137,13 @@
         <v>190</v>
       </c>
       <c r="B188" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="C188" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="D188" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
     </row>
     <row r="189" spans="1:4">
@@ -5142,13 +5151,13 @@
         <v>191</v>
       </c>
       <c r="B189" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C189" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="D189" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
     </row>
     <row r="190" spans="1:4">
@@ -5156,13 +5165,13 @@
         <v>192</v>
       </c>
       <c r="B190" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C190" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="D190" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
     </row>
     <row r="191" spans="1:4">
@@ -5170,13 +5179,13 @@
         <v>193</v>
       </c>
       <c r="B191" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C191" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="D191" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
     </row>
     <row r="192" spans="1:4">
@@ -5184,13 +5193,13 @@
         <v>194</v>
       </c>
       <c r="B192" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C192" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="D192" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
     </row>
     <row r="193" spans="1:4">
@@ -5198,13 +5207,13 @@
         <v>195</v>
       </c>
       <c r="B193" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="C193" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="D193" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
     </row>
     <row r="194" spans="1:4">
@@ -5212,13 +5221,13 @@
         <v>196</v>
       </c>
       <c r="B194" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C194" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="D194" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
     </row>
     <row r="195" spans="1:4">
@@ -5226,13 +5235,13 @@
         <v>197</v>
       </c>
       <c r="B195" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="C195" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="D195" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
     </row>
     <row r="196" spans="1:4">
@@ -5240,13 +5249,13 @@
         <v>198</v>
       </c>
       <c r="B196" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="C196" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D196" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
     </row>
     <row r="197" spans="1:4">
@@ -5254,13 +5263,13 @@
         <v>199</v>
       </c>
       <c r="B197" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C197" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="D197" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
     </row>
     <row r="198" spans="1:4">
@@ -5268,13 +5277,13 @@
         <v>200</v>
       </c>
       <c r="B198" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C198" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="D198" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
     </row>
     <row r="199" spans="1:4">
@@ -5282,13 +5291,13 @@
         <v>201</v>
       </c>
       <c r="B199" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C199" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D199" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
     </row>
     <row r="200" spans="1:4">
@@ -5296,13 +5305,13 @@
         <v>202</v>
       </c>
       <c r="B200" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C200" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D200" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
     </row>
     <row r="201" spans="1:4">
@@ -5310,13 +5319,13 @@
         <v>203</v>
       </c>
       <c r="B201" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C201" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D201" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
     </row>
     <row r="202" spans="1:4">
@@ -5324,13 +5333,13 @@
         <v>204</v>
       </c>
       <c r="B202" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C202" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="D202" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
     </row>
     <row r="203" spans="1:4">
@@ -5338,13 +5347,13 @@
         <v>205</v>
       </c>
       <c r="B203" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C203" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D203" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
     </row>
     <row r="204" spans="1:4">
@@ -5352,13 +5361,13 @@
         <v>206</v>
       </c>
       <c r="B204" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C204" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D204" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
     </row>
     <row r="205" spans="1:4">
@@ -5366,13 +5375,13 @@
         <v>207</v>
       </c>
       <c r="B205" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="C205" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D205" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
     </row>
     <row r="206" spans="1:4">
@@ -5380,13 +5389,13 @@
         <v>208</v>
       </c>
       <c r="B206" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C206" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D206" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
     </row>
     <row r="207" spans="1:4">
@@ -5394,13 +5403,13 @@
         <v>209</v>
       </c>
       <c r="B207" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C207" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="D207" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
     </row>
     <row r="208" spans="1:4">
@@ -5408,13 +5417,13 @@
         <v>210</v>
       </c>
       <c r="B208" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="C208" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D208" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
     </row>
     <row r="209" spans="1:4">
@@ -5422,13 +5431,13 @@
         <v>211</v>
       </c>
       <c r="B209" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C209" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D209" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
     </row>
     <row r="210" spans="1:4">
@@ -5436,13 +5445,13 @@
         <v>212</v>
       </c>
       <c r="B210" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="C210" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D210" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
     </row>
     <row r="211" spans="1:4">
@@ -5450,13 +5459,13 @@
         <v>213</v>
       </c>
       <c r="B211" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C211" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D211" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
     </row>
     <row r="212" spans="1:4">
@@ -5464,13 +5473,13 @@
         <v>214</v>
       </c>
       <c r="B212" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C212" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D212" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
     </row>
     <row r="213" spans="1:4">
@@ -5478,13 +5487,13 @@
         <v>215</v>
       </c>
       <c r="B213" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="C213" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D213" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
     </row>
     <row r="214" spans="1:4">
@@ -5492,13 +5501,13 @@
         <v>216</v>
       </c>
       <c r="B214" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C214" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="D214" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
     </row>
     <row r="215" spans="1:4">
@@ -5506,13 +5515,13 @@
         <v>217</v>
       </c>
       <c r="B215" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C215" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="D215" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
     </row>
     <row r="216" spans="1:4">
@@ -5520,13 +5529,13 @@
         <v>218</v>
       </c>
       <c r="B216" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C216" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D216" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
     </row>
     <row r="217" spans="1:4">
@@ -5534,13 +5543,13 @@
         <v>219</v>
       </c>
       <c r="B217" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C217" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="D217" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
     </row>
     <row r="218" spans="1:4">
@@ -5548,13 +5557,13 @@
         <v>220</v>
       </c>
       <c r="B218" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C218" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D218" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
     </row>
     <row r="219" spans="1:4">
@@ -5562,13 +5571,13 @@
         <v>221</v>
       </c>
       <c r="B219" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="C219" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D219" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
     </row>
     <row r="220" spans="1:4">
@@ -5576,13 +5585,13 @@
         <v>222</v>
       </c>
       <c r="B220" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="C220" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="D220" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
     </row>
     <row r="221" spans="1:4">
@@ -5590,13 +5599,13 @@
         <v>223</v>
       </c>
       <c r="B221" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C221" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D221" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
     </row>
     <row r="222" spans="1:4">
@@ -5604,13 +5613,13 @@
         <v>224</v>
       </c>
       <c r="B222" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C222" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="D222" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
     </row>
     <row r="223" spans="1:4">
@@ -5618,13 +5627,13 @@
         <v>225</v>
       </c>
       <c r="B223" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="C223" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D223" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
     </row>
     <row r="224" spans="1:4">
@@ -5632,13 +5641,13 @@
         <v>226</v>
       </c>
       <c r="B224" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="C224" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="D224" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
     </row>
     <row r="225" spans="1:4">
@@ -5646,13 +5655,13 @@
         <v>227</v>
       </c>
       <c r="B225" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C225" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="D225" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
     </row>
     <row r="226" spans="1:4">
@@ -5660,13 +5669,13 @@
         <v>228</v>
       </c>
       <c r="B226" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C226" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D226" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
     </row>
     <row r="227" spans="1:4">
@@ -5674,13 +5683,13 @@
         <v>229</v>
       </c>
       <c r="B227" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="C227" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D227" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
     </row>
     <row r="228" spans="1:4">
@@ -5688,13 +5697,13 @@
         <v>230</v>
       </c>
       <c r="B228" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C228" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="D228" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
     </row>
     <row r="229" spans="1:4">
@@ -5702,13 +5711,13 @@
         <v>231</v>
       </c>
       <c r="B229" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="C229" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D229" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
     </row>
     <row r="230" spans="1:4">
@@ -5716,13 +5725,13 @@
         <v>232</v>
       </c>
       <c r="B230" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="C230" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="D230" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="231" spans="1:4">
@@ -5730,13 +5739,13 @@
         <v>233</v>
       </c>
       <c r="B231" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C231" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="D231" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
     </row>
     <row r="232" spans="1:4">
@@ -5744,13 +5753,13 @@
         <v>234</v>
       </c>
       <c r="B232" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="C232" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D232" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
     </row>
     <row r="233" spans="1:4">
@@ -5758,13 +5767,13 @@
         <v>235</v>
       </c>
       <c r="B233" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C233" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="D233" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
     </row>
     <row r="234" spans="1:4">
@@ -5778,7 +5787,7 @@
         <v>236</v>
       </c>
       <c r="D234" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
     </row>
     <row r="235" spans="1:4">
@@ -5792,7 +5801,7 @@
         <v>237</v>
       </c>
       <c r="D235" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
     </row>
     <row r="236" spans="1:4">
@@ -5800,13 +5809,13 @@
         <v>238</v>
       </c>
       <c r="B236" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C236" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D236" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
     </row>
     <row r="237" spans="1:4">
@@ -5814,13 +5823,13 @@
         <v>239</v>
       </c>
       <c r="B237" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="C237" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="D237" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
     </row>
     <row r="238" spans="1:4">
@@ -5828,13 +5837,13 @@
         <v>240</v>
       </c>
       <c r="B238" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C238" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="D238" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
     </row>
     <row r="239" spans="1:4">
@@ -5842,13 +5851,13 @@
         <v>241</v>
       </c>
       <c r="B239" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C239" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="D239" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
     </row>
     <row r="240" spans="1:4">
@@ -5856,13 +5865,27 @@
         <v>242</v>
       </c>
       <c r="B240" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C240" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="D240" t="s">
-        <v>718</v>
+        <v>720</v>
+      </c>
+    </row>
+    <row r="241" spans="1:4">
+      <c r="A241" t="s">
+        <v>243</v>
+      </c>
+      <c r="B241" t="s">
+        <v>481</v>
+      </c>
+      <c r="C241" t="s">
+        <v>481</v>
+      </c>
+      <c r="D241" t="s">
+        <v>721</v>
       </c>
     </row>
   </sheetData>

</xml_diff>